<commit_message>
Maestro: bancos metalicos 90 cm (B.MET.090, 4 colores)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/datos/FICHERO_MAESTRO2.xlsx
+++ b/public/datos/FICHERO_MAESTRO2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Helian\Desktop\Fichero Maestro\Sistema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F5A7B2-A484-47F0-B284-1A62C1F5637C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C44ACFEE-C02B-4E29-9F88-65495DD3E9E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="591" xr2:uid="{90124268-D67C-4387-8829-7E3B806257E6}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2945" uniqueCount="1269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3169" uniqueCount="1327">
   <si>
     <t>Marketplace</t>
   </si>
@@ -3921,6 +3921,184 @@
   </si>
   <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790027535/taquillas_maestro/011/antracita/en/infografia_6.jpg</t>
+  </si>
+  <si>
+    <t>B.MET.090_G</t>
+  </si>
+  <si>
+    <t>MET</t>
+  </si>
+  <si>
+    <t>090</t>
+  </si>
+  <si>
+    <t>8437027641312</t>
+  </si>
+  <si>
+    <t>B.MET.090</t>
+  </si>
+  <si>
+    <t>Twinthink Banco Vestuario Metálico Para Gimnasio y Escuelas (Gris)</t>
+  </si>
+  <si>
+    <t>El banco vestuario metálico Twinthink es una solución práctica, resistente y versátil para equipar vestuarios, gimnasios, colegios, oficinas y zonas comunes con un asiento funcional y duradero. Diseñado para ofrecer comodidad y estabilidad en el uso diario, este banco metálico para vestuario combina una estructura robusta con un estilo limpio y profesional que se adapta fácilmente a distintos entornos. Fabricado en acero de alta resistencia, este banco vestuario está pensado para soportar un uso frecuente tanto en espacios interiores como en zonas cubiertas de exterior. Su diseño metálico facilita la limpieza y el mantenimiento, lo que lo convierte en una opción muy práctica para lugares donde la higiene y la durabilidad son esenciales. Gracias a su superficie lisa y a su estructura firme, ofrece una experiencia cómoda y estable al sentarse.&lt;br&gt;&lt;br&gt;Este modelo es ideal para colocar junto a una taquilla vestuario, facilitando el cambio de ropa, calzado o accesorios en gimnasios, centros deportivos, empresas, colegios o vestuarios colectivos. También puede utilizarse como banco exterior en patios cubiertos, entradas o áreas de espera, aportando una solución funcional con estética moderna.&lt;br&gt;&lt;br&gt;Además de su resistencia, el banco metálico de Twinthink destaca por su versatilidad. Puede utilizarse en espacios profesionales o domésticos, adaptándose a distintas necesidades sin perder su estilo sobrio y eficiente. Su formato permite optimizar el espacio disponible y mantener el orden en zonas de paso o de uso común.&lt;br&gt;&lt;br&gt;Si buscas uno de esos bancos metálicos que combinan resistencia, fácil mantenimiento y diseño práctico, el banco para vestuario Twinthink es una excelente opción para mejorar cualquier espacio con una solución duradera, cómoda y funcional.</t>
+  </si>
+  <si>
+    <t>Uso Profesional Para Vestuarios y Gimnasios – Banco diseñado para vestuarios, gimnasios, colegios, zonas de cambio y espacios colectivos donde se necesita una solución resistente, funcional y preparada para uso frecuente.
+Estructura Metálica Resistente – Fabricado con estructura de acero robusta para ofrecer estabilidad y durabilidad en el uso diario. Ideal para entornos profesionales con tránsito continuo y exigencia de resistencia.
+Acabado Duradero y Fácil de Limpiar – Su pintura/acabado protege la superficie y facilita el mantenimiento. El banco conserva una estética limpia y profesional, adecuada para instalaciones deportivas y educativas.
+Medidas Funcionales y Capacidad de Carga – Dimensiones: [90x32x45 cm]. Capacidad de carga recomendada: [150 kg]. Formato pensado para ofrecer una sentada cómoda y un uso estable en espacios compartidos.
+Bajo Mantenimiento y Uso Intensivo – La superficie lisa permite una limpieza rápida y sencilla, algo esencial en bancos para vestuario, gimnasios o colegios donde la higiene y la practicidad son prioritarias.</t>
+  </si>
+  <si>
+    <t>banco vestuario bancos para cocina banco cocina taquilla vestuario bancos banco exterior banquito</t>
+  </si>
+  <si>
+    <t>Twinthink Banco de Vestiário Metálico para Ginásio e Escolas (Cinzento)</t>
+  </si>
+  <si>
+    <t>O banco de vestiário metálico Twinthink é uma solução prática, resistente e versátil para equipar vestiários, ginásios, escolas, escritórios e zonas comuns com um assento funcional e duradouro. Concebido para oferecer conforto e estabilidade no uso diário, este banco metálico para vestiário combina uma estrutura robusta com um estilo limpo e profissional que se adapta facilmente a diferentes ambientes. Fabricado em aço de alta resistência, este banco de vestiário foi pensado para suportar uma utilização frequente tanto em espaços interiores como em zonas cobertas de exterior. O seu design metálico facilita a limpeza e a manutenção, o que o torna uma opção muito prática para locais onde a higiene e a durabilidade são essenciais. Graças à sua superfície lisa e à sua estrutura firme, oferece uma experiência cómoda e estável ao sentar.&lt;br&gt;&lt;br&gt;Este modelo é ideal para colocar junto a um cacifo de vestiário, facilitando a mudança de roupa, calçado ou acessórios em ginásios, centros desportivos, empresas, escolas ou vestiários coletivos. Também pode ser utilizado como banco de exterior em pátios cobertos, entradas ou áreas de espera, proporcionando uma solução funcional com estética moderna.&lt;br&gt;&lt;br&gt;Além da sua resistência, o banco metálico da Twinthink destaca-se pela sua versatilidade. Pode ser utilizado em espaços profissionais ou domésticos, adaptando-se a diferentes necessidades sem perder o seu estilo sóbrio e eficiente. O seu formato permite otimizar o espaço disponível e manter a ordem em zonas de passagem ou de uso comum.&lt;br&gt;&lt;br&gt;Se procura um banco metálico que combine resistência, fácil manutenção e design prático, o banco de vestiário Twinthink é uma excelente opção para melhorar qualquer espaço com uma solução duradoura, cómoda e funcional.</t>
+  </si>
+  <si>
+    <t>Twinthink Banc de Vestiaire Métallique pour Salle de Sport et Écoles (Gris)</t>
+  </si>
+  <si>
+    <t>Le banc de vestiaire métallique Twinthink est une solution pratique, résistante et polyvalente pour équiper vestiaires, salles de sport, écoles, bureaux et espaces communs d'une assise fonctionnelle et durable. Conçu pour offrir confort et stabilité au quotidien, ce banc métallique de vestiaire associe une structure robuste à un style épuré et professionnel qui s'adapte facilement à différents environnements. Fabriqué en acier haute résistance, ce banc de vestiaire est pensé pour supporter un usage fréquent aussi bien à l'intérieur que dans les zones extérieures couvertes. Sa conception métallique facilite le nettoyage et l'entretien, ce qui en fait une option très pratique pour les lieux où l'hygiène et la durabilité sont essentielles. Grâce à sa surface lisse et à sa structure ferme, il offre une assise confortable et stable.&lt;br&gt;&lt;br&gt;Ce modèle est idéal à placer à côté d'un casier de vestiaire, facilitant le changement de vêtements, de chaussures ou d'accessoires dans les salles de sport, centres sportifs, entreprises, écoles ou vestiaires collectifs. Il peut également être utilisé comme banc d'extérieur dans les cours couvertes, les entrées ou les zones d'attente, apportant une solution fonctionnelle à l'esthétique moderne.&lt;br&gt;&lt;br&gt;Outre sa résistance, le banc métallique Twinthink se distingue par sa polyvalence. Il peut être utilisé dans des espaces professionnels ou domestiques, s'adaptant à différents besoins sans perdre son style sobre et efficace. Son format permet d'optimiser l'espace disponible et de maintenir l'ordre dans les zones de passage ou d'usage commun.&lt;br&gt;&lt;br&gt;Si vous cherchez un banc métallique alliant résistance, entretien facile et design pratique, le banc de vestiaire Twinthink est un excellent choix pour améliorer n'importe quel espace avec une solution durable, confortable et fonctionnelle.</t>
+  </si>
+  <si>
+    <t>Twinthink Panca da Spogliatoio in Metallo per Palestra e Scuole (Grigio)</t>
+  </si>
+  <si>
+    <t>La panca da spogliatoio in metallo Twinthink è una soluzione pratica, resistente e versatile per attrezzare spogliatoi, palestre, scuole, uffici e aree comuni con una seduta funzionale e duratura. Progettata per offrire comfort e stabilità nell'uso quotidiano, questa panca metallica da spogliatoio unisce una struttura robusta a uno stile pulito e professionale che si adatta facilmente a diversi ambienti. Realizzata in acciaio ad alta resistenza, questa panca da spogliatoio è pensata per sopportare un uso frequente sia negli spazi interni sia nelle zone esterne coperte. Il suo design metallico facilita la pulizia e la manutenzione, rendendola un'opzione molto pratica per luoghi in cui igiene e durata sono essenziali. Grazie alla superficie liscia e alla struttura solida, offre un'esperienza comoda e stabile da seduti.&lt;br&gt;&lt;br&gt;Questo modello è ideale da collocare accanto a un armadietto da spogliatoio, facilitando il cambio di vestiti, scarpe o accessori in palestre, centri sportivi, aziende, scuole o spogliatoi collettivi. Può essere utilizzata anche come panca da esterno in cortili coperti, ingressi o aree di attesa, offrendo una soluzione funzionale dall'estetica moderna.&lt;br&gt;&lt;br&gt;Oltre alla sua resistenza, la panca metallica Twinthink si distingue per la sua versatilità. Può essere utilizzata in spazi professionali o domestici, adattandosi a diverse esigenze senza perdere il suo stile sobrio ed efficiente. Il suo formato permette di ottimizzare lo spazio disponibile e mantenere l'ordine nelle zone di passaggio o di uso comune.&lt;br&gt;&lt;br&gt;Se cerchi una panca metallica che unisca resistenza, facile manutenzione e design pratico, la panca da spogliatoio Twinthink è un'ottima scelta per migliorare qualsiasi spazio con una soluzione duratura, comoda e funzionale.</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213596/bancos/B.MET.090/gris/img_00.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213599/bancos/B.MET.090/gris/img_01.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213601/bancos/B.MET.090/gris/img_02.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213603/bancos/B.MET.090/gris/img_03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213606/bancos/B.MET.090/gris/img_04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213608/bancos/B.MET.090/gris/img_05.jpg</t>
+  </si>
+  <si>
+    <t>B.MET.090_N</t>
+  </si>
+  <si>
+    <t>8437027641336</t>
+  </si>
+  <si>
+    <t>Twinthink Banco Vestuario Metálico Para Gimnasio y Escuelas (Negro)</t>
+  </si>
+  <si>
+    <t>Twinthink Banco de Vestiário Metálico para Ginásio e Escolas (Preto)</t>
+  </si>
+  <si>
+    <t>Twinthink Banc de Vestiaire Métallique pour Salle de Sport et Écoles (Noir)</t>
+  </si>
+  <si>
+    <t>Twinthink Panca da Spogliatoio in Metallo per Palestra e Scuole (Nero)</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213582/bancos/B.MET.090/negro/img_00.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213584/bancos/B.MET.090/negro/img_01.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213587/bancos/B.MET.090/negro/img_02.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213589/bancos/B.MET.090/negro/img_03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213592/bancos/B.MET.090/negro/img_04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213594/bancos/B.MET.090/negro/img_05.jpg</t>
+  </si>
+  <si>
+    <t>B.MET.090_B</t>
+  </si>
+  <si>
+    <t>8437027641329</t>
+  </si>
+  <si>
+    <t>Twinthink Banco Vestuario Metálico Para Gimnasio y Escuelas (Blanco)</t>
+  </si>
+  <si>
+    <t>Twinthink Banco de Vestiário Metálico para Ginásio e Escolas (Branco)</t>
+  </si>
+  <si>
+    <t>Twinthink Banc de Vestiaire Métallique pour Salle de Sport et Écoles (Blanc)</t>
+  </si>
+  <si>
+    <t>Twinthink Panca da Spogliatoio in Metallo per Palestra e Scuole (Bianco)</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213552/bancos/B.MET.090/blanco/img_00.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213554/bancos/B.MET.090/blanco/img_01.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213557/bancos/B.MET.090/blanco/img_02.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213559/bancos/B.MET.090/blanco/img_03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213562/bancos/B.MET.090/blanco/img_04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213565/bancos/B.MET.090/blanco/img_05.jpg</t>
+  </si>
+  <si>
+    <t>B.MET.090_B-N</t>
+  </si>
+  <si>
+    <t>8437027641343</t>
+  </si>
+  <si>
+    <t>B.MET.090_B&amp;N</t>
+  </si>
+  <si>
+    <t>Twinthink Banco Vestuario Metálico Para Gimnasio y Escuelas (Blanco/Negro)</t>
+  </si>
+  <si>
+    <t>Twinthink Banco de Vestiário Metálico para Ginásio e Escolas (Branco/Preto)</t>
+  </si>
+  <si>
+    <t>Twinthink Banc de Vestiaire Métallique pour Salle de Sport et Écoles (Blanc/Noir)</t>
+  </si>
+  <si>
+    <t>Twinthink Panca da Spogliatoio in Metallo per Palestra e Scuole (Bianco/Nero)</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213567/bancos/B.MET.090/byn/img_00.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213569/bancos/B.MET.090/byn/img_01.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213572/bancos/B.MET.090/byn/img_02.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213575/bancos/B.MET.090/byn/img_03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213577/bancos/B.MET.090/byn/img_04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213580/bancos/B.MET.090/byn/img_05.jpg</t>
   </si>
 </sst>
 </file>
@@ -9812,7 +9990,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C52A7A11-77C7-4197-B539-DBD653EC8E79}">
-  <dimension ref="A1:CQ32"/>
+  <dimension ref="A1:CQ36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -16449,6 +16627,734 @@
         <v>1268</v>
       </c>
     </row>
+    <row r="33" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>1269</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1270</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>1271</v>
+      </c>
+      <c r="D33" t="s">
+        <v>123</v>
+      </c>
+      <c r="E33" t="s">
+        <v>124</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>1272</v>
+      </c>
+      <c r="G33" t="s">
+        <v>126</v>
+      </c>
+      <c r="H33" t="s">
+        <v>1273</v>
+      </c>
+      <c r="I33" t="s">
+        <v>1273</v>
+      </c>
+      <c r="J33" t="s">
+        <v>1273</v>
+      </c>
+      <c r="K33" t="s">
+        <v>1273</v>
+      </c>
+      <c r="L33" t="s">
+        <v>1274</v>
+      </c>
+      <c r="M33" t="s">
+        <v>1275</v>
+      </c>
+      <c r="N33" s="14" t="s">
+        <v>1276</v>
+      </c>
+      <c r="O33" t="s">
+        <v>1277</v>
+      </c>
+      <c r="P33" t="s">
+        <v>1278</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>1279</v>
+      </c>
+      <c r="T33" t="s">
+        <v>1280</v>
+      </c>
+      <c r="U33" t="s">
+        <v>1281</v>
+      </c>
+      <c r="X33" t="s">
+        <v>1282</v>
+      </c>
+      <c r="Y33" t="s">
+        <v>1283</v>
+      </c>
+      <c r="AJ33">
+        <v>45</v>
+      </c>
+      <c r="AK33">
+        <v>90</v>
+      </c>
+      <c r="AL33">
+        <v>32</v>
+      </c>
+      <c r="AM33">
+        <v>12</v>
+      </c>
+      <c r="AN33" t="s">
+        <v>143</v>
+      </c>
+      <c r="AO33" t="s">
+        <v>144</v>
+      </c>
+      <c r="AP33" t="s">
+        <v>145</v>
+      </c>
+      <c r="AQ33" t="s">
+        <v>146</v>
+      </c>
+      <c r="AU33" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB33" t="s">
+        <v>1284</v>
+      </c>
+      <c r="BC33" t="s">
+        <v>1285</v>
+      </c>
+      <c r="BD33" t="s">
+        <v>1286</v>
+      </c>
+      <c r="BE33" t="s">
+        <v>1287</v>
+      </c>
+      <c r="BF33" t="s">
+        <v>1288</v>
+      </c>
+      <c r="BG33" t="s">
+        <v>1289</v>
+      </c>
+      <c r="BH33" t="s">
+        <v>1284</v>
+      </c>
+      <c r="BI33" t="s">
+        <v>1285</v>
+      </c>
+      <c r="BJ33" t="s">
+        <v>1286</v>
+      </c>
+      <c r="BK33" t="s">
+        <v>1287</v>
+      </c>
+      <c r="BL33" t="s">
+        <v>1288</v>
+      </c>
+      <c r="BM33" t="s">
+        <v>1289</v>
+      </c>
+      <c r="BN33" t="s">
+        <v>1284</v>
+      </c>
+      <c r="BO33" t="s">
+        <v>1285</v>
+      </c>
+      <c r="BP33" t="s">
+        <v>1286</v>
+      </c>
+      <c r="BQ33" t="s">
+        <v>1287</v>
+      </c>
+      <c r="BR33" t="s">
+        <v>1288</v>
+      </c>
+      <c r="BS33" t="s">
+        <v>1289</v>
+      </c>
+      <c r="BT33" t="s">
+        <v>1284</v>
+      </c>
+      <c r="BU33" t="s">
+        <v>1285</v>
+      </c>
+      <c r="BV33" t="s">
+        <v>1286</v>
+      </c>
+      <c r="BW33" t="s">
+        <v>1287</v>
+      </c>
+      <c r="BX33" t="s">
+        <v>1288</v>
+      </c>
+      <c r="BY33" t="s">
+        <v>1289</v>
+      </c>
+      <c r="BZ33" t="s">
+        <v>1284</v>
+      </c>
+      <c r="CA33" t="s">
+        <v>1285</v>
+      </c>
+      <c r="CB33" t="s">
+        <v>1286</v>
+      </c>
+      <c r="CC33" t="s">
+        <v>1287</v>
+      </c>
+      <c r="CD33" t="s">
+        <v>1288</v>
+      </c>
+      <c r="CE33" t="s">
+        <v>1289</v>
+      </c>
+    </row>
+    <row r="34" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>1290</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1270</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>1271</v>
+      </c>
+      <c r="D34" t="s">
+        <v>181</v>
+      </c>
+      <c r="E34" t="s">
+        <v>182</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>1291</v>
+      </c>
+      <c r="G34" t="s">
+        <v>126</v>
+      </c>
+      <c r="H34" t="s">
+        <v>1290</v>
+      </c>
+      <c r="I34" t="s">
+        <v>1290</v>
+      </c>
+      <c r="J34" t="s">
+        <v>1290</v>
+      </c>
+      <c r="K34" t="s">
+        <v>1290</v>
+      </c>
+      <c r="L34" t="s">
+        <v>1292</v>
+      </c>
+      <c r="M34" t="s">
+        <v>1275</v>
+      </c>
+      <c r="N34" s="14" t="s">
+        <v>1276</v>
+      </c>
+      <c r="O34" t="s">
+        <v>1277</v>
+      </c>
+      <c r="P34" t="s">
+        <v>1293</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>1279</v>
+      </c>
+      <c r="T34" t="s">
+        <v>1294</v>
+      </c>
+      <c r="U34" t="s">
+        <v>1281</v>
+      </c>
+      <c r="X34" t="s">
+        <v>1295</v>
+      </c>
+      <c r="Y34" t="s">
+        <v>1283</v>
+      </c>
+      <c r="AJ34">
+        <v>45</v>
+      </c>
+      <c r="AK34">
+        <v>90</v>
+      </c>
+      <c r="AL34">
+        <v>32</v>
+      </c>
+      <c r="AM34">
+        <v>12</v>
+      </c>
+      <c r="AN34" t="s">
+        <v>143</v>
+      </c>
+      <c r="AO34" t="s">
+        <v>144</v>
+      </c>
+      <c r="AP34" t="s">
+        <v>145</v>
+      </c>
+      <c r="AQ34" t="s">
+        <v>146</v>
+      </c>
+      <c r="AU34" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB34" t="s">
+        <v>1296</v>
+      </c>
+      <c r="BC34" t="s">
+        <v>1297</v>
+      </c>
+      <c r="BD34" t="s">
+        <v>1298</v>
+      </c>
+      <c r="BE34" t="s">
+        <v>1299</v>
+      </c>
+      <c r="BF34" t="s">
+        <v>1300</v>
+      </c>
+      <c r="BG34" t="s">
+        <v>1301</v>
+      </c>
+      <c r="BH34" t="s">
+        <v>1296</v>
+      </c>
+      <c r="BI34" t="s">
+        <v>1297</v>
+      </c>
+      <c r="BJ34" t="s">
+        <v>1298</v>
+      </c>
+      <c r="BK34" t="s">
+        <v>1299</v>
+      </c>
+      <c r="BL34" t="s">
+        <v>1300</v>
+      </c>
+      <c r="BM34" t="s">
+        <v>1301</v>
+      </c>
+      <c r="BN34" t="s">
+        <v>1296</v>
+      </c>
+      <c r="BO34" t="s">
+        <v>1297</v>
+      </c>
+      <c r="BP34" t="s">
+        <v>1298</v>
+      </c>
+      <c r="BQ34" t="s">
+        <v>1299</v>
+      </c>
+      <c r="BR34" t="s">
+        <v>1300</v>
+      </c>
+      <c r="BS34" t="s">
+        <v>1301</v>
+      </c>
+      <c r="BT34" t="s">
+        <v>1296</v>
+      </c>
+      <c r="BU34" t="s">
+        <v>1297</v>
+      </c>
+      <c r="BV34" t="s">
+        <v>1298</v>
+      </c>
+      <c r="BW34" t="s">
+        <v>1299</v>
+      </c>
+      <c r="BX34" t="s">
+        <v>1300</v>
+      </c>
+      <c r="BY34" t="s">
+        <v>1301</v>
+      </c>
+      <c r="BZ34" t="s">
+        <v>1296</v>
+      </c>
+      <c r="CA34" t="s">
+        <v>1297</v>
+      </c>
+      <c r="CB34" t="s">
+        <v>1298</v>
+      </c>
+      <c r="CC34" t="s">
+        <v>1299</v>
+      </c>
+      <c r="CD34" t="s">
+        <v>1300</v>
+      </c>
+      <c r="CE34" t="s">
+        <v>1301</v>
+      </c>
+    </row>
+    <row r="35" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B35" t="s">
+        <v>1270</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>1271</v>
+      </c>
+      <c r="D35" t="s">
+        <v>220</v>
+      </c>
+      <c r="E35" t="s">
+        <v>221</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>1303</v>
+      </c>
+      <c r="G35" t="s">
+        <v>126</v>
+      </c>
+      <c r="H35" t="s">
+        <v>1302</v>
+      </c>
+      <c r="I35" t="s">
+        <v>1302</v>
+      </c>
+      <c r="J35" t="s">
+        <v>1302</v>
+      </c>
+      <c r="K35" t="s">
+        <v>1302</v>
+      </c>
+      <c r="L35" t="s">
+        <v>1304</v>
+      </c>
+      <c r="M35" t="s">
+        <v>1275</v>
+      </c>
+      <c r="N35" s="14" t="s">
+        <v>1276</v>
+      </c>
+      <c r="O35" t="s">
+        <v>1277</v>
+      </c>
+      <c r="P35" t="s">
+        <v>1305</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>1279</v>
+      </c>
+      <c r="T35" t="s">
+        <v>1306</v>
+      </c>
+      <c r="U35" t="s">
+        <v>1281</v>
+      </c>
+      <c r="X35" t="s">
+        <v>1307</v>
+      </c>
+      <c r="Y35" t="s">
+        <v>1283</v>
+      </c>
+      <c r="AJ35">
+        <v>45</v>
+      </c>
+      <c r="AK35">
+        <v>90</v>
+      </c>
+      <c r="AL35">
+        <v>32</v>
+      </c>
+      <c r="AM35">
+        <v>12</v>
+      </c>
+      <c r="AN35" t="s">
+        <v>143</v>
+      </c>
+      <c r="AO35" t="s">
+        <v>144</v>
+      </c>
+      <c r="AP35" t="s">
+        <v>145</v>
+      </c>
+      <c r="AQ35" t="s">
+        <v>146</v>
+      </c>
+      <c r="AU35" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB35" t="s">
+        <v>1308</v>
+      </c>
+      <c r="BC35" t="s">
+        <v>1309</v>
+      </c>
+      <c r="BD35" t="s">
+        <v>1310</v>
+      </c>
+      <c r="BE35" t="s">
+        <v>1311</v>
+      </c>
+      <c r="BF35" t="s">
+        <v>1312</v>
+      </c>
+      <c r="BG35" t="s">
+        <v>1313</v>
+      </c>
+      <c r="BH35" t="s">
+        <v>1308</v>
+      </c>
+      <c r="BI35" t="s">
+        <v>1309</v>
+      </c>
+      <c r="BJ35" t="s">
+        <v>1310</v>
+      </c>
+      <c r="BK35" t="s">
+        <v>1311</v>
+      </c>
+      <c r="BL35" t="s">
+        <v>1312</v>
+      </c>
+      <c r="BM35" t="s">
+        <v>1313</v>
+      </c>
+      <c r="BN35" t="s">
+        <v>1308</v>
+      </c>
+      <c r="BO35" t="s">
+        <v>1309</v>
+      </c>
+      <c r="BP35" t="s">
+        <v>1310</v>
+      </c>
+      <c r="BQ35" t="s">
+        <v>1311</v>
+      </c>
+      <c r="BR35" t="s">
+        <v>1312</v>
+      </c>
+      <c r="BS35" t="s">
+        <v>1313</v>
+      </c>
+      <c r="BT35" t="s">
+        <v>1308</v>
+      </c>
+      <c r="BU35" t="s">
+        <v>1309</v>
+      </c>
+      <c r="BV35" t="s">
+        <v>1310</v>
+      </c>
+      <c r="BW35" t="s">
+        <v>1311</v>
+      </c>
+      <c r="BX35" t="s">
+        <v>1312</v>
+      </c>
+      <c r="BY35" t="s">
+        <v>1313</v>
+      </c>
+      <c r="BZ35" t="s">
+        <v>1308</v>
+      </c>
+      <c r="CA35" t="s">
+        <v>1309</v>
+      </c>
+      <c r="CB35" t="s">
+        <v>1310</v>
+      </c>
+      <c r="CC35" t="s">
+        <v>1311</v>
+      </c>
+      <c r="CD35" t="s">
+        <v>1312</v>
+      </c>
+      <c r="CE35" t="s">
+        <v>1313</v>
+      </c>
+    </row>
+    <row r="36" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>1314</v>
+      </c>
+      <c r="B36" t="s">
+        <v>1270</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>1271</v>
+      </c>
+      <c r="D36" t="s">
+        <v>258</v>
+      </c>
+      <c r="E36" t="s">
+        <v>259</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>1315</v>
+      </c>
+      <c r="G36" t="s">
+        <v>126</v>
+      </c>
+      <c r="H36" t="s">
+        <v>1316</v>
+      </c>
+      <c r="I36" t="s">
+        <v>1316</v>
+      </c>
+      <c r="J36" t="s">
+        <v>1316</v>
+      </c>
+      <c r="K36" t="s">
+        <v>1316</v>
+      </c>
+      <c r="L36" t="s">
+        <v>1317</v>
+      </c>
+      <c r="M36" t="s">
+        <v>1275</v>
+      </c>
+      <c r="N36" s="14" t="s">
+        <v>1276</v>
+      </c>
+      <c r="O36" t="s">
+        <v>1277</v>
+      </c>
+      <c r="P36" t="s">
+        <v>1318</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>1279</v>
+      </c>
+      <c r="T36" t="s">
+        <v>1319</v>
+      </c>
+      <c r="U36" t="s">
+        <v>1281</v>
+      </c>
+      <c r="X36" t="s">
+        <v>1320</v>
+      </c>
+      <c r="Y36" t="s">
+        <v>1283</v>
+      </c>
+      <c r="AJ36">
+        <v>45</v>
+      </c>
+      <c r="AK36">
+        <v>90</v>
+      </c>
+      <c r="AL36">
+        <v>32</v>
+      </c>
+      <c r="AM36">
+        <v>12</v>
+      </c>
+      <c r="AN36" t="s">
+        <v>143</v>
+      </c>
+      <c r="AO36" t="s">
+        <v>144</v>
+      </c>
+      <c r="AP36" t="s">
+        <v>145</v>
+      </c>
+      <c r="AQ36" t="s">
+        <v>146</v>
+      </c>
+      <c r="AU36" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB36" t="s">
+        <v>1321</v>
+      </c>
+      <c r="BC36" t="s">
+        <v>1322</v>
+      </c>
+      <c r="BD36" t="s">
+        <v>1323</v>
+      </c>
+      <c r="BE36" t="s">
+        <v>1324</v>
+      </c>
+      <c r="BF36" t="s">
+        <v>1325</v>
+      </c>
+      <c r="BG36" t="s">
+        <v>1326</v>
+      </c>
+      <c r="BH36" t="s">
+        <v>1321</v>
+      </c>
+      <c r="BI36" t="s">
+        <v>1322</v>
+      </c>
+      <c r="BJ36" t="s">
+        <v>1323</v>
+      </c>
+      <c r="BK36" t="s">
+        <v>1324</v>
+      </c>
+      <c r="BL36" t="s">
+        <v>1325</v>
+      </c>
+      <c r="BM36" t="s">
+        <v>1326</v>
+      </c>
+      <c r="BN36" t="s">
+        <v>1321</v>
+      </c>
+      <c r="BO36" t="s">
+        <v>1322</v>
+      </c>
+      <c r="BP36" t="s">
+        <v>1323</v>
+      </c>
+      <c r="BQ36" t="s">
+        <v>1324</v>
+      </c>
+      <c r="BR36" t="s">
+        <v>1325</v>
+      </c>
+      <c r="BS36" t="s">
+        <v>1326</v>
+      </c>
+      <c r="BT36" t="s">
+        <v>1321</v>
+      </c>
+      <c r="BU36" t="s">
+        <v>1322</v>
+      </c>
+      <c r="BV36" t="s">
+        <v>1323</v>
+      </c>
+      <c r="BW36" t="s">
+        <v>1324</v>
+      </c>
+      <c r="BX36" t="s">
+        <v>1325</v>
+      </c>
+      <c r="BY36" t="s">
+        <v>1326</v>
+      </c>
+      <c r="BZ36" t="s">
+        <v>1321</v>
+      </c>
+      <c r="CA36" t="s">
+        <v>1322</v>
+      </c>
+      <c r="CB36" t="s">
+        <v>1323</v>
+      </c>
+      <c r="CC36" t="s">
+        <v>1324</v>
+      </c>
+      <c r="CD36" t="s">
+        <v>1325</v>
+      </c>
+      <c r="CE36" t="s">
+        <v>1326</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="CF1:CK1"/>

</xml_diff>

<commit_message>
Maestro: textos en aleman e ingles de los bancos B.MET.090
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/datos/FICHERO_MAESTRO2.xlsx
+++ b/public/datos/FICHERO_MAESTRO2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Helian\Desktop\Fichero Maestro\Sistema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C44ACFEE-C02B-4E29-9F88-65495DD3E9E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EE498BD-27C3-4EA2-8B7D-E5B6E239D898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="591" xr2:uid="{90124268-D67C-4387-8829-7E3B806257E6}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3169" uniqueCount="1327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3201" uniqueCount="1341">
   <si>
     <t>Marketplace</t>
   </si>
@@ -4099,6 +4099,56 @@
   </si>
   <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213580/bancos/B.MET.090/byn/img_05.jpg</t>
+  </si>
+  <si>
+    <t>Twinthink Metall-Umkleidebank für Fitnessstudios und Schulen (Grau)</t>
+  </si>
+  <si>
+    <t>Die Metall-Umkleidebank von Twinthink ist eine praktische, robuste und vielseitige Lösung, um Umkleideräume, Fitnessstudios, Schulen, Büros und Gemeinschaftsbereiche mit einer funktionalen und langlebigen Sitzgelegenheit auszustatten. Sie wurde für Komfort und Stabilität im täglichen Gebrauch entwickelt und verbindet eine robuste Konstruktion mit einem klaren, professionellen Stil, der sich mühelos in unterschiedliche Umgebungen einfügt. Die aus hochfestem Stahl gefertigte Umkleidebank ist für die häufige Nutzung sowohl in Innenräumen als auch in überdachten Außenbereichen ausgelegt. Dank der Metallausführung lässt sie sich leicht reinigen und pflegen – ideal für Orte, an denen Hygiene und Langlebigkeit entscheidend sind. Die glatte Oberfläche und die stabile Konstruktion sorgen für ein bequemes und sicheres Sitzen.&lt;br&gt;&lt;br&gt;Dieses Modell eignet sich ideal als Ergänzung zu einem Umkleidespind und erleichtert das Wechseln von Kleidung, Schuhen oder Accessoires in Fitnessstudios, Sportzentren, Unternehmen, Schulen oder Gemeinschaftsumkleiden. Sie kann auch als Außenbank in überdachten Innenhöfen, Eingangsbereichen oder Wartezonen eingesetzt werden und bietet eine funktionale Lösung mit modernem Design.&lt;br&gt;&lt;br&gt;Neben ihrer Robustheit überzeugt die Metallbank von Twinthink durch ihre Vielseitigkeit. Sie lässt sich im gewerblichen wie im privaten Bereich einsetzen und passt sich unterschiedlichen Anforderungen an, ohne ihren schlichten und effizienten Stil zu verlieren. Ihr Format hilft, den verfügbaren Platz optimal zu nutzen und Durchgangs- oder Gemeinschaftsbereiche ordentlich zu halten.&lt;br&gt;&lt;br&gt;Wenn Sie eine Metallbank suchen, die Robustheit, einfache Pflege und praktisches Design vereint, ist die Umkleidebank von Twinthink eine ausgezeichnete Wahl, um jeden Raum mit einer langlebigen, bequemen und funktionalen Lösung aufzuwerten.</t>
+  </si>
+  <si>
+    <t>Professioneller Einsatz in Umkleiden und Fitnessstudios – Bank für Umkleideräume, Fitnessstudios, Schulen, Umkleidebereiche und Gemeinschaftsräume, in denen eine robuste, funktionale und für die häufige Nutzung ausgelegte Lösung gefragt ist.
+Robuste Metallkonstruktion – Das stabile Stahlgestell sorgt für Standfestigkeit und Langlebigkeit im täglichen Gebrauch. Ideal für gewerbliche Umgebungen mit viel Betrieb und hohen Anforderungen an die Belastbarkeit.
+Langlebige, leicht zu reinigende Oberfläche – Die Lackierung schützt die Oberfläche und erleichtert die Pflege. Die Bank behält ihr sauberes, professionelles Erscheinungsbild und eignet sich ideal für Sport- und Bildungseinrichtungen.
+Praktische Maße und Belastbarkeit – Abmessungen: 90 x 32 x 45 cm. Empfohlene Belastbarkeit: 150 kg. Das Format sorgt für bequemes Sitzen und eine stabile Nutzung in gemeinsam genutzten Räumen.
+Pflegeleicht und für intensive Nutzung – Die glatte Oberfläche lässt sich schnell und einfach reinigen – unverzichtbar für Umkleidebänke in Fitnessstudios oder Schulen, wo Hygiene und Praktikabilität an erster Stelle stehen.</t>
+  </si>
+  <si>
+    <t>umkleidebank sitzbank metall metallbank umkleide bank garderobenbank turnhallenbank spind bank flurbank außenbank sitzbank stahl</t>
+  </si>
+  <si>
+    <t>Twinthink Metal Changing Room Bench for Gyms and Schools (Grey)</t>
+  </si>
+  <si>
+    <t>The Twinthink metal changing room bench is a practical, sturdy and versatile solution for fitting out changing rooms, gyms, schools, offices and communal areas with functional, long-lasting seating. Designed for comfort and stability in everyday use, this metal locker room bench combines a robust structure with a clean, professional style that fits easily into different settings. Made from high-strength steel, this changing room bench is built to withstand frequent use both indoors and in covered outdoor areas. Its metal design makes cleaning and maintenance easy, making it a very practical choice for places where hygiene and durability are essential. Thanks to its smooth surface and solid frame, it offers comfortable and stable seating.&lt;br&gt;&lt;br&gt;This model is ideal for placing next to a changing room locker, making it easier to change clothes, shoes or accessories in gyms, sports centres, workplaces, schools or shared changing rooms. It can also be used as an outdoor bench in covered courtyards, entrances or waiting areas, providing a functional solution with a modern look.&lt;br&gt;&lt;br&gt;As well as being strong, the Twinthink metal bench stands out for its versatility. It can be used in professional or home settings, adapting to different needs without losing its understated, efficient style. Its format helps you make the most of the available space and keep walkways and shared areas tidy.&lt;br&gt;&lt;br&gt;If you are looking for a metal bench that combines strength, easy maintenance and practical design, the Twinthink changing room bench is an excellent choice for upgrading any space with a durable, comfortable and functional solution.</t>
+  </si>
+  <si>
+    <t>Professional Use for Changing Rooms and Gyms – Bench designed for changing rooms, gyms, schools, locker areas and communal spaces that need a sturdy, functional solution ready for frequent use.
+Sturdy Metal Structure – Made with a robust steel frame for stability and durability in everyday use. Ideal for professional environments with constant footfall and high strength requirements.
+Durable, Easy-to-Clean Finish – The painted finish protects the surface and makes maintenance easy. The bench keeps a clean, professional look, suitable for sports and educational facilities.
+Practical Dimensions and Load Capacity – Dimensions: 90 x 32 x 45 cm. Recommended load capacity: 150 kg. Designed to provide comfortable seating and stable use in shared spaces.
+Low Maintenance, Built for Heavy Use – The smooth surface allows quick and easy cleaning, essential for changing room benches in gyms or schools where hygiene and practicality are a priority.</t>
+  </si>
+  <si>
+    <t>changing room bench; metal bench; locker room bench; gym bench; cloakroom bench; school bench; steel bench; outdoor bench; hallway bench; bench seat</t>
+  </si>
+  <si>
+    <t>Twinthink Metall-Umkleidebank für Fitnessstudios und Schulen (Schwarz)</t>
+  </si>
+  <si>
+    <t>Twinthink Metal Changing Room Bench for Gyms and Schools (Black)</t>
+  </si>
+  <si>
+    <t>Twinthink Metall-Umkleidebank für Fitnessstudios und Schulen (Weiß)</t>
+  </si>
+  <si>
+    <t>Twinthink Metal Changing Room Bench for Gyms and Schools (White)</t>
+  </si>
+  <si>
+    <t>Twinthink Metall-Umkleidebank für Fitnessstudios und Schulen (Weiß/Schwarz)</t>
+  </si>
+  <si>
+    <t>Twinthink Metal Changing Room Bench for Gyms and Schools (White/Black)</t>
   </si>
 </sst>
 </file>
@@ -16691,6 +16741,30 @@
       <c r="Y33" t="s">
         <v>1283</v>
       </c>
+      <c r="AB33" t="s">
+        <v>1327</v>
+      </c>
+      <c r="AC33" t="s">
+        <v>1328</v>
+      </c>
+      <c r="AD33" s="14" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AE33" t="s">
+        <v>1330</v>
+      </c>
+      <c r="AF33" t="s">
+        <v>1331</v>
+      </c>
+      <c r="AG33" t="s">
+        <v>1332</v>
+      </c>
+      <c r="AH33" s="14" t="s">
+        <v>1333</v>
+      </c>
+      <c r="AI33" t="s">
+        <v>1334</v>
+      </c>
       <c r="AJ33">
         <v>45</v>
       </c>
@@ -16873,6 +16947,30 @@
       <c r="Y34" t="s">
         <v>1283</v>
       </c>
+      <c r="AB34" t="s">
+        <v>1335</v>
+      </c>
+      <c r="AC34" t="s">
+        <v>1328</v>
+      </c>
+      <c r="AD34" s="14" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AE34" t="s">
+        <v>1330</v>
+      </c>
+      <c r="AF34" t="s">
+        <v>1336</v>
+      </c>
+      <c r="AG34" t="s">
+        <v>1332</v>
+      </c>
+      <c r="AH34" s="14" t="s">
+        <v>1333</v>
+      </c>
+      <c r="AI34" t="s">
+        <v>1334</v>
+      </c>
       <c r="AJ34">
         <v>45</v>
       </c>
@@ -17055,6 +17153,30 @@
       <c r="Y35" t="s">
         <v>1283</v>
       </c>
+      <c r="AB35" t="s">
+        <v>1337</v>
+      </c>
+      <c r="AC35" t="s">
+        <v>1328</v>
+      </c>
+      <c r="AD35" s="14" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AE35" t="s">
+        <v>1330</v>
+      </c>
+      <c r="AF35" t="s">
+        <v>1338</v>
+      </c>
+      <c r="AG35" t="s">
+        <v>1332</v>
+      </c>
+      <c r="AH35" s="14" t="s">
+        <v>1333</v>
+      </c>
+      <c r="AI35" t="s">
+        <v>1334</v>
+      </c>
       <c r="AJ35">
         <v>45</v>
       </c>
@@ -17236,6 +17358,30 @@
       </c>
       <c r="Y36" t="s">
         <v>1283</v>
+      </c>
+      <c r="AB36" t="s">
+        <v>1339</v>
+      </c>
+      <c r="AC36" t="s">
+        <v>1328</v>
+      </c>
+      <c r="AD36" s="14" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AE36" t="s">
+        <v>1330</v>
+      </c>
+      <c r="AF36" t="s">
+        <v>1340</v>
+      </c>
+      <c r="AG36" t="s">
+        <v>1332</v>
+      </c>
+      <c r="AH36" s="14" t="s">
+        <v>1333</v>
+      </c>
+      <c r="AI36" t="s">
+        <v>1334</v>
       </c>
       <c r="AJ36">
         <v>45</v>

</xml_diff>

<commit_message>
Maestro: quitar corchetes de las viñetas ES de los bancos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/datos/FICHERO_MAESTRO2.xlsx
+++ b/public/datos/FICHERO_MAESTRO2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Helian\Desktop\Fichero Maestro\Sistema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EE498BD-27C3-4EA2-8B7D-E5B6E239D898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC75FE3-3CFC-41ED-BCFE-537A60222BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="591" xr2:uid="{90124268-D67C-4387-8829-7E3B806257E6}"/>
   </bookViews>
@@ -3944,13 +3944,6 @@
     <t>El banco vestuario metálico Twinthink es una solución práctica, resistente y versátil para equipar vestuarios, gimnasios, colegios, oficinas y zonas comunes con un asiento funcional y duradero. Diseñado para ofrecer comodidad y estabilidad en el uso diario, este banco metálico para vestuario combina una estructura robusta con un estilo limpio y profesional que se adapta fácilmente a distintos entornos. Fabricado en acero de alta resistencia, este banco vestuario está pensado para soportar un uso frecuente tanto en espacios interiores como en zonas cubiertas de exterior. Su diseño metálico facilita la limpieza y el mantenimiento, lo que lo convierte en una opción muy práctica para lugares donde la higiene y la durabilidad son esenciales. Gracias a su superficie lisa y a su estructura firme, ofrece una experiencia cómoda y estable al sentarse.&lt;br&gt;&lt;br&gt;Este modelo es ideal para colocar junto a una taquilla vestuario, facilitando el cambio de ropa, calzado o accesorios en gimnasios, centros deportivos, empresas, colegios o vestuarios colectivos. También puede utilizarse como banco exterior en patios cubiertos, entradas o áreas de espera, aportando una solución funcional con estética moderna.&lt;br&gt;&lt;br&gt;Además de su resistencia, el banco metálico de Twinthink destaca por su versatilidad. Puede utilizarse en espacios profesionales o domésticos, adaptándose a distintas necesidades sin perder su estilo sobrio y eficiente. Su formato permite optimizar el espacio disponible y mantener el orden en zonas de paso o de uso común.&lt;br&gt;&lt;br&gt;Si buscas uno de esos bancos metálicos que combinan resistencia, fácil mantenimiento y diseño práctico, el banco para vestuario Twinthink es una excelente opción para mejorar cualquier espacio con una solución duradera, cómoda y funcional.</t>
   </si>
   <si>
-    <t>Uso Profesional Para Vestuarios y Gimnasios – Banco diseñado para vestuarios, gimnasios, colegios, zonas de cambio y espacios colectivos donde se necesita una solución resistente, funcional y preparada para uso frecuente.
-Estructura Metálica Resistente – Fabricado con estructura de acero robusta para ofrecer estabilidad y durabilidad en el uso diario. Ideal para entornos profesionales con tránsito continuo y exigencia de resistencia.
-Acabado Duradero y Fácil de Limpiar – Su pintura/acabado protege la superficie y facilita el mantenimiento. El banco conserva una estética limpia y profesional, adecuada para instalaciones deportivas y educativas.
-Medidas Funcionales y Capacidad de Carga – Dimensiones: [90x32x45 cm]. Capacidad de carga recomendada: [150 kg]. Formato pensado para ofrecer una sentada cómoda y un uso estable en espacios compartidos.
-Bajo Mantenimiento y Uso Intensivo – La superficie lisa permite una limpieza rápida y sencilla, algo esencial en bancos para vestuario, gimnasios o colegios donde la higiene y la practicidad son prioritarias.</t>
-  </si>
-  <si>
     <t>banco vestuario bancos para cocina banco cocina taquilla vestuario bancos banco exterior banquito</t>
   </si>
   <si>
@@ -4149,6 +4142,13 @@
   </si>
   <si>
     <t>Twinthink Metal Changing Room Bench for Gyms and Schools (White/Black)</t>
+  </si>
+  <si>
+    <t>Uso Profesional Para Vestuarios y Gimnasios – Banco diseñado para vestuarios, gimnasios, colegios, zonas de cambio y espacios colectivos donde se necesita una solución resistente, funcional y preparada para uso frecuente.
+Estructura Metálica Resistente – Fabricado con estructura de acero robusta para ofrecer estabilidad y durabilidad en el uso diario. Ideal para entornos profesionales con tránsito continuo y exigencia de resistencia.
+Acabado Duradero y Fácil de Limpiar – Su pintura/acabado protege la superficie y facilita el mantenimiento. El banco conserva una estética limpia y profesional, adecuada para instalaciones deportivas y educativas.
+Medidas Funcionales y Capacidad de Carga – Dimensiones: 90x32x45 cm. Capacidad de carga recomendada: 150 kg. Formato pensado para ofrecer una sentada cómoda y un uso estable en espacios compartidos.
+Bajo Mantenimiento y Uso Intensivo – La superficie lisa permite una limpieza rápida y sencilla, algo esencial en bancos para vestuario, gimnasios o colegios donde la higiene y la practicidad son prioritarias.</t>
   </si>
 </sst>
 </file>
@@ -16718,52 +16718,52 @@
         <v>1275</v>
       </c>
       <c r="N33" s="14" t="s">
+        <v>1340</v>
+      </c>
+      <c r="O33" t="s">
         <v>1276</v>
       </c>
-      <c r="O33" t="s">
+      <c r="P33" t="s">
         <v>1277</v>
       </c>
-      <c r="P33" t="s">
+      <c r="Q33" t="s">
         <v>1278</v>
       </c>
-      <c r="Q33" t="s">
+      <c r="T33" t="s">
         <v>1279</v>
       </c>
-      <c r="T33" t="s">
+      <c r="U33" t="s">
         <v>1280</v>
       </c>
-      <c r="U33" t="s">
+      <c r="X33" t="s">
         <v>1281</v>
       </c>
-      <c r="X33" t="s">
+      <c r="Y33" t="s">
         <v>1282</v>
       </c>
-      <c r="Y33" t="s">
-        <v>1283</v>
-      </c>
       <c r="AB33" t="s">
+        <v>1326</v>
+      </c>
+      <c r="AC33" t="s">
         <v>1327</v>
       </c>
-      <c r="AC33" t="s">
+      <c r="AD33" s="14" t="s">
         <v>1328</v>
       </c>
-      <c r="AD33" s="14" t="s">
+      <c r="AE33" t="s">
         <v>1329</v>
       </c>
-      <c r="AE33" t="s">
+      <c r="AF33" t="s">
         <v>1330</v>
       </c>
-      <c r="AF33" t="s">
+      <c r="AG33" t="s">
         <v>1331</v>
       </c>
-      <c r="AG33" t="s">
+      <c r="AH33" s="14" t="s">
         <v>1332</v>
       </c>
-      <c r="AH33" s="14" t="s">
+      <c r="AI33" t="s">
         <v>1333</v>
-      </c>
-      <c r="AI33" t="s">
-        <v>1334</v>
       </c>
       <c r="AJ33">
         <v>45</v>
@@ -16793,99 +16793,99 @@
         <v>149</v>
       </c>
       <c r="BB33" t="s">
+        <v>1283</v>
+      </c>
+      <c r="BC33" t="s">
         <v>1284</v>
       </c>
-      <c r="BC33" t="s">
+      <c r="BD33" t="s">
         <v>1285</v>
       </c>
-      <c r="BD33" t="s">
+      <c r="BE33" t="s">
         <v>1286</v>
       </c>
-      <c r="BE33" t="s">
+      <c r="BF33" t="s">
         <v>1287</v>
       </c>
-      <c r="BF33" t="s">
+      <c r="BG33" t="s">
         <v>1288</v>
       </c>
-      <c r="BG33" t="s">
-        <v>1289</v>
-      </c>
       <c r="BH33" t="s">
+        <v>1283</v>
+      </c>
+      <c r="BI33" t="s">
         <v>1284</v>
       </c>
-      <c r="BI33" t="s">
+      <c r="BJ33" t="s">
         <v>1285</v>
       </c>
-      <c r="BJ33" t="s">
+      <c r="BK33" t="s">
         <v>1286</v>
       </c>
-      <c r="BK33" t="s">
+      <c r="BL33" t="s">
         <v>1287</v>
       </c>
-      <c r="BL33" t="s">
+      <c r="BM33" t="s">
         <v>1288</v>
       </c>
-      <c r="BM33" t="s">
-        <v>1289</v>
-      </c>
       <c r="BN33" t="s">
+        <v>1283</v>
+      </c>
+      <c r="BO33" t="s">
         <v>1284</v>
       </c>
-      <c r="BO33" t="s">
+      <c r="BP33" t="s">
         <v>1285</v>
       </c>
-      <c r="BP33" t="s">
+      <c r="BQ33" t="s">
         <v>1286</v>
       </c>
-      <c r="BQ33" t="s">
+      <c r="BR33" t="s">
         <v>1287</v>
       </c>
-      <c r="BR33" t="s">
+      <c r="BS33" t="s">
         <v>1288</v>
       </c>
-      <c r="BS33" t="s">
-        <v>1289</v>
-      </c>
       <c r="BT33" t="s">
+        <v>1283</v>
+      </c>
+      <c r="BU33" t="s">
         <v>1284</v>
       </c>
-      <c r="BU33" t="s">
+      <c r="BV33" t="s">
         <v>1285</v>
       </c>
-      <c r="BV33" t="s">
+      <c r="BW33" t="s">
         <v>1286</v>
       </c>
-      <c r="BW33" t="s">
+      <c r="BX33" t="s">
         <v>1287</v>
       </c>
-      <c r="BX33" t="s">
+      <c r="BY33" t="s">
         <v>1288</v>
       </c>
-      <c r="BY33" t="s">
-        <v>1289</v>
-      </c>
       <c r="BZ33" t="s">
+        <v>1283</v>
+      </c>
+      <c r="CA33" t="s">
         <v>1284</v>
       </c>
-      <c r="CA33" t="s">
+      <c r="CB33" t="s">
         <v>1285</v>
       </c>
-      <c r="CB33" t="s">
+      <c r="CC33" t="s">
         <v>1286</v>
       </c>
-      <c r="CC33" t="s">
+      <c r="CD33" t="s">
         <v>1287</v>
       </c>
-      <c r="CD33" t="s">
+      <c r="CE33" t="s">
         <v>1288</v>
-      </c>
-      <c r="CE33" t="s">
-        <v>1289</v>
       </c>
     </row>
     <row r="34" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="B34" t="s">
         <v>1270</v>
@@ -16900,76 +16900,76 @@
         <v>182</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
       <c r="G34" t="s">
         <v>126</v>
       </c>
       <c r="H34" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="I34" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="J34" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="K34" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="L34" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="M34" t="s">
         <v>1275</v>
       </c>
       <c r="N34" s="14" t="s">
+        <v>1340</v>
+      </c>
+      <c r="O34" t="s">
         <v>1276</v>
       </c>
-      <c r="O34" t="s">
-        <v>1277</v>
-      </c>
       <c r="P34" t="s">
+        <v>1292</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>1278</v>
+      </c>
+      <c r="T34" t="s">
         <v>1293</v>
       </c>
-      <c r="Q34" t="s">
-        <v>1279</v>
-      </c>
-      <c r="T34" t="s">
+      <c r="U34" t="s">
+        <v>1280</v>
+      </c>
+      <c r="X34" t="s">
         <v>1294</v>
       </c>
-      <c r="U34" t="s">
-        <v>1281</v>
-      </c>
-      <c r="X34" t="s">
-        <v>1295</v>
-      </c>
       <c r="Y34" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="AB34" t="s">
+        <v>1334</v>
+      </c>
+      <c r="AC34" t="s">
+        <v>1327</v>
+      </c>
+      <c r="AD34" s="14" t="s">
+        <v>1328</v>
+      </c>
+      <c r="AE34" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AF34" t="s">
         <v>1335</v>
       </c>
-      <c r="AC34" t="s">
-        <v>1328</v>
-      </c>
-      <c r="AD34" s="14" t="s">
-        <v>1329</v>
-      </c>
-      <c r="AE34" t="s">
-        <v>1330</v>
-      </c>
-      <c r="AF34" t="s">
-        <v>1336</v>
-      </c>
       <c r="AG34" t="s">
+        <v>1331</v>
+      </c>
+      <c r="AH34" s="14" t="s">
         <v>1332</v>
       </c>
-      <c r="AH34" s="14" t="s">
+      <c r="AI34" t="s">
         <v>1333</v>
-      </c>
-      <c r="AI34" t="s">
-        <v>1334</v>
       </c>
       <c r="AJ34">
         <v>45</v>
@@ -16999,99 +16999,99 @@
         <v>149</v>
       </c>
       <c r="BB34" t="s">
+        <v>1295</v>
+      </c>
+      <c r="BC34" t="s">
         <v>1296</v>
       </c>
-      <c r="BC34" t="s">
+      <c r="BD34" t="s">
         <v>1297</v>
       </c>
-      <c r="BD34" t="s">
+      <c r="BE34" t="s">
         <v>1298</v>
       </c>
-      <c r="BE34" t="s">
+      <c r="BF34" t="s">
         <v>1299</v>
       </c>
-      <c r="BF34" t="s">
+      <c r="BG34" t="s">
         <v>1300</v>
       </c>
-      <c r="BG34" t="s">
-        <v>1301</v>
-      </c>
       <c r="BH34" t="s">
+        <v>1295</v>
+      </c>
+      <c r="BI34" t="s">
         <v>1296</v>
       </c>
-      <c r="BI34" t="s">
+      <c r="BJ34" t="s">
         <v>1297</v>
       </c>
-      <c r="BJ34" t="s">
+      <c r="BK34" t="s">
         <v>1298</v>
       </c>
-      <c r="BK34" t="s">
+      <c r="BL34" t="s">
         <v>1299</v>
       </c>
-      <c r="BL34" t="s">
+      <c r="BM34" t="s">
         <v>1300</v>
       </c>
-      <c r="BM34" t="s">
-        <v>1301</v>
-      </c>
       <c r="BN34" t="s">
+        <v>1295</v>
+      </c>
+      <c r="BO34" t="s">
         <v>1296</v>
       </c>
-      <c r="BO34" t="s">
+      <c r="BP34" t="s">
         <v>1297</v>
       </c>
-      <c r="BP34" t="s">
+      <c r="BQ34" t="s">
         <v>1298</v>
       </c>
-      <c r="BQ34" t="s">
+      <c r="BR34" t="s">
         <v>1299</v>
       </c>
-      <c r="BR34" t="s">
+      <c r="BS34" t="s">
         <v>1300</v>
       </c>
-      <c r="BS34" t="s">
-        <v>1301</v>
-      </c>
       <c r="BT34" t="s">
+        <v>1295</v>
+      </c>
+      <c r="BU34" t="s">
         <v>1296</v>
       </c>
-      <c r="BU34" t="s">
+      <c r="BV34" t="s">
         <v>1297</v>
       </c>
-      <c r="BV34" t="s">
+      <c r="BW34" t="s">
         <v>1298</v>
       </c>
-      <c r="BW34" t="s">
+      <c r="BX34" t="s">
         <v>1299</v>
       </c>
-      <c r="BX34" t="s">
+      <c r="BY34" t="s">
         <v>1300</v>
       </c>
-      <c r="BY34" t="s">
-        <v>1301</v>
-      </c>
       <c r="BZ34" t="s">
+        <v>1295</v>
+      </c>
+      <c r="CA34" t="s">
         <v>1296</v>
       </c>
-      <c r="CA34" t="s">
+      <c r="CB34" t="s">
         <v>1297</v>
       </c>
-      <c r="CB34" t="s">
+      <c r="CC34" t="s">
         <v>1298</v>
       </c>
-      <c r="CC34" t="s">
+      <c r="CD34" t="s">
         <v>1299</v>
       </c>
-      <c r="CD34" t="s">
+      <c r="CE34" t="s">
         <v>1300</v>
-      </c>
-      <c r="CE34" t="s">
-        <v>1301</v>
       </c>
     </row>
     <row r="35" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="B35" t="s">
         <v>1270</v>
@@ -17106,76 +17106,76 @@
         <v>221</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="G35" t="s">
         <v>126</v>
       </c>
       <c r="H35" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="I35" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="J35" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="K35" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="L35" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="M35" t="s">
         <v>1275</v>
       </c>
       <c r="N35" s="14" t="s">
+        <v>1340</v>
+      </c>
+      <c r="O35" t="s">
         <v>1276</v>
       </c>
-      <c r="O35" t="s">
-        <v>1277</v>
-      </c>
       <c r="P35" t="s">
+        <v>1304</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>1278</v>
+      </c>
+      <c r="T35" t="s">
         <v>1305</v>
       </c>
-      <c r="Q35" t="s">
-        <v>1279</v>
-      </c>
-      <c r="T35" t="s">
+      <c r="U35" t="s">
+        <v>1280</v>
+      </c>
+      <c r="X35" t="s">
         <v>1306</v>
       </c>
-      <c r="U35" t="s">
-        <v>1281</v>
-      </c>
-      <c r="X35" t="s">
-        <v>1307</v>
-      </c>
       <c r="Y35" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="AB35" t="s">
+        <v>1336</v>
+      </c>
+      <c r="AC35" t="s">
+        <v>1327</v>
+      </c>
+      <c r="AD35" s="14" t="s">
+        <v>1328</v>
+      </c>
+      <c r="AE35" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AF35" t="s">
         <v>1337</v>
       </c>
-      <c r="AC35" t="s">
-        <v>1328</v>
-      </c>
-      <c r="AD35" s="14" t="s">
-        <v>1329</v>
-      </c>
-      <c r="AE35" t="s">
-        <v>1330</v>
-      </c>
-      <c r="AF35" t="s">
-        <v>1338</v>
-      </c>
       <c r="AG35" t="s">
+        <v>1331</v>
+      </c>
+      <c r="AH35" s="14" t="s">
         <v>1332</v>
       </c>
-      <c r="AH35" s="14" t="s">
+      <c r="AI35" t="s">
         <v>1333</v>
-      </c>
-      <c r="AI35" t="s">
-        <v>1334</v>
       </c>
       <c r="AJ35">
         <v>45</v>
@@ -17205,99 +17205,99 @@
         <v>149</v>
       </c>
       <c r="BB35" t="s">
+        <v>1307</v>
+      </c>
+      <c r="BC35" t="s">
         <v>1308</v>
       </c>
-      <c r="BC35" t="s">
+      <c r="BD35" t="s">
         <v>1309</v>
       </c>
-      <c r="BD35" t="s">
+      <c r="BE35" t="s">
         <v>1310</v>
       </c>
-      <c r="BE35" t="s">
+      <c r="BF35" t="s">
         <v>1311</v>
       </c>
-      <c r="BF35" t="s">
+      <c r="BG35" t="s">
         <v>1312</v>
       </c>
-      <c r="BG35" t="s">
-        <v>1313</v>
-      </c>
       <c r="BH35" t="s">
+        <v>1307</v>
+      </c>
+      <c r="BI35" t="s">
         <v>1308</v>
       </c>
-      <c r="BI35" t="s">
+      <c r="BJ35" t="s">
         <v>1309</v>
       </c>
-      <c r="BJ35" t="s">
+      <c r="BK35" t="s">
         <v>1310</v>
       </c>
-      <c r="BK35" t="s">
+      <c r="BL35" t="s">
         <v>1311</v>
       </c>
-      <c r="BL35" t="s">
+      <c r="BM35" t="s">
         <v>1312</v>
       </c>
-      <c r="BM35" t="s">
-        <v>1313</v>
-      </c>
       <c r="BN35" t="s">
+        <v>1307</v>
+      </c>
+      <c r="BO35" t="s">
         <v>1308</v>
       </c>
-      <c r="BO35" t="s">
+      <c r="BP35" t="s">
         <v>1309</v>
       </c>
-      <c r="BP35" t="s">
+      <c r="BQ35" t="s">
         <v>1310</v>
       </c>
-      <c r="BQ35" t="s">
+      <c r="BR35" t="s">
         <v>1311</v>
       </c>
-      <c r="BR35" t="s">
+      <c r="BS35" t="s">
         <v>1312</v>
       </c>
-      <c r="BS35" t="s">
-        <v>1313</v>
-      </c>
       <c r="BT35" t="s">
+        <v>1307</v>
+      </c>
+      <c r="BU35" t="s">
         <v>1308</v>
       </c>
-      <c r="BU35" t="s">
+      <c r="BV35" t="s">
         <v>1309</v>
       </c>
-      <c r="BV35" t="s">
+      <c r="BW35" t="s">
         <v>1310</v>
       </c>
-      <c r="BW35" t="s">
+      <c r="BX35" t="s">
         <v>1311</v>
       </c>
-      <c r="BX35" t="s">
+      <c r="BY35" t="s">
         <v>1312</v>
       </c>
-      <c r="BY35" t="s">
-        <v>1313</v>
-      </c>
       <c r="BZ35" t="s">
+        <v>1307</v>
+      </c>
+      <c r="CA35" t="s">
         <v>1308</v>
       </c>
-      <c r="CA35" t="s">
+      <c r="CB35" t="s">
         <v>1309</v>
       </c>
-      <c r="CB35" t="s">
+      <c r="CC35" t="s">
         <v>1310</v>
       </c>
-      <c r="CC35" t="s">
+      <c r="CD35" t="s">
         <v>1311</v>
       </c>
-      <c r="CD35" t="s">
+      <c r="CE35" t="s">
         <v>1312</v>
-      </c>
-      <c r="CE35" t="s">
-        <v>1313</v>
       </c>
     </row>
     <row r="36" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="B36" t="s">
         <v>1270</v>
@@ -17312,76 +17312,76 @@
         <v>259</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="G36" t="s">
         <v>126</v>
       </c>
       <c r="H36" t="s">
+        <v>1315</v>
+      </c>
+      <c r="I36" t="s">
+        <v>1315</v>
+      </c>
+      <c r="J36" t="s">
+        <v>1315</v>
+      </c>
+      <c r="K36" t="s">
+        <v>1315</v>
+      </c>
+      <c r="L36" t="s">
         <v>1316</v>
-      </c>
-      <c r="I36" t="s">
-        <v>1316</v>
-      </c>
-      <c r="J36" t="s">
-        <v>1316</v>
-      </c>
-      <c r="K36" t="s">
-        <v>1316</v>
-      </c>
-      <c r="L36" t="s">
-        <v>1317</v>
       </c>
       <c r="M36" t="s">
         <v>1275</v>
       </c>
       <c r="N36" s="14" t="s">
+        <v>1340</v>
+      </c>
+      <c r="O36" t="s">
         <v>1276</v>
       </c>
-      <c r="O36" t="s">
-        <v>1277</v>
-      </c>
       <c r="P36" t="s">
+        <v>1317</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>1278</v>
+      </c>
+      <c r="T36" t="s">
         <v>1318</v>
       </c>
-      <c r="Q36" t="s">
-        <v>1279</v>
-      </c>
-      <c r="T36" t="s">
+      <c r="U36" t="s">
+        <v>1280</v>
+      </c>
+      <c r="X36" t="s">
         <v>1319</v>
       </c>
-      <c r="U36" t="s">
-        <v>1281</v>
-      </c>
-      <c r="X36" t="s">
-        <v>1320</v>
-      </c>
       <c r="Y36" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="AB36" t="s">
+        <v>1338</v>
+      </c>
+      <c r="AC36" t="s">
+        <v>1327</v>
+      </c>
+      <c r="AD36" s="14" t="s">
+        <v>1328</v>
+      </c>
+      <c r="AE36" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AF36" t="s">
         <v>1339</v>
       </c>
-      <c r="AC36" t="s">
-        <v>1328</v>
-      </c>
-      <c r="AD36" s="14" t="s">
-        <v>1329</v>
-      </c>
-      <c r="AE36" t="s">
-        <v>1330</v>
-      </c>
-      <c r="AF36" t="s">
-        <v>1340</v>
-      </c>
       <c r="AG36" t="s">
+        <v>1331</v>
+      </c>
+      <c r="AH36" s="14" t="s">
         <v>1332</v>
       </c>
-      <c r="AH36" s="14" t="s">
+      <c r="AI36" t="s">
         <v>1333</v>
-      </c>
-      <c r="AI36" t="s">
-        <v>1334</v>
       </c>
       <c r="AJ36">
         <v>45</v>
@@ -17411,94 +17411,94 @@
         <v>149</v>
       </c>
       <c r="BB36" t="s">
+        <v>1320</v>
+      </c>
+      <c r="BC36" t="s">
         <v>1321</v>
       </c>
-      <c r="BC36" t="s">
+      <c r="BD36" t="s">
         <v>1322</v>
       </c>
-      <c r="BD36" t="s">
+      <c r="BE36" t="s">
         <v>1323</v>
       </c>
-      <c r="BE36" t="s">
+      <c r="BF36" t="s">
         <v>1324</v>
       </c>
-      <c r="BF36" t="s">
+      <c r="BG36" t="s">
         <v>1325</v>
       </c>
-      <c r="BG36" t="s">
-        <v>1326</v>
-      </c>
       <c r="BH36" t="s">
+        <v>1320</v>
+      </c>
+      <c r="BI36" t="s">
         <v>1321</v>
       </c>
-      <c r="BI36" t="s">
+      <c r="BJ36" t="s">
         <v>1322</v>
       </c>
-      <c r="BJ36" t="s">
+      <c r="BK36" t="s">
         <v>1323</v>
       </c>
-      <c r="BK36" t="s">
+      <c r="BL36" t="s">
         <v>1324</v>
       </c>
-      <c r="BL36" t="s">
+      <c r="BM36" t="s">
         <v>1325</v>
       </c>
-      <c r="BM36" t="s">
-        <v>1326</v>
-      </c>
       <c r="BN36" t="s">
+        <v>1320</v>
+      </c>
+      <c r="BO36" t="s">
         <v>1321</v>
       </c>
-      <c r="BO36" t="s">
+      <c r="BP36" t="s">
         <v>1322</v>
       </c>
-      <c r="BP36" t="s">
+      <c r="BQ36" t="s">
         <v>1323</v>
       </c>
-      <c r="BQ36" t="s">
+      <c r="BR36" t="s">
         <v>1324</v>
       </c>
-      <c r="BR36" t="s">
+      <c r="BS36" t="s">
         <v>1325</v>
       </c>
-      <c r="BS36" t="s">
-        <v>1326</v>
-      </c>
       <c r="BT36" t="s">
+        <v>1320</v>
+      </c>
+      <c r="BU36" t="s">
         <v>1321</v>
       </c>
-      <c r="BU36" t="s">
+      <c r="BV36" t="s">
         <v>1322</v>
       </c>
-      <c r="BV36" t="s">
+      <c r="BW36" t="s">
         <v>1323</v>
       </c>
-      <c r="BW36" t="s">
+      <c r="BX36" t="s">
         <v>1324</v>
       </c>
-      <c r="BX36" t="s">
+      <c r="BY36" t="s">
         <v>1325</v>
       </c>
-      <c r="BY36" t="s">
-        <v>1326</v>
-      </c>
       <c r="BZ36" t="s">
+        <v>1320</v>
+      </c>
+      <c r="CA36" t="s">
         <v>1321</v>
       </c>
-      <c r="CA36" t="s">
+      <c r="CB36" t="s">
         <v>1322</v>
       </c>
-      <c r="CB36" t="s">
+      <c r="CC36" t="s">
         <v>1323</v>
       </c>
-      <c r="CC36" t="s">
+      <c r="CD36" t="s">
         <v>1324</v>
       </c>
-      <c r="CD36" t="s">
+      <c r="CE36" t="s">
         <v>1325</v>
-      </c>
-      <c r="CE36" t="s">
-        <v>1326</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Maestro: bancos metalicos 150 cm (B.MET.150, 4 colores)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/datos/FICHERO_MAESTRO2.xlsx
+++ b/public/datos/FICHERO_MAESTRO2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Helian\Desktop\Fichero Maestro\Sistema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC75FE3-3CFC-41ED-BCFE-537A60222BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAEA62F0-F392-43B2-B041-015034B42A7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="591" xr2:uid="{90124268-D67C-4387-8829-7E3B806257E6}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3201" uniqueCount="1341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3469" uniqueCount="1460">
   <si>
     <t>Marketplace</t>
   </si>
@@ -4149,6 +4149,387 @@
 Acabado Duradero y Fácil de Limpiar – Su pintura/acabado protege la superficie y facilita el mantenimiento. El banco conserva una estética limpia y profesional, adecuada para instalaciones deportivas y educativas.
 Medidas Funcionales y Capacidad de Carga – Dimensiones: 90x32x45 cm. Capacidad de carga recomendada: 150 kg. Formato pensado para ofrecer una sentada cómoda y un uso estable en espacios compartidos.
 Bajo Mantenimiento y Uso Intensivo – La superficie lisa permite una limpieza rápida y sencilla, algo esencial en bancos para vestuario, gimnasios o colegios donde la higiene y la practicidad son prioritarias.</t>
+  </si>
+  <si>
+    <t>B.MET.150_G</t>
+  </si>
+  <si>
+    <t>150</t>
+  </si>
+  <si>
+    <t>8437027641350</t>
+  </si>
+  <si>
+    <t>B.MET.150</t>
+  </si>
+  <si>
+    <t>El banco vestuario metálico Twinthink es una solución práctica, resistente y versátil para equipar vestuarios, gimnasios, colegios, oficinas y zonas comunes con un asiento funcional y duradero. Diseñado para ofrecer comodidad y estabilidad en el uso diario, este banco metálico para vestuario combina una estructura robusta con un estilo limpio y profesional que se adapta fácilmente a distintos entornos.&lt;br&gt;&lt;br&gt;Fabricado en acero de alta resistencia, este banco vestuario está pensado para soportar un uso frecuente tanto en espacios interiores como en zonas cubiertas de exterior. Su diseño metálico facilita la limpieza y el mantenimiento, lo que lo convierte en una opción muy práctica para lugares donde la higiene y la durabilidad son esenciales. Gracias a su superficie lisa y a su estructura firme, ofrece una experiencia cómoda y estable al sentarse.&lt;br&gt;&lt;br&gt;Este modelo es ideal para colocar junto a una taquilla vestuario, facilitando el cambio de ropa, calzado o accesorios en gimnasios, centros deportivos, empresas, colegios o vestuarios colectivos. También puede utilizarse como banco exterior en patios cubiertos, entradas o áreas de espera, aportando una solución funcional con estética moderna.&lt;br&gt;&lt;br&gt;Además de su resistencia, el banco metálico de Twinthink destaca por su versatilidad. Puede utilizarse en espacios profesionales o domésticos, adaptándose a distintas necesidades sin perder su estilo sobrio y eficiente. Su formato permite optimizar el espacio disponible y mantener el orden en zonas de paso o de uso común.&lt;br&gt;&lt;br&gt;Si buscas uno de esos bancos metálicos que combinan resistencia, fácil mantenimiento y diseño práctico, el banco para vestuario Twinthink es una excelente opción para mejorar cualquier espacio con una solución duradera, cómoda y funcional.</t>
+  </si>
+  <si>
+    <t>Uso profesional para vestuarios y gimnasios – Banco diseñado para vestuarios, gimnasios, colegios y espacios colectivos que necesitan una solución resistente, funcional y preparada para uso frecuente.
+Dos niveles: asiento y zapatero – Asiento de 4 lamas en la parte superior y nivel inferior para dejar el calzado, para mantener el vestuario ordenado.
+Estructura de acero y pies regulables – Estructura robusta, firme y estable para el uso diario. Los pies regulables en altura nivelan el banco en suelos irregulares.
+Medidas y capacidad de carga – Dimensiones: 150 x 32 x 45 cm. Capacidad de carga recomendada: 250 kg. Espacio para que se sienten varias personas a la vez.
+Fácil de limpiar – Superficie lisa y acabado duradero que se limpia en segundos, algo esencial en vestuarios, gimnasios o colegios donde la higiene es prioritaria.</t>
+  </si>
+  <si>
+    <t>O banco de vestiário metálico Twinthink é uma solução prática, resistente e versátil para equipar vestiários, ginásios, escolas, escritórios e zonas comuns com um assento funcional e duradouro. Concebido para oferecer conforto e estabilidade no uso diário, este banco metálico para vestiário combina uma estrutura robusta com um estilo limpo e profissional que se adapta facilmente a diferentes ambientes.&lt;br&gt;&lt;br&gt;Fabricado em aço de alta resistência, este banco de vestiário foi pensado para suportar uma utilização frequente tanto em espaços interiores como em zonas cobertas de exterior. O seu design metálico facilita a limpeza e a manutenção, o que o torna uma opção muito prática para locais onde a higiene e a durabilidade são essenciais. Graças à sua superfície lisa e à sua estrutura firme, oferece uma experiência cómoda e estável ao sentar.&lt;br&gt;&lt;br&gt;Este modelo é ideal para colocar junto a um cacifo de vestiário, facilitando a mudança de roupa, calçado ou acessórios em ginásios, centros desportivos, empresas, escolas ou vestiários coletivos. Também pode ser utilizado como banco de exterior em pátios cobertos, entradas ou áreas de espera, proporcionando uma solução funcional com estética moderna.&lt;br&gt;&lt;br&gt;Além da sua resistência, o banco metálico da Twinthink destaca-se pela sua versatilidade. Pode ser utilizado em espaços profissionais ou domésticos, adaptando-se a diferentes necessidades sem perder o seu estilo sóbrio e eficiente. O seu formato permite otimizar o espaço disponível e manter a ordem em zonas de passagem ou de uso comum.&lt;br&gt;&lt;br&gt;Se procura um banco metálico que combine resistência, fácil manutenção e design prático, o banco de vestiário Twinthink é uma excelente opção para melhorar qualquer espaço com uma solução duradoura, cómoda e funcional.</t>
+  </si>
+  <si>
+    <t>Uso profissional para vestiários e ginásios – Banco concebido para vestiários, ginásios, escolas e espaços coletivos que precisam de uma solução resistente, funcional e preparada para uso frequente.
+Dois níveis: assento e sapateira – Assento de 4 ripas na parte superior e nível inferior para o calçado, para manter o vestiário arrumado.
+Estrutura em aço e pés reguláveis – Estrutura robusta, firme e estável para o uso diário. Os pés reguláveis em altura nivelam o banco em pavimentos irregulares.
+Medidas e capacidade de carga – Dimensões: 150 x 32 x 45 cm. Carga recomendada: 250 kg. Espaço para várias pessoas se sentarem ao mesmo tempo.
+Fácil de limpar – Superfície lisa e acabamento duradouro que se limpa em segundos, essencial em vestiários, ginásios ou escolas onde a higiene é prioritária.</t>
+  </si>
+  <si>
+    <t>Le banc de vestiaire métallique Twinthink est une solution pratique, résistante et polyvalente pour équiper vestiaires, salles de sport, écoles, bureaux et espaces communs d'une assise fonctionnelle et durable. Conçu pour offrir confort et stabilité au quotidien, ce banc métallique de vestiaire associe une structure robuste à un style épuré et professionnel qui s'adapte facilement à différents environnements.&lt;br&gt;&lt;br&gt;Fabriqué en acier haute résistance, ce banc de vestiaire est pensé pour supporter un usage fréquent aussi bien à l'intérieur que dans les zones extérieures couvertes. Sa conception métallique facilite le nettoyage et l'entretien, ce qui en fait une option très pratique pour les lieux où l'hygiène et la durabilité sont essentielles. Grâce à sa surface lisse et à sa structure ferme, il offre une assise confortable et stable.&lt;br&gt;&lt;br&gt;Ce modèle est idéal à placer à côté d'un casier de vestiaire, facilitant le changement de vêtements, de chaussures ou d'accessoires dans les salles de sport, centres sportifs, entreprises, écoles ou vestiaires collectifs. Il peut également être utilisé comme banc d'extérieur dans les cours couvertes, les entrées ou les zones d'attente, apportant une solution fonctionnelle à l'esthétique moderne.&lt;br&gt;&lt;br&gt;Outre sa résistance, le banc métallique Twinthink se distingue par sa polyvalence. Il peut être utilisé dans des espaces professionnels ou domestiques, s'adaptant à différents besoins sans perdre son style sobre et efficace. Son format permet d'optimiser l'espace disponible et de maintenir l'ordre dans les zones de passage ou d'usage commun.&lt;br&gt;&lt;br&gt;Si vous cherchez un banc métallique alliant résistance, entretien facile et design pratique, le banc de vestiaire Twinthink est un excellent choix pour améliorer n'importe quel espace avec une solution durable, confortable et fonctionnelle.</t>
+  </si>
+  <si>
+    <t>Usage professionnel pour vestiaires et salles de sport – Banc conçu pour les vestiaires, salles de sport, écoles et espaces collectifs qui ont besoin d'une solution résistante, fonctionnelle et prête pour un usage fréquent.
+Deux niveaux : assise et range-chaussures – Assise à 4 lattes en partie haute et niveau inférieur pour poser les chaussures, pour garder le vestiaire bien rangé.
+Structure en acier et pieds réglables – Structure robuste, ferme et stable pour un usage quotidien. Les pieds réglables en hauteur mettent le banc à niveau sur les sols irréguliers.
+Dimensions et capacité de charge – Dimensions : 150 x 32 x 45 cm. Charge recommandée : 250 kg. De la place pour que plusieurs personnes s'assoient en même temps.
+Facile à nettoyer – Surface lisse et finition durable qui se nettoie en quelques secondes, essentiel dans les vestiaires, salles de sport ou écoles où l'hygiène est prioritaire.</t>
+  </si>
+  <si>
+    <t>La panca da spogliatoio in metallo Twinthink è una soluzione pratica, resistente e versatile per attrezzare spogliatoi, palestre, scuole, uffici e aree comuni con una seduta funzionale e duratura. Progettata per offrire comfort e stabilità nell'uso quotidiano, questa panca metallica da spogliatoio unisce una struttura robusta a uno stile pulito e professionale che si adatta facilmente a diversi ambienti.&lt;br&gt;&lt;br&gt;Realizzata in acciaio ad alta resistenza, questa panca da spogliatoio è pensata per sopportare un uso frequente sia negli spazi interni sia nelle zone esterne coperte. Il suo design metallico facilita la pulizia e la manutenzione, rendendola un'opzione molto pratica per luoghi in cui igiene e durata sono essenziali. Grazie alla superficie liscia e alla struttura solida, offre un'esperienza comoda e stabile da seduti.&lt;br&gt;&lt;br&gt;Questo modello è ideale da collocare accanto a un armadietto da spogliatoio, facilitando il cambio di vestiti, scarpe o accessori in palestre, centri sportivi, aziende, scuole o spogliatoi collettivi. Può essere utilizzata anche come panca da esterno in cortili coperti, ingressi o aree di attesa, offrendo una soluzione funzionale dall'estetica moderna.&lt;br&gt;&lt;br&gt;Oltre alla sua resistenza, la panca metallica Twinthink si distingue per la sua versatilità. Può essere utilizzata in spazi professionali o domestici, adattandosi a diverse esigenze senza perdere il suo stile sobrio ed efficiente. Il suo formato permette di ottimizzare lo spazio disponibile e mantenere l'ordine nelle zone di passaggio o di uso comune.&lt;br&gt;&lt;br&gt;Se cerchi una panca metallica che unisca resistenza, facile manutenzione e design pratico, la panca da spogliatoio Twinthink è un'ottima scelta per migliorare qualsiasi spazio con una soluzione duratura, comoda e funzionale.</t>
+  </si>
+  <si>
+    <t>Uso professionale per spogliatoi e palestre – Panca progettata per spogliatoi, palestre, scuole e spazi collettivi che richiedono una soluzione resistente, funzionale e pronta per un uso frequente.
+Due livelli: seduta e portascarpe – Seduta a 4 listelli nella parte superiore e ripiano inferiore per le scarpe, per mantenere lo spogliatoio in ordine.
+Struttura in acciaio e piedini regolabili – Struttura robusta, solida e stabile per l'uso quotidiano. I piedini regolabili in altezza livellano la panca sui pavimenti irregolari.
+Misure e portata – Dimensioni: 150 x 32 x 45 cm. Portata consigliata: 250 kg. Spazio per far sedere più persone contemporaneamente.
+Facile da pulire – Superficie liscia e finitura resistente che si pulisce in pochi secondi, essenziale in spogliatoi, palestre o scuole dove l'igiene è una priorità.</t>
+  </si>
+  <si>
+    <t>Die Metall-Umkleidebank von Twinthink ist eine praktische, robuste und vielseitige Lösung, um Umkleideräume, Fitnessstudios, Schulen, Büros und Gemeinschaftsbereiche mit einer funktionalen und langlebigen Sitzgelegenheit auszustatten. Sie wurde für Komfort und Stabilität im täglichen Gebrauch entwickelt und verbindet eine robuste Konstruktion mit einem klaren, professionellen Stil, der sich mühelos in unterschiedliche Umgebungen einfügt.&lt;br&gt;&lt;br&gt;Die aus hochfestem Stahl gefertigte Umkleidebank ist für die häufige Nutzung sowohl in Innenräumen als auch in überdachten Außenbereichen ausgelegt. Dank der Metallausführung lässt sie sich leicht reinigen und pflegen – ideal für Orte, an denen Hygiene und Langlebigkeit entscheidend sind. Die glatte Oberfläche und die stabile Konstruktion sorgen für ein bequemes und sicheres Sitzen.&lt;br&gt;&lt;br&gt;Dieses Modell eignet sich ideal als Ergänzung zu einem Umkleidespind und erleichtert das Wechseln von Kleidung, Schuhen oder Accessoires in Fitnessstudios, Sportzentren, Unternehmen, Schulen oder Gemeinschaftsumkleiden. Sie kann auch als Außenbank in überdachten Innenhöfen, Eingangsbereichen oder Wartezonen eingesetzt werden und bietet eine funktionale Lösung mit modernem Design.&lt;br&gt;&lt;br&gt;Neben ihrer Robustheit überzeugt die Metallbank von Twinthink durch ihre Vielseitigkeit. Sie lässt sich im gewerblichen wie im privaten Bereich einsetzen und passt sich unterschiedlichen Anforderungen an, ohne ihren schlichten und effizienten Stil zu verlieren. Ihr Format hilft, den verfügbaren Platz optimal zu nutzen und Durchgangs- oder Gemeinschaftsbereiche ordentlich zu halten.&lt;br&gt;&lt;br&gt;Wenn Sie eine Metallbank suchen, die Robustheit, einfache Pflege und praktisches Design vereint, ist die Umkleidebank von Twinthink eine ausgezeichnete Wahl, um jeden Raum mit einer langlebigen, bequemen und funktionalen Lösung aufzuwerten.</t>
+  </si>
+  <si>
+    <t>Professioneller Einsatz in Umkleiden und Fitnessstudios – Bank für Umkleideräume, Fitnessstudios, Schulen und Gemeinschaftsräume, in denen eine robuste, funktionale und für die häufige Nutzung ausgelegte Lösung gefragt ist.
+Zwei Ebenen: Sitz und Schuhablage – Sitzfläche aus 4 Latten oben und eine untere Ebene für Schuhe, damit die Umkleide ordentlich bleibt.
+Stahlgestell und verstellbare Füße – Robustes, festes und stabiles Gestell für den täglichen Gebrauch. Die höhenverstellbaren Füße gleichen unebene Böden aus.
+Maße und Belastbarkeit – Abmessungen: 150 x 32 x 45 cm. Empfohlene Belastbarkeit: 250 kg. Platz für mehrere Personen gleichzeitig.
+Leicht zu reinigen – Glatte Oberfläche und langlebige Beschichtung, in Sekunden gereinigt – unverzichtbar in Umkleiden, Fitnessstudios oder Schulen, wo Hygiene an erster Stelle steht.</t>
+  </si>
+  <si>
+    <t>Professional Use for Changing Rooms and Gyms – Bench designed for changing rooms, gyms, schools and communal spaces that need a sturdy, functional solution ready for frequent use.
+Two Levels: Seat and Shoe Rack – 4-slat seat on top and a lower level for shoes, keeping the changing room tidy.
+Steel Frame and Adjustable Feet – Robust, firm and stable frame for everyday use. Height-adjustable feet level the bench on uneven floors.
+Dimensions and Load Capacity – Dimensions: 150 x 32 x 45 cm. Recommended load capacity: 250 kg. Room for several people to sit at once.
+Easy to Clean – Smooth surface and durable finish that wipes clean in seconds, essential in changing rooms, gyms or schools where hygiene is a priority.</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195056/bancos/B.MET.150/gris/es/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195061/bancos/B.MET.150/gris/es/pt01.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195066/bancos/B.MET.150/gris/es/pt02.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195073/bancos/B.MET.150/gris/es/pt03.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195078/bancos/B.MET.150/gris/es/pt04.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195084/bancos/B.MET.150/gris/es/pt05.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195143/bancos/B.MET.150/gris/it/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195148/bancos/B.MET.150/gris/it/pt01.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195155/bancos/B.MET.150/gris/it/pt02.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195164/bancos/B.MET.150/gris/it/pt03.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195169/bancos/B.MET.150/gris/it/pt04.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195175/bancos/B.MET.150/gris/it/pt05.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195103/bancos/B.MET.150/gris/fr/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195108/bancos/B.MET.150/gris/fr/pt01.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195114/bancos/B.MET.150/gris/fr/pt02.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195118/bancos/B.MET.150/gris/fr/pt03.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195122/bancos/B.MET.150/gris/fr/pt04.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195127/bancos/B.MET.150/gris/fr/pt05.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195006/bancos/B.MET.150/gris/en/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195011/bancos/B.MET.150/gris/en/pt01.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195017/bancos/B.MET.150/gris/en/pt02.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195023/bancos/B.MET.150/gris/en/pt03.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195029/bancos/B.MET.150/gris/en/pt04.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195036/bancos/B.MET.150/gris/en/pt05.png</t>
+  </si>
+  <si>
+    <t>B.MET.150_N</t>
+  </si>
+  <si>
+    <t>8437027641374</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195250/bancos/B.MET.150/negro/es/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195252/bancos/B.MET.150/negro/es/pt01.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195254/bancos/B.MET.150/negro/es/pt02.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195256/bancos/B.MET.150/negro/es/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195257/bancos/B.MET.150/negro/es/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195259/bancos/B.MET.150/negro/es/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195309/bancos/B.MET.150/negro/it/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195314/bancos/B.MET.150/negro/it/pt01.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195320/bancos/B.MET.150/negro/it/pt02.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195326/bancos/B.MET.150/negro/it/pt03.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195332/bancos/B.MET.150/negro/it/pt04.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195337/bancos/B.MET.150/negro/it/pt05.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195267/bancos/B.MET.150/negro/fr/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195272/bancos/B.MET.150/negro/fr/pt01.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195277/bancos/B.MET.150/negro/fr/pt02.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195281/bancos/B.MET.150/negro/fr/pt03.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195285/bancos/B.MET.150/negro/fr/pt04.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195290/bancos/B.MET.150/negro/fr/pt05.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195198/bancos/B.MET.150/negro/en/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195204/bancos/B.MET.150/negro/en/pt01.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195209/bancos/B.MET.150/negro/en/pt02.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195215/bancos/B.MET.150/negro/en/pt03.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195220/bancos/B.MET.150/negro/en/pt04.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195226/bancos/B.MET.150/negro/en/pt05.png</t>
+  </si>
+  <si>
+    <t>B.MET.150_B</t>
+  </si>
+  <si>
+    <t>8437027641367</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194731/bancos/B.MET.150/blanco/es/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194736/bancos/B.MET.150/blanco/es/pt01.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194741/bancos/B.MET.150/blanco/es/pt02.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194747/bancos/B.MET.150/blanco/es/pt03.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194751/bancos/B.MET.150/blanco/es/pt04.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194756/bancos/B.MET.150/blanco/es/pt05.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194794/bancos/B.MET.150/blanco/it/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194799/bancos/B.MET.150/blanco/it/pt01.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194809/bancos/B.MET.150/blanco/it/pt02.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194812/bancos/B.MET.150/blanco/it/pt03.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194819/bancos/B.MET.150/blanco/it/pt04.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194829/bancos/B.MET.150/blanco/it/pt05.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194777/bancos/B.MET.150/blanco/fr/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194779/bancos/B.MET.150/blanco/fr/pt01.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194780/bancos/B.MET.150/blanco/fr/pt02.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194782/bancos/B.MET.150/blanco/fr/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194784/bancos/B.MET.150/blanco/fr/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194786/bancos/B.MET.150/blanco/fr/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194688/bancos/B.MET.150/blanco/en/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194693/bancos/B.MET.150/blanco/en/pt01.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194698/bancos/B.MET.150/blanco/en/pt02.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194704/bancos/B.MET.150/blanco/en/pt03.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194708/bancos/B.MET.150/blanco/en/pt04.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194714/bancos/B.MET.150/blanco/en/pt05.png</t>
+  </si>
+  <si>
+    <t>B.MET.150_B-N</t>
+  </si>
+  <si>
+    <t>8437027641381</t>
+  </si>
+  <si>
+    <t>B.MET.150_B&amp;N</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194896/bancos/B.MET.150/byn/es/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194901/bancos/B.MET.150/byn/es/pt01.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194908/bancos/B.MET.150/byn/es/pt02.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194913/bancos/B.MET.150/byn/es/pt03.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194919/bancos/B.MET.150/byn/es/pt04.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194924/bancos/B.MET.150/byn/es/pt05.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194963/bancos/B.MET.150/byn/it/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194967/bancos/B.MET.150/byn/it/pt01.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194971/bancos/B.MET.150/byn/it/pt02.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194976/bancos/B.MET.150/byn/it/pt03.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194980/bancos/B.MET.150/byn/it/pt04.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194985/bancos/B.MET.150/byn/it/pt05.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194942/bancos/B.MET.150/byn/fr/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194944/bancos/B.MET.150/byn/fr/pt01.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194947/bancos/B.MET.150/byn/fr/pt02.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194949/bancos/B.MET.150/byn/fr/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194951/bancos/B.MET.150/byn/fr/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194953/bancos/B.MET.150/byn/fr/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194850/bancos/B.MET.150/byn/en/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194856/bancos/B.MET.150/byn/en/pt01.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194861/bancos/B.MET.150/byn/en/pt02.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194866/bancos/B.MET.150/byn/en/pt03.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194872/bancos/B.MET.150/byn/en/pt04.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194877/bancos/B.MET.150/byn/en/pt05.png</t>
   </si>
 </sst>
 </file>
@@ -10040,7 +10421,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C52A7A11-77C7-4197-B539-DBD653EC8E79}">
-  <dimension ref="A1:CQ36"/>
+  <dimension ref="A1:CQ40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -17501,6 +17882,866 @@
         <v>1325</v>
       </c>
     </row>
+    <row r="37" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B37" t="s">
+        <v>1270</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>1342</v>
+      </c>
+      <c r="D37" t="s">
+        <v>123</v>
+      </c>
+      <c r="E37" t="s">
+        <v>124</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>1343</v>
+      </c>
+      <c r="G37" t="s">
+        <v>126</v>
+      </c>
+      <c r="H37" t="s">
+        <v>1344</v>
+      </c>
+      <c r="I37" t="s">
+        <v>1344</v>
+      </c>
+      <c r="J37" t="s">
+        <v>1344</v>
+      </c>
+      <c r="K37" t="s">
+        <v>1344</v>
+      </c>
+      <c r="L37" t="s">
+        <v>1274</v>
+      </c>
+      <c r="M37" t="s">
+        <v>1345</v>
+      </c>
+      <c r="N37" s="14" t="s">
+        <v>1346</v>
+      </c>
+      <c r="O37" t="s">
+        <v>1276</v>
+      </c>
+      <c r="P37" t="s">
+        <v>1277</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>1347</v>
+      </c>
+      <c r="R37" s="14" t="s">
+        <v>1348</v>
+      </c>
+      <c r="T37" t="s">
+        <v>1279</v>
+      </c>
+      <c r="U37" t="s">
+        <v>1349</v>
+      </c>
+      <c r="V37" s="14" t="s">
+        <v>1350</v>
+      </c>
+      <c r="X37" t="s">
+        <v>1281</v>
+      </c>
+      <c r="Y37" t="s">
+        <v>1351</v>
+      </c>
+      <c r="Z37" s="14" t="s">
+        <v>1352</v>
+      </c>
+      <c r="AB37" t="s">
+        <v>1326</v>
+      </c>
+      <c r="AC37" t="s">
+        <v>1353</v>
+      </c>
+      <c r="AD37" s="14" t="s">
+        <v>1354</v>
+      </c>
+      <c r="AE37" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AF37" t="s">
+        <v>1330</v>
+      </c>
+      <c r="AG37" t="s">
+        <v>1331</v>
+      </c>
+      <c r="AH37" s="14" t="s">
+        <v>1355</v>
+      </c>
+      <c r="AI37" t="s">
+        <v>1333</v>
+      </c>
+      <c r="AJ37">
+        <v>45</v>
+      </c>
+      <c r="AK37">
+        <v>150</v>
+      </c>
+      <c r="AL37">
+        <v>32</v>
+      </c>
+      <c r="AM37">
+        <v>15</v>
+      </c>
+      <c r="AN37" t="s">
+        <v>143</v>
+      </c>
+      <c r="AO37" t="s">
+        <v>144</v>
+      </c>
+      <c r="AP37" t="s">
+        <v>145</v>
+      </c>
+      <c r="AQ37" t="s">
+        <v>146</v>
+      </c>
+      <c r="AU37" t="s">
+        <v>1356</v>
+      </c>
+      <c r="BB37" t="s">
+        <v>1357</v>
+      </c>
+      <c r="BC37" t="s">
+        <v>1358</v>
+      </c>
+      <c r="BD37" t="s">
+        <v>1359</v>
+      </c>
+      <c r="BE37" t="s">
+        <v>1360</v>
+      </c>
+      <c r="BF37" t="s">
+        <v>1361</v>
+      </c>
+      <c r="BG37" t="s">
+        <v>1362</v>
+      </c>
+      <c r="BH37" t="s">
+        <v>1363</v>
+      </c>
+      <c r="BI37" t="s">
+        <v>1364</v>
+      </c>
+      <c r="BJ37" t="s">
+        <v>1365</v>
+      </c>
+      <c r="BK37" t="s">
+        <v>1366</v>
+      </c>
+      <c r="BL37" t="s">
+        <v>1367</v>
+      </c>
+      <c r="BM37" t="s">
+        <v>1368</v>
+      </c>
+      <c r="BN37" t="s">
+        <v>1369</v>
+      </c>
+      <c r="BO37" t="s">
+        <v>1370</v>
+      </c>
+      <c r="BP37" t="s">
+        <v>1371</v>
+      </c>
+      <c r="BQ37" t="s">
+        <v>1372</v>
+      </c>
+      <c r="BR37" t="s">
+        <v>1373</v>
+      </c>
+      <c r="BS37" t="s">
+        <v>1374</v>
+      </c>
+      <c r="BT37" t="s">
+        <v>1375</v>
+      </c>
+      <c r="BU37" t="s">
+        <v>1376</v>
+      </c>
+      <c r="BV37" t="s">
+        <v>1377</v>
+      </c>
+      <c r="BW37" t="s">
+        <v>1378</v>
+      </c>
+      <c r="BX37" t="s">
+        <v>1379</v>
+      </c>
+      <c r="BY37" t="s">
+        <v>1380</v>
+      </c>
+      <c r="BZ37" t="s">
+        <v>1375</v>
+      </c>
+      <c r="CA37" t="s">
+        <v>1376</v>
+      </c>
+      <c r="CB37" t="s">
+        <v>1377</v>
+      </c>
+      <c r="CC37" t="s">
+        <v>1378</v>
+      </c>
+      <c r="CD37" t="s">
+        <v>1379</v>
+      </c>
+      <c r="CE37" t="s">
+        <v>1380</v>
+      </c>
+    </row>
+    <row r="38" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>1381</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1270</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>1342</v>
+      </c>
+      <c r="D38" t="s">
+        <v>181</v>
+      </c>
+      <c r="E38" t="s">
+        <v>182</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>1382</v>
+      </c>
+      <c r="G38" t="s">
+        <v>126</v>
+      </c>
+      <c r="H38" t="s">
+        <v>1381</v>
+      </c>
+      <c r="I38" t="s">
+        <v>1381</v>
+      </c>
+      <c r="J38" t="s">
+        <v>1381</v>
+      </c>
+      <c r="K38" t="s">
+        <v>1381</v>
+      </c>
+      <c r="L38" t="s">
+        <v>1291</v>
+      </c>
+      <c r="M38" t="s">
+        <v>1345</v>
+      </c>
+      <c r="N38" s="14" t="s">
+        <v>1346</v>
+      </c>
+      <c r="O38" t="s">
+        <v>1276</v>
+      </c>
+      <c r="P38" t="s">
+        <v>1292</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>1347</v>
+      </c>
+      <c r="R38" s="14" t="s">
+        <v>1348</v>
+      </c>
+      <c r="T38" t="s">
+        <v>1293</v>
+      </c>
+      <c r="U38" t="s">
+        <v>1349</v>
+      </c>
+      <c r="V38" s="14" t="s">
+        <v>1350</v>
+      </c>
+      <c r="X38" t="s">
+        <v>1294</v>
+      </c>
+      <c r="Y38" t="s">
+        <v>1351</v>
+      </c>
+      <c r="Z38" s="14" t="s">
+        <v>1352</v>
+      </c>
+      <c r="AB38" t="s">
+        <v>1334</v>
+      </c>
+      <c r="AC38" t="s">
+        <v>1353</v>
+      </c>
+      <c r="AD38" s="14" t="s">
+        <v>1354</v>
+      </c>
+      <c r="AE38" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AF38" t="s">
+        <v>1335</v>
+      </c>
+      <c r="AG38" t="s">
+        <v>1331</v>
+      </c>
+      <c r="AH38" s="14" t="s">
+        <v>1355</v>
+      </c>
+      <c r="AI38" t="s">
+        <v>1333</v>
+      </c>
+      <c r="AJ38">
+        <v>45</v>
+      </c>
+      <c r="AK38">
+        <v>150</v>
+      </c>
+      <c r="AL38">
+        <v>32</v>
+      </c>
+      <c r="AM38">
+        <v>15</v>
+      </c>
+      <c r="AN38" t="s">
+        <v>143</v>
+      </c>
+      <c r="AO38" t="s">
+        <v>144</v>
+      </c>
+      <c r="AP38" t="s">
+        <v>145</v>
+      </c>
+      <c r="AQ38" t="s">
+        <v>146</v>
+      </c>
+      <c r="AU38" t="s">
+        <v>1356</v>
+      </c>
+      <c r="BB38" t="s">
+        <v>1383</v>
+      </c>
+      <c r="BC38" t="s">
+        <v>1384</v>
+      </c>
+      <c r="BD38" t="s">
+        <v>1385</v>
+      </c>
+      <c r="BE38" t="s">
+        <v>1386</v>
+      </c>
+      <c r="BF38" t="s">
+        <v>1387</v>
+      </c>
+      <c r="BG38" t="s">
+        <v>1388</v>
+      </c>
+      <c r="BH38" t="s">
+        <v>1389</v>
+      </c>
+      <c r="BI38" t="s">
+        <v>1390</v>
+      </c>
+      <c r="BJ38" t="s">
+        <v>1391</v>
+      </c>
+      <c r="BK38" t="s">
+        <v>1392</v>
+      </c>
+      <c r="BL38" t="s">
+        <v>1393</v>
+      </c>
+      <c r="BM38" t="s">
+        <v>1394</v>
+      </c>
+      <c r="BN38" t="s">
+        <v>1395</v>
+      </c>
+      <c r="BO38" t="s">
+        <v>1396</v>
+      </c>
+      <c r="BP38" t="s">
+        <v>1397</v>
+      </c>
+      <c r="BQ38" t="s">
+        <v>1398</v>
+      </c>
+      <c r="BR38" t="s">
+        <v>1399</v>
+      </c>
+      <c r="BS38" t="s">
+        <v>1400</v>
+      </c>
+      <c r="BT38" t="s">
+        <v>1401</v>
+      </c>
+      <c r="BU38" t="s">
+        <v>1402</v>
+      </c>
+      <c r="BV38" t="s">
+        <v>1403</v>
+      </c>
+      <c r="BW38" t="s">
+        <v>1404</v>
+      </c>
+      <c r="BX38" t="s">
+        <v>1405</v>
+      </c>
+      <c r="BY38" t="s">
+        <v>1406</v>
+      </c>
+      <c r="BZ38" t="s">
+        <v>1401</v>
+      </c>
+      <c r="CA38" t="s">
+        <v>1402</v>
+      </c>
+      <c r="CB38" t="s">
+        <v>1403</v>
+      </c>
+      <c r="CC38" t="s">
+        <v>1404</v>
+      </c>
+      <c r="CD38" t="s">
+        <v>1405</v>
+      </c>
+      <c r="CE38" t="s">
+        <v>1406</v>
+      </c>
+    </row>
+    <row r="39" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>1407</v>
+      </c>
+      <c r="B39" t="s">
+        <v>1270</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>1342</v>
+      </c>
+      <c r="D39" t="s">
+        <v>220</v>
+      </c>
+      <c r="E39" t="s">
+        <v>221</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>1408</v>
+      </c>
+      <c r="G39" t="s">
+        <v>126</v>
+      </c>
+      <c r="H39" t="s">
+        <v>1407</v>
+      </c>
+      <c r="I39" t="s">
+        <v>1407</v>
+      </c>
+      <c r="J39" t="s">
+        <v>1407</v>
+      </c>
+      <c r="K39" t="s">
+        <v>1407</v>
+      </c>
+      <c r="L39" t="s">
+        <v>1303</v>
+      </c>
+      <c r="M39" t="s">
+        <v>1345</v>
+      </c>
+      <c r="N39" s="14" t="s">
+        <v>1346</v>
+      </c>
+      <c r="O39" t="s">
+        <v>1276</v>
+      </c>
+      <c r="P39" t="s">
+        <v>1304</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>1347</v>
+      </c>
+      <c r="R39" s="14" t="s">
+        <v>1348</v>
+      </c>
+      <c r="T39" t="s">
+        <v>1305</v>
+      </c>
+      <c r="U39" t="s">
+        <v>1349</v>
+      </c>
+      <c r="V39" s="14" t="s">
+        <v>1350</v>
+      </c>
+      <c r="X39" t="s">
+        <v>1306</v>
+      </c>
+      <c r="Y39" t="s">
+        <v>1351</v>
+      </c>
+      <c r="Z39" s="14" t="s">
+        <v>1352</v>
+      </c>
+      <c r="AB39" t="s">
+        <v>1336</v>
+      </c>
+      <c r="AC39" t="s">
+        <v>1353</v>
+      </c>
+      <c r="AD39" s="14" t="s">
+        <v>1354</v>
+      </c>
+      <c r="AE39" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AF39" t="s">
+        <v>1337</v>
+      </c>
+      <c r="AG39" t="s">
+        <v>1331</v>
+      </c>
+      <c r="AH39" s="14" t="s">
+        <v>1355</v>
+      </c>
+      <c r="AI39" t="s">
+        <v>1333</v>
+      </c>
+      <c r="AJ39">
+        <v>45</v>
+      </c>
+      <c r="AK39">
+        <v>150</v>
+      </c>
+      <c r="AL39">
+        <v>32</v>
+      </c>
+      <c r="AM39">
+        <v>15</v>
+      </c>
+      <c r="AN39" t="s">
+        <v>143</v>
+      </c>
+      <c r="AO39" t="s">
+        <v>144</v>
+      </c>
+      <c r="AP39" t="s">
+        <v>145</v>
+      </c>
+      <c r="AQ39" t="s">
+        <v>146</v>
+      </c>
+      <c r="AU39" t="s">
+        <v>1356</v>
+      </c>
+      <c r="BB39" t="s">
+        <v>1409</v>
+      </c>
+      <c r="BC39" t="s">
+        <v>1410</v>
+      </c>
+      <c r="BD39" t="s">
+        <v>1411</v>
+      </c>
+      <c r="BE39" t="s">
+        <v>1412</v>
+      </c>
+      <c r="BF39" t="s">
+        <v>1413</v>
+      </c>
+      <c r="BG39" t="s">
+        <v>1414</v>
+      </c>
+      <c r="BH39" t="s">
+        <v>1415</v>
+      </c>
+      <c r="BI39" t="s">
+        <v>1416</v>
+      </c>
+      <c r="BJ39" t="s">
+        <v>1417</v>
+      </c>
+      <c r="BK39" t="s">
+        <v>1418</v>
+      </c>
+      <c r="BL39" t="s">
+        <v>1419</v>
+      </c>
+      <c r="BM39" t="s">
+        <v>1420</v>
+      </c>
+      <c r="BN39" t="s">
+        <v>1421</v>
+      </c>
+      <c r="BO39" t="s">
+        <v>1422</v>
+      </c>
+      <c r="BP39" t="s">
+        <v>1423</v>
+      </c>
+      <c r="BQ39" t="s">
+        <v>1424</v>
+      </c>
+      <c r="BR39" t="s">
+        <v>1425</v>
+      </c>
+      <c r="BS39" t="s">
+        <v>1426</v>
+      </c>
+      <c r="BT39" t="s">
+        <v>1427</v>
+      </c>
+      <c r="BU39" t="s">
+        <v>1428</v>
+      </c>
+      <c r="BV39" t="s">
+        <v>1429</v>
+      </c>
+      <c r="BW39" t="s">
+        <v>1430</v>
+      </c>
+      <c r="BX39" t="s">
+        <v>1431</v>
+      </c>
+      <c r="BY39" t="s">
+        <v>1432</v>
+      </c>
+      <c r="BZ39" t="s">
+        <v>1427</v>
+      </c>
+      <c r="CA39" t="s">
+        <v>1428</v>
+      </c>
+      <c r="CB39" t="s">
+        <v>1429</v>
+      </c>
+      <c r="CC39" t="s">
+        <v>1430</v>
+      </c>
+      <c r="CD39" t="s">
+        <v>1431</v>
+      </c>
+      <c r="CE39" t="s">
+        <v>1432</v>
+      </c>
+    </row>
+    <row r="40" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>1433</v>
+      </c>
+      <c r="B40" t="s">
+        <v>1270</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>1342</v>
+      </c>
+      <c r="D40" t="s">
+        <v>258</v>
+      </c>
+      <c r="E40" t="s">
+        <v>259</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>1434</v>
+      </c>
+      <c r="G40" t="s">
+        <v>126</v>
+      </c>
+      <c r="H40" t="s">
+        <v>1435</v>
+      </c>
+      <c r="I40" t="s">
+        <v>1435</v>
+      </c>
+      <c r="J40" t="s">
+        <v>1435</v>
+      </c>
+      <c r="K40" t="s">
+        <v>1435</v>
+      </c>
+      <c r="L40" t="s">
+        <v>1316</v>
+      </c>
+      <c r="M40" t="s">
+        <v>1345</v>
+      </c>
+      <c r="N40" s="14" t="s">
+        <v>1346</v>
+      </c>
+      <c r="O40" t="s">
+        <v>1276</v>
+      </c>
+      <c r="P40" t="s">
+        <v>1317</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>1347</v>
+      </c>
+      <c r="R40" s="14" t="s">
+        <v>1348</v>
+      </c>
+      <c r="T40" t="s">
+        <v>1318</v>
+      </c>
+      <c r="U40" t="s">
+        <v>1349</v>
+      </c>
+      <c r="V40" s="14" t="s">
+        <v>1350</v>
+      </c>
+      <c r="X40" t="s">
+        <v>1319</v>
+      </c>
+      <c r="Y40" t="s">
+        <v>1351</v>
+      </c>
+      <c r="Z40" s="14" t="s">
+        <v>1352</v>
+      </c>
+      <c r="AB40" t="s">
+        <v>1338</v>
+      </c>
+      <c r="AC40" t="s">
+        <v>1353</v>
+      </c>
+      <c r="AD40" s="14" t="s">
+        <v>1354</v>
+      </c>
+      <c r="AE40" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AF40" t="s">
+        <v>1339</v>
+      </c>
+      <c r="AG40" t="s">
+        <v>1331</v>
+      </c>
+      <c r="AH40" s="14" t="s">
+        <v>1355</v>
+      </c>
+      <c r="AI40" t="s">
+        <v>1333</v>
+      </c>
+      <c r="AJ40">
+        <v>45</v>
+      </c>
+      <c r="AK40">
+        <v>150</v>
+      </c>
+      <c r="AL40">
+        <v>32</v>
+      </c>
+      <c r="AM40">
+        <v>15</v>
+      </c>
+      <c r="AN40" t="s">
+        <v>143</v>
+      </c>
+      <c r="AO40" t="s">
+        <v>144</v>
+      </c>
+      <c r="AP40" t="s">
+        <v>145</v>
+      </c>
+      <c r="AQ40" t="s">
+        <v>146</v>
+      </c>
+      <c r="AU40" t="s">
+        <v>1356</v>
+      </c>
+      <c r="BB40" t="s">
+        <v>1436</v>
+      </c>
+      <c r="BC40" t="s">
+        <v>1437</v>
+      </c>
+      <c r="BD40" t="s">
+        <v>1438</v>
+      </c>
+      <c r="BE40" t="s">
+        <v>1439</v>
+      </c>
+      <c r="BF40" t="s">
+        <v>1440</v>
+      </c>
+      <c r="BG40" t="s">
+        <v>1441</v>
+      </c>
+      <c r="BH40" t="s">
+        <v>1442</v>
+      </c>
+      <c r="BI40" t="s">
+        <v>1443</v>
+      </c>
+      <c r="BJ40" t="s">
+        <v>1444</v>
+      </c>
+      <c r="BK40" t="s">
+        <v>1445</v>
+      </c>
+      <c r="BL40" t="s">
+        <v>1446</v>
+      </c>
+      <c r="BM40" t="s">
+        <v>1447</v>
+      </c>
+      <c r="BN40" t="s">
+        <v>1448</v>
+      </c>
+      <c r="BO40" t="s">
+        <v>1449</v>
+      </c>
+      <c r="BP40" t="s">
+        <v>1450</v>
+      </c>
+      <c r="BQ40" t="s">
+        <v>1451</v>
+      </c>
+      <c r="BR40" t="s">
+        <v>1452</v>
+      </c>
+      <c r="BS40" t="s">
+        <v>1453</v>
+      </c>
+      <c r="BT40" t="s">
+        <v>1454</v>
+      </c>
+      <c r="BU40" t="s">
+        <v>1455</v>
+      </c>
+      <c r="BV40" t="s">
+        <v>1456</v>
+      </c>
+      <c r="BW40" t="s">
+        <v>1457</v>
+      </c>
+      <c r="BX40" t="s">
+        <v>1458</v>
+      </c>
+      <c r="BY40" t="s">
+        <v>1459</v>
+      </c>
+      <c r="BZ40" t="s">
+        <v>1454</v>
+      </c>
+      <c r="CA40" t="s">
+        <v>1455</v>
+      </c>
+      <c r="CB40" t="s">
+        <v>1456</v>
+      </c>
+      <c r="CC40" t="s">
+        <v>1457</v>
+      </c>
+      <c r="CD40" t="s">
+        <v>1458</v>
+      </c>
+      <c r="CE40" t="s">
+        <v>1459</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="CF1:CK1"/>

</xml_diff>

<commit_message>
﻿Bancos B.MET.090 y B.MET.150 en Leroy y Makro
- Leroy Merlin · Bancos: portal nuevo con la plantilla de bancos exportada de
  Leroy (categoria Banco de interior); el catalogo de taquillas ya no los incluye.
- Motor: filtro por tipo de producto (soloTipos/excluirTipos) y traduccion de
  valores en el Mapa (color, plazas).
- Maestro: ofertas de Leroy de los 8 bancos en la hoja Ofertas.
- Makro: los 8 bancos en las plantillas de oferta de los 6 paises; las plantillas
  guardadas en el navegador reciben las filas nuevas sin perder las suyas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/datos/FICHERO_MAESTRO2.xlsx
+++ b/public/datos/FICHERO_MAESTRO2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Helian\Desktop\Fichero Maestro\Sistema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAEA62F0-F392-43B2-B041-015034B42A7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FFA02DC-3675-4C08-9D09-1F6F328B2CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="591" xr2:uid="{90124268-D67C-4387-8829-7E3B806257E6}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3469" uniqueCount="1460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3517" uniqueCount="1460">
   <si>
     <t>Marketplace</t>
   </si>
@@ -5035,7 +5035,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2896C02-6550-4E5B-A893-D4B82D18FB32}">
-  <dimension ref="A1:J201"/>
+  <dimension ref="A1:J209"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -10180,7 +10180,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>52</v>
       </c>
@@ -10206,7 +10206,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>52</v>
       </c>
@@ -10232,7 +10232,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>52</v>
       </c>
@@ -10258,7 +10258,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>52</v>
       </c>
@@ -10284,7 +10284,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>52</v>
       </c>
@@ -10310,7 +10310,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>52</v>
       </c>
@@ -10336,7 +10336,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>52</v>
       </c>
@@ -10362,7 +10362,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>52</v>
       </c>
@@ -10388,7 +10388,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>52</v>
       </c>
@@ -10412,6 +10412,238 @@
       </c>
       <c r="H201" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="202" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A202" t="s">
+        <v>10</v>
+      </c>
+      <c r="B202" t="s">
+        <v>11</v>
+      </c>
+      <c r="C202" s="1" t="s">
+        <v>1272</v>
+      </c>
+      <c r="D202" t="s">
+        <v>1269</v>
+      </c>
+      <c r="E202">
+        <v>110</v>
+      </c>
+      <c r="F202">
+        <v>104</v>
+      </c>
+      <c r="G202">
+        <v>2</v>
+      </c>
+      <c r="H202" t="s">
+        <v>13</v>
+      </c>
+      <c r="I202" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="203" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A203" t="s">
+        <v>10</v>
+      </c>
+      <c r="B203" t="s">
+        <v>11</v>
+      </c>
+      <c r="C203" s="1" t="s">
+        <v>1290</v>
+      </c>
+      <c r="D203" t="s">
+        <v>1289</v>
+      </c>
+      <c r="E203">
+        <v>110</v>
+      </c>
+      <c r="F203">
+        <v>75</v>
+      </c>
+      <c r="G203">
+        <v>2</v>
+      </c>
+      <c r="H203" t="s">
+        <v>13</v>
+      </c>
+      <c r="I203" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="204" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A204" t="s">
+        <v>10</v>
+      </c>
+      <c r="B204" t="s">
+        <v>11</v>
+      </c>
+      <c r="C204" s="1" t="s">
+        <v>1302</v>
+      </c>
+      <c r="D204" t="s">
+        <v>1301</v>
+      </c>
+      <c r="E204">
+        <v>110</v>
+      </c>
+      <c r="F204">
+        <v>25</v>
+      </c>
+      <c r="G204">
+        <v>2</v>
+      </c>
+      <c r="H204" t="s">
+        <v>13</v>
+      </c>
+      <c r="I204" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="205" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A205" t="s">
+        <v>10</v>
+      </c>
+      <c r="B205" t="s">
+        <v>11</v>
+      </c>
+      <c r="C205" s="1" t="s">
+        <v>1314</v>
+      </c>
+      <c r="D205" t="s">
+        <v>1313</v>
+      </c>
+      <c r="E205">
+        <v>100</v>
+      </c>
+      <c r="F205">
+        <v>27</v>
+      </c>
+      <c r="G205">
+        <v>2</v>
+      </c>
+      <c r="H205" t="s">
+        <v>13</v>
+      </c>
+      <c r="I205" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="206" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A206" t="s">
+        <v>10</v>
+      </c>
+      <c r="B206" t="s">
+        <v>11</v>
+      </c>
+      <c r="C206" s="1" t="s">
+        <v>1343</v>
+      </c>
+      <c r="D206" t="s">
+        <v>1341</v>
+      </c>
+      <c r="E206">
+        <v>144</v>
+      </c>
+      <c r="F206">
+        <v>0</v>
+      </c>
+      <c r="G206">
+        <v>2</v>
+      </c>
+      <c r="H206" t="s">
+        <v>13</v>
+      </c>
+      <c r="I206" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="207" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A207" t="s">
+        <v>10</v>
+      </c>
+      <c r="B207" t="s">
+        <v>11</v>
+      </c>
+      <c r="C207" s="1" t="s">
+        <v>1382</v>
+      </c>
+      <c r="D207" t="s">
+        <v>1381</v>
+      </c>
+      <c r="E207">
+        <v>144</v>
+      </c>
+      <c r="F207">
+        <v>0</v>
+      </c>
+      <c r="G207">
+        <v>2</v>
+      </c>
+      <c r="H207" t="s">
+        <v>13</v>
+      </c>
+      <c r="I207" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="208" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A208" t="s">
+        <v>10</v>
+      </c>
+      <c r="B208" t="s">
+        <v>11</v>
+      </c>
+      <c r="C208" s="1" t="s">
+        <v>1408</v>
+      </c>
+      <c r="D208" t="s">
+        <v>1407</v>
+      </c>
+      <c r="E208">
+        <v>144</v>
+      </c>
+      <c r="F208">
+        <v>0</v>
+      </c>
+      <c r="G208">
+        <v>2</v>
+      </c>
+      <c r="H208" t="s">
+        <v>13</v>
+      </c>
+      <c r="I208" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="209" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A209" t="s">
+        <v>10</v>
+      </c>
+      <c r="B209" t="s">
+        <v>11</v>
+      </c>
+      <c r="C209" s="1" t="s">
+        <v>1434</v>
+      </c>
+      <c r="D209" t="s">
+        <v>1433</v>
+      </c>
+      <c r="E209">
+        <v>144</v>
+      </c>
+      <c r="F209">
+        <v>0</v>
+      </c>
+      <c r="G209">
+        <v>2</v>
+      </c>
+      <c r="H209" t="s">
+        <v>13</v>
+      </c>
+      <c r="I209" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Leroy: plantilla de ofertas nueva (97 columnas) con precio por pais
- Plantilla offers-es_ES de Leroy del 28/09/2026. La anterior tenia las columnas
  desplazadas: Standard/ES/canales caian en las de contribucion ecologica.
- Precio por canal: 001 Francia, 002 Portugal, 003 Espana, 005 Italia. Descuento =
  precio real, precio = real + 20. IVA Standard, pais de almacenaje ES y canales
  LMES,LMFR,LMIT,LMPT por codigo de columna.
- Maestro: filas LeroyMerlin/FR (20) e IT (10) con los precios del fichero subido
  a Leroy el 18/09; las actualiza el CSV de precios.
- Salvaguarda: precio de pais por debajo de la mitad del de Espana -> canal vacio y aviso.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/datos/FICHERO_MAESTRO2.xlsx
+++ b/public/datos/FICHERO_MAESTRO2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Helian\Desktop\Fichero Maestro\Sistema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FFA02DC-3675-4C08-9D09-1F6F328B2CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2831B141-AF20-4C03-83A9-B3709CB47209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="591" xr2:uid="{90124268-D67C-4387-8829-7E3B806257E6}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3517" uniqueCount="1460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3637" uniqueCount="1460">
   <si>
     <t>Marketplace</t>
   </si>
@@ -5035,7 +5035,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2896C02-6550-4E5B-A893-D4B82D18FB32}">
-  <dimension ref="A1:J209"/>
+  <dimension ref="A1:J239"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -10644,6 +10644,516 @@
       </c>
       <c r="I209" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="210" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A210" t="s">
+        <v>10</v>
+      </c>
+      <c r="B210" t="s">
+        <v>54</v>
+      </c>
+      <c r="C210" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D210" t="s">
+        <v>12</v>
+      </c>
+      <c r="E210">
+        <v>130.99</v>
+      </c>
+    </row>
+    <row r="211" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A211" t="s">
+        <v>10</v>
+      </c>
+      <c r="B211" t="s">
+        <v>54</v>
+      </c>
+      <c r="C211" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="D211" t="s">
+        <v>15</v>
+      </c>
+      <c r="E211">
+        <v>130.99</v>
+      </c>
+    </row>
+    <row r="212" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A212" t="s">
+        <v>10</v>
+      </c>
+      <c r="B212" t="s">
+        <v>54</v>
+      </c>
+      <c r="C212" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="D212" t="s">
+        <v>16</v>
+      </c>
+      <c r="E212">
+        <v>130.99</v>
+      </c>
+    </row>
+    <row r="213" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A213" t="s">
+        <v>10</v>
+      </c>
+      <c r="B213" t="s">
+        <v>54</v>
+      </c>
+      <c r="C213" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="D213" t="s">
+        <v>18</v>
+      </c>
+      <c r="E213">
+        <v>130.99</v>
+      </c>
+    </row>
+    <row r="214" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A214" t="s">
+        <v>10</v>
+      </c>
+      <c r="B214" t="s">
+        <v>54</v>
+      </c>
+      <c r="C214" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="D214" t="s">
+        <v>19</v>
+      </c>
+      <c r="E214">
+        <v>355.99</v>
+      </c>
+    </row>
+    <row r="215" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A215" t="s">
+        <v>10</v>
+      </c>
+      <c r="B215" t="s">
+        <v>54</v>
+      </c>
+      <c r="C215" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="D215" t="s">
+        <v>20</v>
+      </c>
+      <c r="E215">
+        <v>355.99</v>
+      </c>
+    </row>
+    <row r="216" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A216" t="s">
+        <v>10</v>
+      </c>
+      <c r="B216" t="s">
+        <v>54</v>
+      </c>
+      <c r="C216" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="D216" t="s">
+        <v>21</v>
+      </c>
+      <c r="E216">
+        <v>355.99</v>
+      </c>
+    </row>
+    <row r="217" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A217" t="s">
+        <v>10</v>
+      </c>
+      <c r="B217" t="s">
+        <v>54</v>
+      </c>
+      <c r="C217" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="D217" t="s">
+        <v>22</v>
+      </c>
+      <c r="E217">
+        <v>284.79000000000002</v>
+      </c>
+    </row>
+    <row r="218" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A218" t="s">
+        <v>10</v>
+      </c>
+      <c r="B218" t="s">
+        <v>54</v>
+      </c>
+      <c r="C218" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="D218" t="s">
+        <v>23</v>
+      </c>
+      <c r="E218">
+        <v>217.99</v>
+      </c>
+    </row>
+    <row r="219" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A219" t="s">
+        <v>10</v>
+      </c>
+      <c r="B219" t="s">
+        <v>54</v>
+      </c>
+      <c r="C219" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="D219" t="s">
+        <v>25</v>
+      </c>
+      <c r="E219">
+        <v>201.99</v>
+      </c>
+    </row>
+    <row r="220" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A220" t="s">
+        <v>10</v>
+      </c>
+      <c r="B220" t="s">
+        <v>54</v>
+      </c>
+      <c r="C220" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="D220" t="s">
+        <v>26</v>
+      </c>
+      <c r="E220">
+        <v>201.99</v>
+      </c>
+    </row>
+    <row r="221" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A221" t="s">
+        <v>10</v>
+      </c>
+      <c r="B221" t="s">
+        <v>54</v>
+      </c>
+      <c r="C221" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="D221" t="s">
+        <v>28</v>
+      </c>
+      <c r="E221">
+        <v>201.99</v>
+      </c>
+    </row>
+    <row r="222" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A222" t="s">
+        <v>10</v>
+      </c>
+      <c r="B222" t="s">
+        <v>54</v>
+      </c>
+      <c r="C222" s="1" t="s">
+        <v>622</v>
+      </c>
+      <c r="D222" t="s">
+        <v>29</v>
+      </c>
+      <c r="E222">
+        <v>230.99</v>
+      </c>
+    </row>
+    <row r="223" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A223" t="s">
+        <v>10</v>
+      </c>
+      <c r="B223" t="s">
+        <v>54</v>
+      </c>
+      <c r="C223" s="1" t="s">
+        <v>668</v>
+      </c>
+      <c r="D223" t="s">
+        <v>30</v>
+      </c>
+      <c r="E223">
+        <v>214.99</v>
+      </c>
+    </row>
+    <row r="224" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A224" t="s">
+        <v>10</v>
+      </c>
+      <c r="B224" t="s">
+        <v>54</v>
+      </c>
+      <c r="C224" s="1" t="s">
+        <v>709</v>
+      </c>
+      <c r="D224" t="s">
+        <v>31</v>
+      </c>
+      <c r="E224">
+        <v>222.99</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A225" t="s">
+        <v>10</v>
+      </c>
+      <c r="B225" t="s">
+        <v>54</v>
+      </c>
+      <c r="C225" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="D225" t="s">
+        <v>32</v>
+      </c>
+      <c r="E225">
+        <v>222.99</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A226" t="s">
+        <v>10</v>
+      </c>
+      <c r="B226" t="s">
+        <v>54</v>
+      </c>
+      <c r="C226" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="D226" t="s">
+        <v>33</v>
+      </c>
+      <c r="E226">
+        <v>324.99</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A227" t="s">
+        <v>10</v>
+      </c>
+      <c r="B227" t="s">
+        <v>54</v>
+      </c>
+      <c r="C227" s="1" t="s">
+        <v>837</v>
+      </c>
+      <c r="D227" t="s">
+        <v>35</v>
+      </c>
+      <c r="E227">
+        <v>312.98</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A228" t="s">
+        <v>10</v>
+      </c>
+      <c r="B228" t="s">
+        <v>54</v>
+      </c>
+      <c r="C228" s="1" t="s">
+        <v>878</v>
+      </c>
+      <c r="D228" t="s">
+        <v>36</v>
+      </c>
+      <c r="E228">
+        <v>312.99</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A229" t="s">
+        <v>10</v>
+      </c>
+      <c r="B229" t="s">
+        <v>54</v>
+      </c>
+      <c r="C229" s="1" t="s">
+        <v>917</v>
+      </c>
+      <c r="D229" t="s">
+        <v>38</v>
+      </c>
+      <c r="E229">
+        <v>300.99</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A230" t="s">
+        <v>10</v>
+      </c>
+      <c r="B230" t="s">
+        <v>49</v>
+      </c>
+      <c r="C230" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D230" t="s">
+        <v>12</v>
+      </c>
+      <c r="E230">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A231" t="s">
+        <v>10</v>
+      </c>
+      <c r="B231" t="s">
+        <v>49</v>
+      </c>
+      <c r="C231" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="D231" t="s">
+        <v>15</v>
+      </c>
+      <c r="E231">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A232" t="s">
+        <v>10</v>
+      </c>
+      <c r="B232" t="s">
+        <v>49</v>
+      </c>
+      <c r="C232" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="D232" t="s">
+        <v>19</v>
+      </c>
+      <c r="E232">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A233" t="s">
+        <v>10</v>
+      </c>
+      <c r="B233" t="s">
+        <v>49</v>
+      </c>
+      <c r="C233" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="D233" t="s">
+        <v>20</v>
+      </c>
+      <c r="E233">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A234" t="s">
+        <v>10</v>
+      </c>
+      <c r="B234" t="s">
+        <v>49</v>
+      </c>
+      <c r="C234" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="D234" t="s">
+        <v>23</v>
+      </c>
+      <c r="E234">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A235" t="s">
+        <v>10</v>
+      </c>
+      <c r="B235" t="s">
+        <v>49</v>
+      </c>
+      <c r="C235" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="D235" t="s">
+        <v>25</v>
+      </c>
+      <c r="E235">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A236" t="s">
+        <v>10</v>
+      </c>
+      <c r="B236" t="s">
+        <v>49</v>
+      </c>
+      <c r="C236" s="1" t="s">
+        <v>622</v>
+      </c>
+      <c r="D236" t="s">
+        <v>29</v>
+      </c>
+      <c r="E236">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A237" t="s">
+        <v>10</v>
+      </c>
+      <c r="B237" t="s">
+        <v>49</v>
+      </c>
+      <c r="C237" s="1" t="s">
+        <v>668</v>
+      </c>
+      <c r="D237" t="s">
+        <v>30</v>
+      </c>
+      <c r="E237">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A238" t="s">
+        <v>10</v>
+      </c>
+      <c r="B238" t="s">
+        <v>49</v>
+      </c>
+      <c r="C238" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="D238" t="s">
+        <v>33</v>
+      </c>
+      <c r="E238">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A239" t="s">
+        <v>10</v>
+      </c>
+      <c r="B239" t="s">
+        <v>49</v>
+      </c>
+      <c r="C239" s="1" t="s">
+        <v>837</v>
+      </c>
+      <c r="D239" t="s">
+        <v>35</v>
+      </c>
+      <c r="E239">
+        <v>309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Leroy: ofertas de las taquillas efecto madera y antracita
- Maestro: 10 filas LeroyMerlin/ALL (_M y _A) con precio, stock, clase logistica
  y plazo del fichero de ofertas subido a Leroy el 18/09.
- CSV de precios y stock: reconoce Madera (_M) y Antracita (_A); antes Madera
  se ignoraba.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/datos/FICHERO_MAESTRO2.xlsx
+++ b/public/datos/FICHERO_MAESTRO2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Helian\Desktop\Fichero Maestro\Sistema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2831B141-AF20-4C03-83A9-B3709CB47209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2588990C-AFC4-4378-9BC9-BFFC5C24AC2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="591" xr2:uid="{90124268-D67C-4387-8829-7E3B806257E6}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3637" uniqueCount="1460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3697" uniqueCount="1460">
   <si>
     <t>Marketplace</t>
   </si>
@@ -5035,7 +5035,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2896C02-6550-4E5B-A893-D4B82D18FB32}">
-  <dimension ref="A1:J239"/>
+  <dimension ref="A1:J249"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -10901,7 +10901,7 @@
         <v>222.99</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>10</v>
       </c>
@@ -10918,7 +10918,7 @@
         <v>222.99</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>10</v>
       </c>
@@ -10935,7 +10935,7 @@
         <v>324.99</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>10</v>
       </c>
@@ -10952,7 +10952,7 @@
         <v>312.98</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>10</v>
       </c>
@@ -10969,7 +10969,7 @@
         <v>312.99</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>10</v>
       </c>
@@ -10986,7 +10986,7 @@
         <v>300.99</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>10</v>
       </c>
@@ -11003,7 +11003,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>10</v>
       </c>
@@ -11020,7 +11020,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>10</v>
       </c>
@@ -11037,7 +11037,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>10</v>
       </c>
@@ -11054,7 +11054,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>10</v>
       </c>
@@ -11071,7 +11071,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>10</v>
       </c>
@@ -11088,7 +11088,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>10</v>
       </c>
@@ -11105,7 +11105,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>10</v>
       </c>
@@ -11122,7 +11122,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>10</v>
       </c>
@@ -11139,7 +11139,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>10</v>
       </c>
@@ -11154,6 +11154,296 @@
       </c>
       <c r="E239">
         <v>309</v>
+      </c>
+    </row>
+    <row r="240" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A240" t="s">
+        <v>10</v>
+      </c>
+      <c r="B240" t="s">
+        <v>11</v>
+      </c>
+      <c r="C240" s="1" t="s">
+        <v>959</v>
+      </c>
+      <c r="D240" t="s">
+        <v>956</v>
+      </c>
+      <c r="E240">
+        <v>120</v>
+      </c>
+      <c r="F240">
+        <v>0</v>
+      </c>
+      <c r="G240">
+        <v>2</v>
+      </c>
+      <c r="H240" t="s">
+        <v>13</v>
+      </c>
+      <c r="I240" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="241" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A241" t="s">
+        <v>10</v>
+      </c>
+      <c r="B241" t="s">
+        <v>11</v>
+      </c>
+      <c r="C241" s="1" t="s">
+        <v>992</v>
+      </c>
+      <c r="D241" t="s">
+        <v>989</v>
+      </c>
+      <c r="E241">
+        <v>119</v>
+      </c>
+      <c r="F241">
+        <v>0</v>
+      </c>
+      <c r="G241">
+        <v>2</v>
+      </c>
+      <c r="H241" t="s">
+        <v>13</v>
+      </c>
+      <c r="I241" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="242" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A242" t="s">
+        <v>10</v>
+      </c>
+      <c r="B242" t="s">
+        <v>11</v>
+      </c>
+      <c r="C242" s="1" t="s">
+        <v>1023</v>
+      </c>
+      <c r="D242" t="s">
+        <v>1022</v>
+      </c>
+      <c r="E242">
+        <v>300</v>
+      </c>
+      <c r="F242">
+        <v>0</v>
+      </c>
+      <c r="G242">
+        <v>2</v>
+      </c>
+      <c r="H242" t="s">
+        <v>13</v>
+      </c>
+      <c r="I242" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="243" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A243" t="s">
+        <v>10</v>
+      </c>
+      <c r="B243" t="s">
+        <v>11</v>
+      </c>
+      <c r="C243" s="1" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D243" t="s">
+        <v>1053</v>
+      </c>
+      <c r="E243">
+        <v>300</v>
+      </c>
+      <c r="F243">
+        <v>0</v>
+      </c>
+      <c r="G243">
+        <v>2</v>
+      </c>
+      <c r="H243" t="s">
+        <v>13</v>
+      </c>
+      <c r="I243" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="244" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A244" t="s">
+        <v>10</v>
+      </c>
+      <c r="B244" t="s">
+        <v>11</v>
+      </c>
+      <c r="C244" s="1" t="s">
+        <v>1085</v>
+      </c>
+      <c r="D244" t="s">
+        <v>1084</v>
+      </c>
+      <c r="E244">
+        <v>179</v>
+      </c>
+      <c r="F244">
+        <v>0</v>
+      </c>
+      <c r="G244">
+        <v>2</v>
+      </c>
+      <c r="H244" t="s">
+        <v>13</v>
+      </c>
+      <c r="I244" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="245" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A245" t="s">
+        <v>10</v>
+      </c>
+      <c r="B245" t="s">
+        <v>11</v>
+      </c>
+      <c r="C245" s="1" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D245" t="s">
+        <v>1115</v>
+      </c>
+      <c r="E245">
+        <v>179</v>
+      </c>
+      <c r="F245">
+        <v>0</v>
+      </c>
+      <c r="G245">
+        <v>2</v>
+      </c>
+      <c r="H245" t="s">
+        <v>13</v>
+      </c>
+      <c r="I245" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="246" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A246" t="s">
+        <v>10</v>
+      </c>
+      <c r="B246" t="s">
+        <v>11</v>
+      </c>
+      <c r="C246" s="1" t="s">
+        <v>1147</v>
+      </c>
+      <c r="D246" t="s">
+        <v>1146</v>
+      </c>
+      <c r="E246">
+        <v>199</v>
+      </c>
+      <c r="F246">
+        <v>0</v>
+      </c>
+      <c r="G246">
+        <v>2</v>
+      </c>
+      <c r="H246" t="s">
+        <v>13</v>
+      </c>
+      <c r="I246" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="247" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A247" t="s">
+        <v>10</v>
+      </c>
+      <c r="B247" t="s">
+        <v>11</v>
+      </c>
+      <c r="C247" s="1" t="s">
+        <v>1178</v>
+      </c>
+      <c r="D247" t="s">
+        <v>1177</v>
+      </c>
+      <c r="E247">
+        <v>200</v>
+      </c>
+      <c r="F247">
+        <v>0</v>
+      </c>
+      <c r="G247">
+        <v>2</v>
+      </c>
+      <c r="H247" t="s">
+        <v>13</v>
+      </c>
+      <c r="I247" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="248" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A248" t="s">
+        <v>10</v>
+      </c>
+      <c r="B248" t="s">
+        <v>11</v>
+      </c>
+      <c r="C248" s="1" t="s">
+        <v>1209</v>
+      </c>
+      <c r="D248" t="s">
+        <v>1208</v>
+      </c>
+      <c r="E248">
+        <v>279</v>
+      </c>
+      <c r="F248">
+        <v>0</v>
+      </c>
+      <c r="G248">
+        <v>2</v>
+      </c>
+      <c r="H248" t="s">
+        <v>13</v>
+      </c>
+      <c r="I248" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="249" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A249" t="s">
+        <v>10</v>
+      </c>
+      <c r="B249" t="s">
+        <v>11</v>
+      </c>
+      <c r="C249" s="1" t="s">
+        <v>1240</v>
+      </c>
+      <c r="D249" t="s">
+        <v>1239</v>
+      </c>
+      <c r="E249">
+        <v>279</v>
+      </c>
+      <c r="F249">
+        <v>0</v>
+      </c>
+      <c r="G249">
+        <v>2</v>
+      </c>
+      <c r="H249" t="s">
+        <v>13</v>
+      </c>
+      <c r="I249" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Maestro: fotos de los bancos de 150 = main, 7, 4, 3 y 5 de cada idioma
Bloques Espana/Italia/Francia en su idioma y Alemania/Reino Unido en ingles;
la Image 6 queda vacia.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/datos/FICHERO_MAESTRO2.xlsx
+++ b/public/datos/FICHERO_MAESTRO2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Helian\Desktop\Fichero Maestro\Sistema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2588990C-AFC4-4378-9BC9-BFFC5C24AC2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79AFF6EE-D4ED-4ECC-A339-C71839C403D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="591" xr2:uid="{90124268-D67C-4387-8829-7E3B806257E6}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3697" uniqueCount="1460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3677" uniqueCount="1444">
   <si>
     <t>Marketplace</t>
   </si>
@@ -4226,12 +4226,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195056/bancos/B.MET.150/gris/es/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195061/bancos/B.MET.150/gris/es/pt01.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195066/bancos/B.MET.150/gris/es/pt02.png</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195073/bancos/B.MET.150/gris/es/pt03.png</t>
   </si>
   <si>
@@ -4244,12 +4238,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195143/bancos/B.MET.150/gris/it/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195148/bancos/B.MET.150/gris/it/pt01.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195155/bancos/B.MET.150/gris/it/pt02.png</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195164/bancos/B.MET.150/gris/it/pt03.png</t>
   </si>
   <si>
@@ -4262,12 +4250,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195103/bancos/B.MET.150/gris/fr/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195108/bancos/B.MET.150/gris/fr/pt01.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195114/bancos/B.MET.150/gris/fr/pt02.png</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195118/bancos/B.MET.150/gris/fr/pt03.png</t>
   </si>
   <si>
@@ -4280,12 +4262,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195006/bancos/B.MET.150/gris/en/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195011/bancos/B.MET.150/gris/en/pt01.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195017/bancos/B.MET.150/gris/en/pt02.png</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195023/bancos/B.MET.150/gris/en/pt03.png</t>
   </si>
   <si>
@@ -4304,12 +4280,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195250/bancos/B.MET.150/negro/es/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195252/bancos/B.MET.150/negro/es/pt01.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195254/bancos/B.MET.150/negro/es/pt02.jpg</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195256/bancos/B.MET.150/negro/es/pt03.jpg</t>
   </si>
   <si>
@@ -4322,12 +4292,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195309/bancos/B.MET.150/negro/it/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195314/bancos/B.MET.150/negro/it/pt01.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195320/bancos/B.MET.150/negro/it/pt02.png</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195326/bancos/B.MET.150/negro/it/pt03.png</t>
   </si>
   <si>
@@ -4340,12 +4304,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195267/bancos/B.MET.150/negro/fr/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195272/bancos/B.MET.150/negro/fr/pt01.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195277/bancos/B.MET.150/negro/fr/pt02.png</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195281/bancos/B.MET.150/negro/fr/pt03.png</t>
   </si>
   <si>
@@ -4358,12 +4316,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195198/bancos/B.MET.150/negro/en/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195204/bancos/B.MET.150/negro/en/pt01.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195209/bancos/B.MET.150/negro/en/pt02.png</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195215/bancos/B.MET.150/negro/en/pt03.png</t>
   </si>
   <si>
@@ -4382,12 +4334,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194731/bancos/B.MET.150/blanco/es/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194736/bancos/B.MET.150/blanco/es/pt01.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194741/bancos/B.MET.150/blanco/es/pt02.png</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194747/bancos/B.MET.150/blanco/es/pt03.png</t>
   </si>
   <si>
@@ -4400,12 +4346,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194794/bancos/B.MET.150/blanco/it/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194799/bancos/B.MET.150/blanco/it/pt01.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194809/bancos/B.MET.150/blanco/it/pt02.png</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194812/bancos/B.MET.150/blanco/it/pt03.png</t>
   </si>
   <si>
@@ -4418,12 +4358,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194777/bancos/B.MET.150/blanco/fr/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194779/bancos/B.MET.150/blanco/fr/pt01.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194780/bancos/B.MET.150/blanco/fr/pt02.jpg</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194782/bancos/B.MET.150/blanco/fr/pt03.jpg</t>
   </si>
   <si>
@@ -4436,12 +4370,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194688/bancos/B.MET.150/blanco/en/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194693/bancos/B.MET.150/blanco/en/pt01.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194698/bancos/B.MET.150/blanco/en/pt02.png</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194704/bancos/B.MET.150/blanco/en/pt03.png</t>
   </si>
   <si>
@@ -4463,12 +4391,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194896/bancos/B.MET.150/byn/es/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194901/bancos/B.MET.150/byn/es/pt01.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194908/bancos/B.MET.150/byn/es/pt02.png</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194913/bancos/B.MET.150/byn/es/pt03.png</t>
   </si>
   <si>
@@ -4481,12 +4403,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194963/bancos/B.MET.150/byn/it/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194967/bancos/B.MET.150/byn/it/pt01.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194971/bancos/B.MET.150/byn/it/pt02.png</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194976/bancos/B.MET.150/byn/it/pt03.png</t>
   </si>
   <si>
@@ -4499,12 +4415,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194942/bancos/B.MET.150/byn/fr/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194944/bancos/B.MET.150/byn/fr/pt01.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194947/bancos/B.MET.150/byn/fr/pt02.jpg</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194949/bancos/B.MET.150/byn/fr/pt03.jpg</t>
   </si>
   <si>
@@ -4517,12 +4427,6 @@
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194850/bancos/B.MET.150/byn/en/main.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194856/bancos/B.MET.150/byn/en/pt01.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194861/bancos/B.MET.150/byn/en/pt02.png</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194866/bancos/B.MET.150/byn/en/pt03.png</t>
   </si>
   <si>
@@ -4530,6 +4434,54 @@
   </si>
   <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194877/bancos/B.MET.150/byn/en/pt05.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195095/bancos/B.MET.150/gris/es/pt07.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195190/bancos/B.MET.150/gris/it/pt07.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195135/bancos/B.MET.150/gris/fr/pt07.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195047/bancos/B.MET.150/gris/en/pt07.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195263/bancos/B.MET.150/negro/es/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195346/bancos/B.MET.150/negro/it/pt07.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195302/bancos/B.MET.150/negro/fr/pt07.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790195238/bancos/B.MET.150/negro/en/pt07.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194768/bancos/B.MET.150/blanco/es/pt07.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194843/bancos/B.MET.150/blanco/it/pt07.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194790/bancos/B.MET.150/blanco/fr/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194723/bancos/B.MET.150/blanco/en/pt07.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194935/bancos/B.MET.150/byn/es/pt07.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194997/bancos/B.MET.150/byn/it/pt07.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194958/bancos/B.MET.150/byn/fr/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194889/bancos/B.MET.150/byn/en/pt07.png</t>
   </si>
 </sst>
 </file>
@@ -10567,10 +10519,10 @@
         <v>11</v>
       </c>
       <c r="C207" s="1" t="s">
-        <v>1382</v>
+        <v>1374</v>
       </c>
       <c r="D207" t="s">
-        <v>1381</v>
+        <v>1373</v>
       </c>
       <c r="E207">
         <v>144</v>
@@ -10596,10 +10548,10 @@
         <v>11</v>
       </c>
       <c r="C208" s="1" t="s">
-        <v>1408</v>
+        <v>1392</v>
       </c>
       <c r="D208" t="s">
-        <v>1407</v>
+        <v>1391</v>
       </c>
       <c r="E208">
         <v>144</v>
@@ -10625,10 +10577,10 @@
         <v>11</v>
       </c>
       <c r="C209" s="1" t="s">
-        <v>1434</v>
+        <v>1410</v>
       </c>
       <c r="D209" t="s">
-        <v>1433</v>
+        <v>1409</v>
       </c>
       <c r="E209">
         <v>144</v>
@@ -19042,96 +18994,81 @@
         <v>1357</v>
       </c>
       <c r="BC37" t="s">
-        <v>1358</v>
+        <v>1428</v>
       </c>
       <c r="BD37" t="s">
         <v>1359</v>
       </c>
       <c r="BE37" t="s">
+        <v>1358</v>
+      </c>
+      <c r="BF37" t="s">
         <v>1360</v>
       </c>
-      <c r="BF37" t="s">
+      <c r="BH37" t="s">
         <v>1361</v>
       </c>
-      <c r="BG37" t="s">
+      <c r="BI37" t="s">
+        <v>1429</v>
+      </c>
+      <c r="BJ37" t="s">
+        <v>1363</v>
+      </c>
+      <c r="BK37" t="s">
         <v>1362</v>
       </c>
-      <c r="BH37" t="s">
-        <v>1363</v>
-      </c>
-      <c r="BI37" t="s">
+      <c r="BL37" t="s">
         <v>1364</v>
       </c>
-      <c r="BJ37" t="s">
+      <c r="BN37" t="s">
         <v>1365</v>
       </c>
-      <c r="BK37" t="s">
+      <c r="BO37" t="s">
+        <v>1430</v>
+      </c>
+      <c r="BP37" t="s">
+        <v>1367</v>
+      </c>
+      <c r="BQ37" t="s">
         <v>1366</v>
       </c>
-      <c r="BL37" t="s">
-        <v>1367</v>
-      </c>
-      <c r="BM37" t="s">
+      <c r="BR37" t="s">
         <v>1368</v>
       </c>
-      <c r="BN37" t="s">
+      <c r="BT37" t="s">
         <v>1369</v>
       </c>
-      <c r="BO37" t="s">
+      <c r="BU37" t="s">
+        <v>1431</v>
+      </c>
+      <c r="BV37" t="s">
+        <v>1371</v>
+      </c>
+      <c r="BW37" t="s">
         <v>1370</v>
       </c>
-      <c r="BP37" t="s">
+      <c r="BX37" t="s">
+        <v>1372</v>
+      </c>
+      <c r="BZ37" t="s">
+        <v>1369</v>
+      </c>
+      <c r="CA37" t="s">
+        <v>1431</v>
+      </c>
+      <c r="CB37" t="s">
         <v>1371</v>
       </c>
-      <c r="BQ37" t="s">
+      <c r="CC37" t="s">
+        <v>1370</v>
+      </c>
+      <c r="CD37" t="s">
         <v>1372</v>
-      </c>
-      <c r="BR37" t="s">
-        <v>1373</v>
-      </c>
-      <c r="BS37" t="s">
-        <v>1374</v>
-      </c>
-      <c r="BT37" t="s">
-        <v>1375</v>
-      </c>
-      <c r="BU37" t="s">
-        <v>1376</v>
-      </c>
-      <c r="BV37" t="s">
-        <v>1377</v>
-      </c>
-      <c r="BW37" t="s">
-        <v>1378</v>
-      </c>
-      <c r="BX37" t="s">
-        <v>1379</v>
-      </c>
-      <c r="BY37" t="s">
-        <v>1380</v>
-      </c>
-      <c r="BZ37" t="s">
-        <v>1375</v>
-      </c>
-      <c r="CA37" t="s">
-        <v>1376</v>
-      </c>
-      <c r="CB37" t="s">
-        <v>1377</v>
-      </c>
-      <c r="CC37" t="s">
-        <v>1378</v>
-      </c>
-      <c r="CD37" t="s">
-        <v>1379</v>
-      </c>
-      <c r="CE37" t="s">
-        <v>1380</v>
       </c>
     </row>
     <row r="38" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>1381</v>
+        <v>1373</v>
       </c>
       <c r="B38" t="s">
         <v>1270</v>
@@ -19146,22 +19083,22 @@
         <v>182</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>1382</v>
+        <v>1374</v>
       </c>
       <c r="G38" t="s">
         <v>126</v>
       </c>
       <c r="H38" t="s">
-        <v>1381</v>
+        <v>1373</v>
       </c>
       <c r="I38" t="s">
-        <v>1381</v>
+        <v>1373</v>
       </c>
       <c r="J38" t="s">
-        <v>1381</v>
+        <v>1373</v>
       </c>
       <c r="K38" t="s">
-        <v>1381</v>
+        <v>1373</v>
       </c>
       <c r="L38" t="s">
         <v>1291</v>
@@ -19254,99 +19191,84 @@
         <v>1356</v>
       </c>
       <c r="BB38" t="s">
+        <v>1375</v>
+      </c>
+      <c r="BC38" t="s">
+        <v>1432</v>
+      </c>
+      <c r="BD38" t="s">
+        <v>1377</v>
+      </c>
+      <c r="BE38" t="s">
+        <v>1376</v>
+      </c>
+      <c r="BF38" t="s">
+        <v>1378</v>
+      </c>
+      <c r="BH38" t="s">
+        <v>1379</v>
+      </c>
+      <c r="BI38" t="s">
+        <v>1433</v>
+      </c>
+      <c r="BJ38" t="s">
+        <v>1381</v>
+      </c>
+      <c r="BK38" t="s">
+        <v>1380</v>
+      </c>
+      <c r="BL38" t="s">
+        <v>1382</v>
+      </c>
+      <c r="BN38" t="s">
         <v>1383</v>
       </c>
-      <c r="BC38" t="s">
+      <c r="BO38" t="s">
+        <v>1434</v>
+      </c>
+      <c r="BP38" t="s">
+        <v>1385</v>
+      </c>
+      <c r="BQ38" t="s">
         <v>1384</v>
       </c>
-      <c r="BD38" t="s">
-        <v>1385</v>
-      </c>
-      <c r="BE38" t="s">
+      <c r="BR38" t="s">
         <v>1386</v>
       </c>
-      <c r="BF38" t="s">
+      <c r="BT38" t="s">
         <v>1387</v>
       </c>
-      <c r="BG38" t="s">
+      <c r="BU38" t="s">
+        <v>1435</v>
+      </c>
+      <c r="BV38" t="s">
+        <v>1389</v>
+      </c>
+      <c r="BW38" t="s">
         <v>1388</v>
       </c>
-      <c r="BH38" t="s">
+      <c r="BX38" t="s">
+        <v>1390</v>
+      </c>
+      <c r="BZ38" t="s">
+        <v>1387</v>
+      </c>
+      <c r="CA38" t="s">
+        <v>1435</v>
+      </c>
+      <c r="CB38" t="s">
         <v>1389</v>
       </c>
-      <c r="BI38" t="s">
+      <c r="CC38" t="s">
+        <v>1388</v>
+      </c>
+      <c r="CD38" t="s">
         <v>1390</v>
-      </c>
-      <c r="BJ38" t="s">
-        <v>1391</v>
-      </c>
-      <c r="BK38" t="s">
-        <v>1392</v>
-      </c>
-      <c r="BL38" t="s">
-        <v>1393</v>
-      </c>
-      <c r="BM38" t="s">
-        <v>1394</v>
-      </c>
-      <c r="BN38" t="s">
-        <v>1395</v>
-      </c>
-      <c r="BO38" t="s">
-        <v>1396</v>
-      </c>
-      <c r="BP38" t="s">
-        <v>1397</v>
-      </c>
-      <c r="BQ38" t="s">
-        <v>1398</v>
-      </c>
-      <c r="BR38" t="s">
-        <v>1399</v>
-      </c>
-      <c r="BS38" t="s">
-        <v>1400</v>
-      </c>
-      <c r="BT38" t="s">
-        <v>1401</v>
-      </c>
-      <c r="BU38" t="s">
-        <v>1402</v>
-      </c>
-      <c r="BV38" t="s">
-        <v>1403</v>
-      </c>
-      <c r="BW38" t="s">
-        <v>1404</v>
-      </c>
-      <c r="BX38" t="s">
-        <v>1405</v>
-      </c>
-      <c r="BY38" t="s">
-        <v>1406</v>
-      </c>
-      <c r="BZ38" t="s">
-        <v>1401</v>
-      </c>
-      <c r="CA38" t="s">
-        <v>1402</v>
-      </c>
-      <c r="CB38" t="s">
-        <v>1403</v>
-      </c>
-      <c r="CC38" t="s">
-        <v>1404</v>
-      </c>
-      <c r="CD38" t="s">
-        <v>1405</v>
-      </c>
-      <c r="CE38" t="s">
-        <v>1406</v>
       </c>
     </row>
     <row r="39" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>1407</v>
+        <v>1391</v>
       </c>
       <c r="B39" t="s">
         <v>1270</v>
@@ -19361,22 +19283,22 @@
         <v>221</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>1408</v>
+        <v>1392</v>
       </c>
       <c r="G39" t="s">
         <v>126</v>
       </c>
       <c r="H39" t="s">
-        <v>1407</v>
+        <v>1391</v>
       </c>
       <c r="I39" t="s">
-        <v>1407</v>
+        <v>1391</v>
       </c>
       <c r="J39" t="s">
-        <v>1407</v>
+        <v>1391</v>
       </c>
       <c r="K39" t="s">
-        <v>1407</v>
+        <v>1391</v>
       </c>
       <c r="L39" t="s">
         <v>1303</v>
@@ -19469,99 +19391,84 @@
         <v>1356</v>
       </c>
       <c r="BB39" t="s">
-        <v>1409</v>
+        <v>1393</v>
       </c>
       <c r="BC39" t="s">
-        <v>1410</v>
+        <v>1436</v>
       </c>
       <c r="BD39" t="s">
-        <v>1411</v>
+        <v>1395</v>
       </c>
       <c r="BE39" t="s">
-        <v>1412</v>
+        <v>1394</v>
       </c>
       <c r="BF39" t="s">
-        <v>1413</v>
-      </c>
-      <c r="BG39" t="s">
-        <v>1414</v>
+        <v>1396</v>
       </c>
       <c r="BH39" t="s">
-        <v>1415</v>
+        <v>1397</v>
       </c>
       <c r="BI39" t="s">
-        <v>1416</v>
+        <v>1437</v>
       </c>
       <c r="BJ39" t="s">
-        <v>1417</v>
+        <v>1399</v>
       </c>
       <c r="BK39" t="s">
-        <v>1418</v>
+        <v>1398</v>
       </c>
       <c r="BL39" t="s">
-        <v>1419</v>
-      </c>
-      <c r="BM39" t="s">
-        <v>1420</v>
+        <v>1400</v>
       </c>
       <c r="BN39" t="s">
-        <v>1421</v>
+        <v>1401</v>
       </c>
       <c r="BO39" t="s">
-        <v>1422</v>
+        <v>1438</v>
       </c>
       <c r="BP39" t="s">
-        <v>1423</v>
+        <v>1403</v>
       </c>
       <c r="BQ39" t="s">
-        <v>1424</v>
+        <v>1402</v>
       </c>
       <c r="BR39" t="s">
-        <v>1425</v>
-      </c>
-      <c r="BS39" t="s">
-        <v>1426</v>
+        <v>1404</v>
       </c>
       <c r="BT39" t="s">
-        <v>1427</v>
+        <v>1405</v>
       </c>
       <c r="BU39" t="s">
-        <v>1428</v>
+        <v>1439</v>
       </c>
       <c r="BV39" t="s">
-        <v>1429</v>
+        <v>1407</v>
       </c>
       <c r="BW39" t="s">
-        <v>1430</v>
+        <v>1406</v>
       </c>
       <c r="BX39" t="s">
-        <v>1431</v>
-      </c>
-      <c r="BY39" t="s">
-        <v>1432</v>
+        <v>1408</v>
       </c>
       <c r="BZ39" t="s">
-        <v>1427</v>
+        <v>1405</v>
       </c>
       <c r="CA39" t="s">
-        <v>1428</v>
+        <v>1439</v>
       </c>
       <c r="CB39" t="s">
-        <v>1429</v>
+        <v>1407</v>
       </c>
       <c r="CC39" t="s">
-        <v>1430</v>
+        <v>1406</v>
       </c>
       <c r="CD39" t="s">
-        <v>1431</v>
-      </c>
-      <c r="CE39" t="s">
-        <v>1432</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="40" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>1433</v>
+        <v>1409</v>
       </c>
       <c r="B40" t="s">
         <v>1270</v>
@@ -19576,22 +19483,22 @@
         <v>259</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>1434</v>
+        <v>1410</v>
       </c>
       <c r="G40" t="s">
         <v>126</v>
       </c>
       <c r="H40" t="s">
-        <v>1435</v>
+        <v>1411</v>
       </c>
       <c r="I40" t="s">
-        <v>1435</v>
+        <v>1411</v>
       </c>
       <c r="J40" t="s">
-        <v>1435</v>
+        <v>1411</v>
       </c>
       <c r="K40" t="s">
-        <v>1435</v>
+        <v>1411</v>
       </c>
       <c r="L40" t="s">
         <v>1316</v>
@@ -19684,94 +19591,79 @@
         <v>1356</v>
       </c>
       <c r="BB40" t="s">
-        <v>1436</v>
+        <v>1412</v>
       </c>
       <c r="BC40" t="s">
-        <v>1437</v>
+        <v>1440</v>
       </c>
       <c r="BD40" t="s">
-        <v>1438</v>
+        <v>1414</v>
       </c>
       <c r="BE40" t="s">
-        <v>1439</v>
+        <v>1413</v>
       </c>
       <c r="BF40" t="s">
-        <v>1440</v>
-      </c>
-      <c r="BG40" t="s">
+        <v>1415</v>
+      </c>
+      <c r="BH40" t="s">
+        <v>1416</v>
+      </c>
+      <c r="BI40" t="s">
         <v>1441</v>
       </c>
-      <c r="BH40" t="s">
+      <c r="BJ40" t="s">
+        <v>1418</v>
+      </c>
+      <c r="BK40" t="s">
+        <v>1417</v>
+      </c>
+      <c r="BL40" t="s">
+        <v>1419</v>
+      </c>
+      <c r="BN40" t="s">
+        <v>1420</v>
+      </c>
+      <c r="BO40" t="s">
         <v>1442</v>
       </c>
-      <c r="BI40" t="s">
+      <c r="BP40" t="s">
+        <v>1422</v>
+      </c>
+      <c r="BQ40" t="s">
+        <v>1421</v>
+      </c>
+      <c r="BR40" t="s">
+        <v>1423</v>
+      </c>
+      <c r="BT40" t="s">
+        <v>1424</v>
+      </c>
+      <c r="BU40" t="s">
         <v>1443</v>
       </c>
-      <c r="BJ40" t="s">
-        <v>1444</v>
-      </c>
-      <c r="BK40" t="s">
-        <v>1445</v>
-      </c>
-      <c r="BL40" t="s">
-        <v>1446</v>
-      </c>
-      <c r="BM40" t="s">
-        <v>1447</v>
-      </c>
-      <c r="BN40" t="s">
-        <v>1448</v>
-      </c>
-      <c r="BO40" t="s">
-        <v>1449</v>
-      </c>
-      <c r="BP40" t="s">
-        <v>1450</v>
-      </c>
-      <c r="BQ40" t="s">
-        <v>1451</v>
-      </c>
-      <c r="BR40" t="s">
-        <v>1452</v>
-      </c>
-      <c r="BS40" t="s">
-        <v>1453</v>
-      </c>
-      <c r="BT40" t="s">
-        <v>1454</v>
-      </c>
-      <c r="BU40" t="s">
-        <v>1455</v>
-      </c>
       <c r="BV40" t="s">
-        <v>1456</v>
+        <v>1426</v>
       </c>
       <c r="BW40" t="s">
-        <v>1457</v>
+        <v>1425</v>
       </c>
       <c r="BX40" t="s">
-        <v>1458</v>
-      </c>
-      <c r="BY40" t="s">
-        <v>1459</v>
+        <v>1427</v>
       </c>
       <c r="BZ40" t="s">
-        <v>1454</v>
+        <v>1424</v>
       </c>
       <c r="CA40" t="s">
-        <v>1455</v>
+        <v>1443</v>
       </c>
       <c r="CB40" t="s">
-        <v>1456</v>
+        <v>1426</v>
       </c>
       <c r="CC40" t="s">
-        <v>1457</v>
+        <v>1425</v>
       </c>
       <c r="CD40" t="s">
-        <v>1458</v>
-      </c>
-      <c r="CE40" t="s">
-        <v>1459</v>
+        <v>1427</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Maestro: fotos nuevas de los bancos de 90 = main, 7, 4, 3 y 5 de cada idioma
Subidas a Cloudinary en bancos/B.MET.090/<color>/<idioma>/. Espana/Italia/Francia
en su idioma, Alemania/Reino Unido en ingles; la Image 6 queda vacia.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/datos/FICHERO_MAESTRO2.xlsx
+++ b/public/datos/FICHERO_MAESTRO2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Helian\Desktop\Fichero Maestro\Sistema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79AFF6EE-D4ED-4ECC-A339-C71839C403D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A1C7CFF-FE87-40E6-A87F-9F04B82B8B7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="591" xr2:uid="{90124268-D67C-4387-8829-7E3B806257E6}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3677" uniqueCount="1444">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3657" uniqueCount="1500">
   <si>
     <t>Marketplace</t>
   </si>
@@ -3965,24 +3965,6 @@
     <t>La panca da spogliatoio in metallo Twinthink è una soluzione pratica, resistente e versatile per attrezzare spogliatoi, palestre, scuole, uffici e aree comuni con una seduta funzionale e duratura. Progettata per offrire comfort e stabilità nell'uso quotidiano, questa panca metallica da spogliatoio unisce una struttura robusta a uno stile pulito e professionale che si adatta facilmente a diversi ambienti. Realizzata in acciaio ad alta resistenza, questa panca da spogliatoio è pensata per sopportare un uso frequente sia negli spazi interni sia nelle zone esterne coperte. Il suo design metallico facilita la pulizia e la manutenzione, rendendola un'opzione molto pratica per luoghi in cui igiene e durata sono essenziali. Grazie alla superficie liscia e alla struttura solida, offre un'esperienza comoda e stabile da seduti.&lt;br&gt;&lt;br&gt;Questo modello è ideale da collocare accanto a un armadietto da spogliatoio, facilitando il cambio di vestiti, scarpe o accessori in palestre, centri sportivi, aziende, scuole o spogliatoi collettivi. Può essere utilizzata anche come panca da esterno in cortili coperti, ingressi o aree di attesa, offrendo una soluzione funzionale dall'estetica moderna.&lt;br&gt;&lt;br&gt;Oltre alla sua resistenza, la panca metallica Twinthink si distingue per la sua versatilità. Può essere utilizzata in spazi professionali o domestici, adattandosi a diverse esigenze senza perdere il suo stile sobrio ed efficiente. Il suo formato permette di ottimizzare lo spazio disponibile e mantenere l'ordine nelle zone di passaggio o di uso comune.&lt;br&gt;&lt;br&gt;Se cerchi una panca metallica che unisca resistenza, facile manutenzione e design pratico, la panca da spogliatoio Twinthink è un'ottima scelta per migliorare qualsiasi spazio con una soluzione duratura, comoda e funzionale.</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213596/bancos/B.MET.090/gris/img_00.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213599/bancos/B.MET.090/gris/img_01.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213601/bancos/B.MET.090/gris/img_02.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213603/bancos/B.MET.090/gris/img_03.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213606/bancos/B.MET.090/gris/img_04.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213608/bancos/B.MET.090/gris/img_05.jpg</t>
-  </si>
-  <si>
     <t>B.MET.090_N</t>
   </si>
   <si>
@@ -4001,24 +3983,6 @@
     <t>Twinthink Panca da Spogliatoio in Metallo per Palestra e Scuole (Nero)</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213582/bancos/B.MET.090/negro/img_00.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213584/bancos/B.MET.090/negro/img_01.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213587/bancos/B.MET.090/negro/img_02.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213589/bancos/B.MET.090/negro/img_03.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213592/bancos/B.MET.090/negro/img_04.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213594/bancos/B.MET.090/negro/img_05.jpg</t>
-  </si>
-  <si>
     <t>B.MET.090_B</t>
   </si>
   <si>
@@ -4037,24 +4001,6 @@
     <t>Twinthink Panca da Spogliatoio in Metallo per Palestra e Scuole (Bianco)</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213552/bancos/B.MET.090/blanco/img_00.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213554/bancos/B.MET.090/blanco/img_01.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213557/bancos/B.MET.090/blanco/img_02.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213559/bancos/B.MET.090/blanco/img_03.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213562/bancos/B.MET.090/blanco/img_04.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213565/bancos/B.MET.090/blanco/img_05.jpg</t>
-  </si>
-  <si>
     <t>B.MET.090_B-N</t>
   </si>
   <si>
@@ -4074,24 +4020,6 @@
   </si>
   <si>
     <t>Twinthink Panca da Spogliatoio in Metallo per Palestra e Scuole (Bianco/Nero)</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213567/bancos/B.MET.090/byn/img_00.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213569/bancos/B.MET.090/byn/img_01.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213572/bancos/B.MET.090/byn/img_02.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213575/bancos/B.MET.090/byn/img_03.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213577/bancos/B.MET.090/byn/img_04.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1784213580/bancos/B.MET.090/byn/img_05.jpg</t>
   </si>
   <si>
     <t>Twinthink Metall-Umkleidebank für Fitnessstudios und Schulen (Grau)</t>
@@ -4482,6 +4410,246 @@
   </si>
   <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790194889/bancos/B.MET.150/byn/en/pt07.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694982/bancos/B.MET.090/gris/es/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694985/bancos/B.MET.090/gris/es/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694987/bancos/B.MET.090/gris/es/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694990/bancos/B.MET.090/gris/es/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694992/bancos/B.MET.090/gris/es/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695005/bancos/B.MET.090/gris/it/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695008/bancos/B.MET.090/gris/it/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695010/bancos/B.MET.090/gris/it/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695012/bancos/B.MET.090/gris/it/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695014/bancos/B.MET.090/gris/it/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694994/bancos/B.MET.090/gris/fr/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694996/bancos/B.MET.090/gris/fr/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694999/bancos/B.MET.090/gris/fr/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695001/bancos/B.MET.090/gris/fr/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695003/bancos/B.MET.090/gris/fr/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694970/bancos/B.MET.090/gris/en/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694974/bancos/B.MET.090/gris/en/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694976/bancos/B.MET.090/gris/en/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694978/bancos/B.MET.090/gris/en/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694980/bancos/B.MET.090/gris/en/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695027/bancos/B.MET.090/negro/es/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695029/bancos/B.MET.090/negro/es/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695032/bancos/B.MET.090/negro/es/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695034/bancos/B.MET.090/negro/es/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695036/bancos/B.MET.090/negro/es/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695050/bancos/B.MET.090/negro/it/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695053/bancos/B.MET.090/negro/it/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695055/bancos/B.MET.090/negro/it/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695057/bancos/B.MET.090/negro/it/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695060/bancos/B.MET.090/negro/it/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695039/bancos/B.MET.090/negro/fr/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695041/bancos/B.MET.090/negro/fr/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695043/bancos/B.MET.090/negro/fr/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695046/bancos/B.MET.090/negro/fr/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695048/bancos/B.MET.090/negro/fr/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695016/bancos/B.MET.090/negro/en/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695019/bancos/B.MET.090/negro/en/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695021/bancos/B.MET.090/negro/en/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695023/bancos/B.MET.090/negro/en/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790695025/bancos/B.MET.090/negro/en/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694891/bancos/B.MET.090/blanco/es/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694893/bancos/B.MET.090/blanco/es/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694895/bancos/B.MET.090/blanco/es/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694898/bancos/B.MET.090/blanco/es/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694900/bancos/B.MET.090/blanco/es/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694913/bancos/B.MET.090/blanco/it/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694915/bancos/B.MET.090/blanco/it/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694917/bancos/B.MET.090/blanco/it/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694919/bancos/B.MET.090/blanco/it/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694921/bancos/B.MET.090/blanco/it/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694902/bancos/B.MET.090/blanco/fr/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694904/bancos/B.MET.090/blanco/fr/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694906/bancos/B.MET.090/blanco/fr/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694908/bancos/B.MET.090/blanco/fr/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694910/bancos/B.MET.090/blanco/fr/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694880/bancos/B.MET.090/blanco/en/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694883/bancos/B.MET.090/blanco/en/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694885/bancos/B.MET.090/blanco/en/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694887/bancos/B.MET.090/blanco/en/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694889/bancos/B.MET.090/blanco/en/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694934/bancos/B.MET.090/byn/es/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694936/bancos/B.MET.090/byn/es/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694938/bancos/B.MET.090/byn/es/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694941/bancos/B.MET.090/byn/es/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694944/bancos/B.MET.090/byn/es/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694957/bancos/B.MET.090/byn/it/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694959/bancos/B.MET.090/byn/it/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694961/bancos/B.MET.090/byn/it/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694964/bancos/B.MET.090/byn/it/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694966/bancos/B.MET.090/byn/it/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694947/bancos/B.MET.090/byn/fr/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694949/bancos/B.MET.090/byn/fr/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694951/bancos/B.MET.090/byn/fr/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694953/bancos/B.MET.090/byn/fr/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694955/bancos/B.MET.090/byn/fr/pt05.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694923/bancos/B.MET.090/byn/en/main.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694926/bancos/B.MET.090/byn/en/pt07.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694928/bancos/B.MET.090/byn/en/pt04.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694930/bancos/B.MET.090/byn/en/pt03.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694932/bancos/B.MET.090/byn/en/pt05.jpg</t>
   </si>
 </sst>
 </file>
@@ -10403,10 +10571,10 @@
         <v>11</v>
       </c>
       <c r="C203" s="1" t="s">
-        <v>1290</v>
+        <v>1284</v>
       </c>
       <c r="D203" t="s">
-        <v>1289</v>
+        <v>1283</v>
       </c>
       <c r="E203">
         <v>110</v>
@@ -10432,10 +10600,10 @@
         <v>11</v>
       </c>
       <c r="C204" s="1" t="s">
-        <v>1302</v>
+        <v>1290</v>
       </c>
       <c r="D204" t="s">
-        <v>1301</v>
+        <v>1289</v>
       </c>
       <c r="E204">
         <v>110</v>
@@ -10461,10 +10629,10 @@
         <v>11</v>
       </c>
       <c r="C205" s="1" t="s">
-        <v>1314</v>
+        <v>1296</v>
       </c>
       <c r="D205" t="s">
-        <v>1313</v>
+        <v>1295</v>
       </c>
       <c r="E205">
         <v>100</v>
@@ -10490,10 +10658,10 @@
         <v>11</v>
       </c>
       <c r="C206" s="1" t="s">
-        <v>1343</v>
+        <v>1319</v>
       </c>
       <c r="D206" t="s">
-        <v>1341</v>
+        <v>1317</v>
       </c>
       <c r="E206">
         <v>144</v>
@@ -10519,10 +10687,10 @@
         <v>11</v>
       </c>
       <c r="C207" s="1" t="s">
-        <v>1374</v>
+        <v>1350</v>
       </c>
       <c r="D207" t="s">
-        <v>1373</v>
+        <v>1349</v>
       </c>
       <c r="E207">
         <v>144</v>
@@ -10548,10 +10716,10 @@
         <v>11</v>
       </c>
       <c r="C208" s="1" t="s">
-        <v>1392</v>
+        <v>1368</v>
       </c>
       <c r="D208" t="s">
-        <v>1391</v>
+        <v>1367</v>
       </c>
       <c r="E208">
         <v>144</v>
@@ -10577,10 +10745,10 @@
         <v>11</v>
       </c>
       <c r="C209" s="1" t="s">
-        <v>1410</v>
+        <v>1386</v>
       </c>
       <c r="D209" t="s">
-        <v>1409</v>
+        <v>1385</v>
       </c>
       <c r="E209">
         <v>144</v>
@@ -18042,7 +18210,7 @@
         <v>1268</v>
       </c>
     </row>
-    <row r="33" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>1269</v>
       </c>
@@ -18083,7 +18251,7 @@
         <v>1275</v>
       </c>
       <c r="N33" s="14" t="s">
-        <v>1340</v>
+        <v>1316</v>
       </c>
       <c r="O33" t="s">
         <v>1276</v>
@@ -18107,28 +18275,28 @@
         <v>1282</v>
       </c>
       <c r="AB33" t="s">
-        <v>1326</v>
+        <v>1302</v>
       </c>
       <c r="AC33" t="s">
-        <v>1327</v>
+        <v>1303</v>
       </c>
       <c r="AD33" s="14" t="s">
-        <v>1328</v>
+        <v>1304</v>
       </c>
       <c r="AE33" t="s">
-        <v>1329</v>
+        <v>1305</v>
       </c>
       <c r="AF33" t="s">
-        <v>1330</v>
+        <v>1306</v>
       </c>
       <c r="AG33" t="s">
-        <v>1331</v>
+        <v>1307</v>
       </c>
       <c r="AH33" s="14" t="s">
-        <v>1332</v>
+        <v>1308</v>
       </c>
       <c r="AI33" t="s">
-        <v>1333</v>
+        <v>1309</v>
       </c>
       <c r="AJ33">
         <v>45</v>
@@ -18158,99 +18326,84 @@
         <v>149</v>
       </c>
       <c r="BB33" t="s">
+        <v>1420</v>
+      </c>
+      <c r="BC33" t="s">
+        <v>1421</v>
+      </c>
+      <c r="BD33" t="s">
+        <v>1422</v>
+      </c>
+      <c r="BE33" t="s">
+        <v>1423</v>
+      </c>
+      <c r="BF33" t="s">
+        <v>1424</v>
+      </c>
+      <c r="BH33" t="s">
+        <v>1425</v>
+      </c>
+      <c r="BI33" t="s">
+        <v>1426</v>
+      </c>
+      <c r="BJ33" t="s">
+        <v>1427</v>
+      </c>
+      <c r="BK33" t="s">
+        <v>1428</v>
+      </c>
+      <c r="BL33" t="s">
+        <v>1429</v>
+      </c>
+      <c r="BN33" t="s">
+        <v>1430</v>
+      </c>
+      <c r="BO33" t="s">
+        <v>1431</v>
+      </c>
+      <c r="BP33" t="s">
+        <v>1432</v>
+      </c>
+      <c r="BQ33" t="s">
+        <v>1433</v>
+      </c>
+      <c r="BR33" t="s">
+        <v>1434</v>
+      </c>
+      <c r="BT33" t="s">
+        <v>1435</v>
+      </c>
+      <c r="BU33" t="s">
+        <v>1436</v>
+      </c>
+      <c r="BV33" t="s">
+        <v>1437</v>
+      </c>
+      <c r="BW33" t="s">
+        <v>1438</v>
+      </c>
+      <c r="BX33" t="s">
+        <v>1439</v>
+      </c>
+      <c r="BZ33" t="s">
+        <v>1435</v>
+      </c>
+      <c r="CA33" t="s">
+        <v>1436</v>
+      </c>
+      <c r="CB33" t="s">
+        <v>1437</v>
+      </c>
+      <c r="CC33" t="s">
+        <v>1438</v>
+      </c>
+      <c r="CD33" t="s">
+        <v>1439</v>
+      </c>
+    </row>
+    <row r="34" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>1283</v>
-      </c>
-      <c r="BC33" t="s">
-        <v>1284</v>
-      </c>
-      <c r="BD33" t="s">
-        <v>1285</v>
-      </c>
-      <c r="BE33" t="s">
-        <v>1286</v>
-      </c>
-      <c r="BF33" t="s">
-        <v>1287</v>
-      </c>
-      <c r="BG33" t="s">
-        <v>1288</v>
-      </c>
-      <c r="BH33" t="s">
-        <v>1283</v>
-      </c>
-      <c r="BI33" t="s">
-        <v>1284</v>
-      </c>
-      <c r="BJ33" t="s">
-        <v>1285</v>
-      </c>
-      <c r="BK33" t="s">
-        <v>1286</v>
-      </c>
-      <c r="BL33" t="s">
-        <v>1287</v>
-      </c>
-      <c r="BM33" t="s">
-        <v>1288</v>
-      </c>
-      <c r="BN33" t="s">
-        <v>1283</v>
-      </c>
-      <c r="BO33" t="s">
-        <v>1284</v>
-      </c>
-      <c r="BP33" t="s">
-        <v>1285</v>
-      </c>
-      <c r="BQ33" t="s">
-        <v>1286</v>
-      </c>
-      <c r="BR33" t="s">
-        <v>1287</v>
-      </c>
-      <c r="BS33" t="s">
-        <v>1288</v>
-      </c>
-      <c r="BT33" t="s">
-        <v>1283</v>
-      </c>
-      <c r="BU33" t="s">
-        <v>1284</v>
-      </c>
-      <c r="BV33" t="s">
-        <v>1285</v>
-      </c>
-      <c r="BW33" t="s">
-        <v>1286</v>
-      </c>
-      <c r="BX33" t="s">
-        <v>1287</v>
-      </c>
-      <c r="BY33" t="s">
-        <v>1288</v>
-      </c>
-      <c r="BZ33" t="s">
-        <v>1283</v>
-      </c>
-      <c r="CA33" t="s">
-        <v>1284</v>
-      </c>
-      <c r="CB33" t="s">
-        <v>1285</v>
-      </c>
-      <c r="CC33" t="s">
-        <v>1286</v>
-      </c>
-      <c r="CD33" t="s">
-        <v>1287</v>
-      </c>
-      <c r="CE33" t="s">
-        <v>1288</v>
-      </c>
-    </row>
-    <row r="34" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>1289</v>
       </c>
       <c r="B34" t="s">
         <v>1270</v>
@@ -18265,76 +18418,76 @@
         <v>182</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>1290</v>
+        <v>1284</v>
       </c>
       <c r="G34" t="s">
         <v>126</v>
       </c>
       <c r="H34" t="s">
-        <v>1289</v>
+        <v>1283</v>
       </c>
       <c r="I34" t="s">
-        <v>1289</v>
+        <v>1283</v>
       </c>
       <c r="J34" t="s">
-        <v>1289</v>
+        <v>1283</v>
       </c>
       <c r="K34" t="s">
-        <v>1289</v>
+        <v>1283</v>
       </c>
       <c r="L34" t="s">
-        <v>1291</v>
+        <v>1285</v>
       </c>
       <c r="M34" t="s">
         <v>1275</v>
       </c>
       <c r="N34" s="14" t="s">
-        <v>1340</v>
+        <v>1316</v>
       </c>
       <c r="O34" t="s">
         <v>1276</v>
       </c>
       <c r="P34" t="s">
-        <v>1292</v>
+        <v>1286</v>
       </c>
       <c r="Q34" t="s">
         <v>1278</v>
       </c>
       <c r="T34" t="s">
-        <v>1293</v>
+        <v>1287</v>
       </c>
       <c r="U34" t="s">
         <v>1280</v>
       </c>
       <c r="X34" t="s">
-        <v>1294</v>
+        <v>1288</v>
       </c>
       <c r="Y34" t="s">
         <v>1282</v>
       </c>
       <c r="AB34" t="s">
-        <v>1334</v>
+        <v>1310</v>
       </c>
       <c r="AC34" t="s">
-        <v>1327</v>
+        <v>1303</v>
       </c>
       <c r="AD34" s="14" t="s">
-        <v>1328</v>
+        <v>1304</v>
       </c>
       <c r="AE34" t="s">
-        <v>1329</v>
+        <v>1305</v>
       </c>
       <c r="AF34" t="s">
-        <v>1335</v>
+        <v>1311</v>
       </c>
       <c r="AG34" t="s">
-        <v>1331</v>
+        <v>1307</v>
       </c>
       <c r="AH34" s="14" t="s">
-        <v>1332</v>
+        <v>1308</v>
       </c>
       <c r="AI34" t="s">
-        <v>1333</v>
+        <v>1309</v>
       </c>
       <c r="AJ34">
         <v>45</v>
@@ -18364,99 +18517,84 @@
         <v>149</v>
       </c>
       <c r="BB34" t="s">
-        <v>1295</v>
+        <v>1440</v>
       </c>
       <c r="BC34" t="s">
-        <v>1296</v>
+        <v>1441</v>
       </c>
       <c r="BD34" t="s">
-        <v>1297</v>
+        <v>1442</v>
       </c>
       <c r="BE34" t="s">
-        <v>1298</v>
+        <v>1443</v>
       </c>
       <c r="BF34" t="s">
-        <v>1299</v>
-      </c>
-      <c r="BG34" t="s">
-        <v>1300</v>
+        <v>1444</v>
       </c>
       <c r="BH34" t="s">
-        <v>1295</v>
+        <v>1445</v>
       </c>
       <c r="BI34" t="s">
-        <v>1296</v>
+        <v>1446</v>
       </c>
       <c r="BJ34" t="s">
-        <v>1297</v>
+        <v>1447</v>
       </c>
       <c r="BK34" t="s">
-        <v>1298</v>
+        <v>1448</v>
       </c>
       <c r="BL34" t="s">
-        <v>1299</v>
-      </c>
-      <c r="BM34" t="s">
-        <v>1300</v>
+        <v>1449</v>
       </c>
       <c r="BN34" t="s">
-        <v>1295</v>
+        <v>1450</v>
       </c>
       <c r="BO34" t="s">
-        <v>1296</v>
+        <v>1451</v>
       </c>
       <c r="BP34" t="s">
-        <v>1297</v>
+        <v>1452</v>
       </c>
       <c r="BQ34" t="s">
-        <v>1298</v>
+        <v>1453</v>
       </c>
       <c r="BR34" t="s">
-        <v>1299</v>
-      </c>
-      <c r="BS34" t="s">
-        <v>1300</v>
+        <v>1454</v>
       </c>
       <c r="BT34" t="s">
-        <v>1295</v>
+        <v>1455</v>
       </c>
       <c r="BU34" t="s">
-        <v>1296</v>
+        <v>1456</v>
       </c>
       <c r="BV34" t="s">
-        <v>1297</v>
+        <v>1457</v>
       </c>
       <c r="BW34" t="s">
-        <v>1298</v>
+        <v>1458</v>
       </c>
       <c r="BX34" t="s">
-        <v>1299</v>
-      </c>
-      <c r="BY34" t="s">
-        <v>1300</v>
+        <v>1459</v>
       </c>
       <c r="BZ34" t="s">
-        <v>1295</v>
+        <v>1455</v>
       </c>
       <c r="CA34" t="s">
-        <v>1296</v>
+        <v>1456</v>
       </c>
       <c r="CB34" t="s">
-        <v>1297</v>
+        <v>1457</v>
       </c>
       <c r="CC34" t="s">
-        <v>1298</v>
+        <v>1458</v>
       </c>
       <c r="CD34" t="s">
-        <v>1299</v>
-      </c>
-      <c r="CE34" t="s">
-        <v>1300</v>
-      </c>
-    </row>
-    <row r="35" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+        <v>1459</v>
+      </c>
+    </row>
+    <row r="35" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>1301</v>
+        <v>1289</v>
       </c>
       <c r="B35" t="s">
         <v>1270</v>
@@ -18471,76 +18609,76 @@
         <v>221</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>1302</v>
+        <v>1290</v>
       </c>
       <c r="G35" t="s">
         <v>126</v>
       </c>
       <c r="H35" t="s">
-        <v>1301</v>
+        <v>1289</v>
       </c>
       <c r="I35" t="s">
-        <v>1301</v>
+        <v>1289</v>
       </c>
       <c r="J35" t="s">
-        <v>1301</v>
+        <v>1289</v>
       </c>
       <c r="K35" t="s">
-        <v>1301</v>
+        <v>1289</v>
       </c>
       <c r="L35" t="s">
-        <v>1303</v>
+        <v>1291</v>
       </c>
       <c r="M35" t="s">
         <v>1275</v>
       </c>
       <c r="N35" s="14" t="s">
-        <v>1340</v>
+        <v>1316</v>
       </c>
       <c r="O35" t="s">
         <v>1276</v>
       </c>
       <c r="P35" t="s">
-        <v>1304</v>
+        <v>1292</v>
       </c>
       <c r="Q35" t="s">
         <v>1278</v>
       </c>
       <c r="T35" t="s">
-        <v>1305</v>
+        <v>1293</v>
       </c>
       <c r="U35" t="s">
         <v>1280</v>
       </c>
       <c r="X35" t="s">
-        <v>1306</v>
+        <v>1294</v>
       </c>
       <c r="Y35" t="s">
         <v>1282</v>
       </c>
       <c r="AB35" t="s">
-        <v>1336</v>
+        <v>1312</v>
       </c>
       <c r="AC35" t="s">
-        <v>1327</v>
+        <v>1303</v>
       </c>
       <c r="AD35" s="14" t="s">
-        <v>1328</v>
+        <v>1304</v>
       </c>
       <c r="AE35" t="s">
-        <v>1329</v>
+        <v>1305</v>
       </c>
       <c r="AF35" t="s">
-        <v>1337</v>
+        <v>1313</v>
       </c>
       <c r="AG35" t="s">
-        <v>1331</v>
+        <v>1307</v>
       </c>
       <c r="AH35" s="14" t="s">
-        <v>1332</v>
+        <v>1308</v>
       </c>
       <c r="AI35" t="s">
-        <v>1333</v>
+        <v>1309</v>
       </c>
       <c r="AJ35">
         <v>45</v>
@@ -18570,99 +18708,84 @@
         <v>149</v>
       </c>
       <c r="BB35" t="s">
-        <v>1307</v>
+        <v>1460</v>
       </c>
       <c r="BC35" t="s">
-        <v>1308</v>
+        <v>1461</v>
       </c>
       <c r="BD35" t="s">
-        <v>1309</v>
+        <v>1462</v>
       </c>
       <c r="BE35" t="s">
-        <v>1310</v>
+        <v>1463</v>
       </c>
       <c r="BF35" t="s">
-        <v>1311</v>
-      </c>
-      <c r="BG35" t="s">
-        <v>1312</v>
+        <v>1464</v>
       </c>
       <c r="BH35" t="s">
-        <v>1307</v>
+        <v>1465</v>
       </c>
       <c r="BI35" t="s">
-        <v>1308</v>
+        <v>1466</v>
       </c>
       <c r="BJ35" t="s">
-        <v>1309</v>
+        <v>1467</v>
       </c>
       <c r="BK35" t="s">
-        <v>1310</v>
+        <v>1468</v>
       </c>
       <c r="BL35" t="s">
-        <v>1311</v>
-      </c>
-      <c r="BM35" t="s">
-        <v>1312</v>
+        <v>1469</v>
       </c>
       <c r="BN35" t="s">
-        <v>1307</v>
+        <v>1470</v>
       </c>
       <c r="BO35" t="s">
-        <v>1308</v>
+        <v>1471</v>
       </c>
       <c r="BP35" t="s">
-        <v>1309</v>
+        <v>1472</v>
       </c>
       <c r="BQ35" t="s">
-        <v>1310</v>
+        <v>1473</v>
       </c>
       <c r="BR35" t="s">
-        <v>1311</v>
-      </c>
-      <c r="BS35" t="s">
-        <v>1312</v>
+        <v>1474</v>
       </c>
       <c r="BT35" t="s">
-        <v>1307</v>
+        <v>1475</v>
       </c>
       <c r="BU35" t="s">
-        <v>1308</v>
+        <v>1476</v>
       </c>
       <c r="BV35" t="s">
-        <v>1309</v>
+        <v>1477</v>
       </c>
       <c r="BW35" t="s">
-        <v>1310</v>
+        <v>1478</v>
       </c>
       <c r="BX35" t="s">
-        <v>1311</v>
-      </c>
-      <c r="BY35" t="s">
-        <v>1312</v>
+        <v>1479</v>
       </c>
       <c r="BZ35" t="s">
-        <v>1307</v>
+        <v>1475</v>
       </c>
       <c r="CA35" t="s">
-        <v>1308</v>
+        <v>1476</v>
       </c>
       <c r="CB35" t="s">
-        <v>1309</v>
+        <v>1477</v>
       </c>
       <c r="CC35" t="s">
-        <v>1310</v>
+        <v>1478</v>
       </c>
       <c r="CD35" t="s">
-        <v>1311</v>
-      </c>
-      <c r="CE35" t="s">
-        <v>1312</v>
-      </c>
-    </row>
-    <row r="36" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+        <v>1479</v>
+      </c>
+    </row>
+    <row r="36" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>1313</v>
+        <v>1295</v>
       </c>
       <c r="B36" t="s">
         <v>1270</v>
@@ -18677,76 +18800,76 @@
         <v>259</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>1314</v>
+        <v>1296</v>
       </c>
       <c r="G36" t="s">
         <v>126</v>
       </c>
       <c r="H36" t="s">
-        <v>1315</v>
+        <v>1297</v>
       </c>
       <c r="I36" t="s">
-        <v>1315</v>
+        <v>1297</v>
       </c>
       <c r="J36" t="s">
-        <v>1315</v>
+        <v>1297</v>
       </c>
       <c r="K36" t="s">
-        <v>1315</v>
+        <v>1297</v>
       </c>
       <c r="L36" t="s">
-        <v>1316</v>
+        <v>1298</v>
       </c>
       <c r="M36" t="s">
         <v>1275</v>
       </c>
       <c r="N36" s="14" t="s">
-        <v>1340</v>
+        <v>1316</v>
       </c>
       <c r="O36" t="s">
         <v>1276</v>
       </c>
       <c r="P36" t="s">
-        <v>1317</v>
+        <v>1299</v>
       </c>
       <c r="Q36" t="s">
         <v>1278</v>
       </c>
       <c r="T36" t="s">
-        <v>1318</v>
+        <v>1300</v>
       </c>
       <c r="U36" t="s">
         <v>1280</v>
       </c>
       <c r="X36" t="s">
-        <v>1319</v>
+        <v>1301</v>
       </c>
       <c r="Y36" t="s">
         <v>1282</v>
       </c>
       <c r="AB36" t="s">
-        <v>1338</v>
+        <v>1314</v>
       </c>
       <c r="AC36" t="s">
-        <v>1327</v>
+        <v>1303</v>
       </c>
       <c r="AD36" s="14" t="s">
-        <v>1328</v>
+        <v>1304</v>
       </c>
       <c r="AE36" t="s">
-        <v>1329</v>
+        <v>1305</v>
       </c>
       <c r="AF36" t="s">
-        <v>1339</v>
+        <v>1315</v>
       </c>
       <c r="AG36" t="s">
-        <v>1331</v>
+        <v>1307</v>
       </c>
       <c r="AH36" s="14" t="s">
-        <v>1332</v>
+        <v>1308</v>
       </c>
       <c r="AI36" t="s">
-        <v>1333</v>
+        <v>1309</v>
       </c>
       <c r="AJ36">
         <v>45</v>
@@ -18776,105 +18899,90 @@
         <v>149</v>
       </c>
       <c r="BB36" t="s">
-        <v>1320</v>
+        <v>1480</v>
       </c>
       <c r="BC36" t="s">
-        <v>1321</v>
+        <v>1481</v>
       </c>
       <c r="BD36" t="s">
-        <v>1322</v>
+        <v>1482</v>
       </c>
       <c r="BE36" t="s">
-        <v>1323</v>
+        <v>1483</v>
       </c>
       <c r="BF36" t="s">
-        <v>1324</v>
-      </c>
-      <c r="BG36" t="s">
-        <v>1325</v>
+        <v>1484</v>
       </c>
       <c r="BH36" t="s">
-        <v>1320</v>
+        <v>1485</v>
       </c>
       <c r="BI36" t="s">
-        <v>1321</v>
+        <v>1486</v>
       </c>
       <c r="BJ36" t="s">
-        <v>1322</v>
+        <v>1487</v>
       </c>
       <c r="BK36" t="s">
-        <v>1323</v>
+        <v>1488</v>
       </c>
       <c r="BL36" t="s">
-        <v>1324</v>
-      </c>
-      <c r="BM36" t="s">
-        <v>1325</v>
+        <v>1489</v>
       </c>
       <c r="BN36" t="s">
-        <v>1320</v>
+        <v>1490</v>
       </c>
       <c r="BO36" t="s">
-        <v>1321</v>
+        <v>1491</v>
       </c>
       <c r="BP36" t="s">
-        <v>1322</v>
+        <v>1492</v>
       </c>
       <c r="BQ36" t="s">
-        <v>1323</v>
+        <v>1493</v>
       </c>
       <c r="BR36" t="s">
-        <v>1324</v>
-      </c>
-      <c r="BS36" t="s">
-        <v>1325</v>
+        <v>1494</v>
       </c>
       <c r="BT36" t="s">
-        <v>1320</v>
+        <v>1495</v>
       </c>
       <c r="BU36" t="s">
-        <v>1321</v>
+        <v>1496</v>
       </c>
       <c r="BV36" t="s">
-        <v>1322</v>
+        <v>1497</v>
       </c>
       <c r="BW36" t="s">
-        <v>1323</v>
+        <v>1498</v>
       </c>
       <c r="BX36" t="s">
-        <v>1324</v>
-      </c>
-      <c r="BY36" t="s">
-        <v>1325</v>
+        <v>1499</v>
       </c>
       <c r="BZ36" t="s">
-        <v>1320</v>
+        <v>1495</v>
       </c>
       <c r="CA36" t="s">
-        <v>1321</v>
+        <v>1496</v>
       </c>
       <c r="CB36" t="s">
-        <v>1322</v>
+        <v>1497</v>
       </c>
       <c r="CC36" t="s">
-        <v>1323</v>
+        <v>1498</v>
       </c>
       <c r="CD36" t="s">
-        <v>1324</v>
-      </c>
-      <c r="CE36" t="s">
-        <v>1325</v>
-      </c>
-    </row>
-    <row r="37" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+        <v>1499</v>
+      </c>
+    </row>
+    <row r="37" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>1341</v>
+        <v>1317</v>
       </c>
       <c r="B37" t="s">
         <v>1270</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>1342</v>
+        <v>1318</v>
       </c>
       <c r="D37" t="s">
         <v>123</v>
@@ -18883,31 +18991,31 @@
         <v>124</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>1343</v>
+        <v>1319</v>
       </c>
       <c r="G37" t="s">
         <v>126</v>
       </c>
       <c r="H37" t="s">
-        <v>1344</v>
+        <v>1320</v>
       </c>
       <c r="I37" t="s">
-        <v>1344</v>
+        <v>1320</v>
       </c>
       <c r="J37" t="s">
-        <v>1344</v>
+        <v>1320</v>
       </c>
       <c r="K37" t="s">
-        <v>1344</v>
+        <v>1320</v>
       </c>
       <c r="L37" t="s">
         <v>1274</v>
       </c>
       <c r="M37" t="s">
-        <v>1345</v>
+        <v>1321</v>
       </c>
       <c r="N37" s="14" t="s">
-        <v>1346</v>
+        <v>1322</v>
       </c>
       <c r="O37" t="s">
         <v>1276</v>
@@ -18916,52 +19024,52 @@
         <v>1277</v>
       </c>
       <c r="Q37" t="s">
-        <v>1347</v>
+        <v>1323</v>
       </c>
       <c r="R37" s="14" t="s">
-        <v>1348</v>
+        <v>1324</v>
       </c>
       <c r="T37" t="s">
         <v>1279</v>
       </c>
       <c r="U37" t="s">
-        <v>1349</v>
+        <v>1325</v>
       </c>
       <c r="V37" s="14" t="s">
-        <v>1350</v>
+        <v>1326</v>
       </c>
       <c r="X37" t="s">
         <v>1281</v>
       </c>
       <c r="Y37" t="s">
-        <v>1351</v>
+        <v>1327</v>
       </c>
       <c r="Z37" s="14" t="s">
-        <v>1352</v>
+        <v>1328</v>
       </c>
       <c r="AB37" t="s">
-        <v>1326</v>
+        <v>1302</v>
       </c>
       <c r="AC37" t="s">
-        <v>1353</v>
+        <v>1329</v>
       </c>
       <c r="AD37" s="14" t="s">
-        <v>1354</v>
+        <v>1330</v>
       </c>
       <c r="AE37" t="s">
-        <v>1329</v>
+        <v>1305</v>
       </c>
       <c r="AF37" t="s">
-        <v>1330</v>
+        <v>1306</v>
       </c>
       <c r="AG37" t="s">
+        <v>1307</v>
+      </c>
+      <c r="AH37" s="14" t="s">
         <v>1331</v>
       </c>
-      <c r="AH37" s="14" t="s">
-        <v>1355</v>
-      </c>
       <c r="AI37" t="s">
-        <v>1333</v>
+        <v>1309</v>
       </c>
       <c r="AJ37">
         <v>45</v>
@@ -18988,93 +19096,93 @@
         <v>146</v>
       </c>
       <c r="AU37" t="s">
-        <v>1356</v>
+        <v>1332</v>
       </c>
       <c r="BB37" t="s">
-        <v>1357</v>
+        <v>1333</v>
       </c>
       <c r="BC37" t="s">
-        <v>1428</v>
+        <v>1404</v>
       </c>
       <c r="BD37" t="s">
-        <v>1359</v>
+        <v>1335</v>
       </c>
       <c r="BE37" t="s">
-        <v>1358</v>
+        <v>1334</v>
       </c>
       <c r="BF37" t="s">
-        <v>1360</v>
+        <v>1336</v>
       </c>
       <c r="BH37" t="s">
-        <v>1361</v>
+        <v>1337</v>
       </c>
       <c r="BI37" t="s">
-        <v>1429</v>
+        <v>1405</v>
       </c>
       <c r="BJ37" t="s">
-        <v>1363</v>
+        <v>1339</v>
       </c>
       <c r="BK37" t="s">
-        <v>1362</v>
+        <v>1338</v>
       </c>
       <c r="BL37" t="s">
-        <v>1364</v>
+        <v>1340</v>
       </c>
       <c r="BN37" t="s">
-        <v>1365</v>
+        <v>1341</v>
       </c>
       <c r="BO37" t="s">
-        <v>1430</v>
+        <v>1406</v>
       </c>
       <c r="BP37" t="s">
-        <v>1367</v>
+        <v>1343</v>
       </c>
       <c r="BQ37" t="s">
-        <v>1366</v>
+        <v>1342</v>
       </c>
       <c r="BR37" t="s">
-        <v>1368</v>
+        <v>1344</v>
       </c>
       <c r="BT37" t="s">
-        <v>1369</v>
+        <v>1345</v>
       </c>
       <c r="BU37" t="s">
-        <v>1431</v>
+        <v>1407</v>
       </c>
       <c r="BV37" t="s">
-        <v>1371</v>
+        <v>1347</v>
       </c>
       <c r="BW37" t="s">
-        <v>1370</v>
+        <v>1346</v>
       </c>
       <c r="BX37" t="s">
-        <v>1372</v>
+        <v>1348</v>
       </c>
       <c r="BZ37" t="s">
-        <v>1369</v>
+        <v>1345</v>
       </c>
       <c r="CA37" t="s">
-        <v>1431</v>
+        <v>1407</v>
       </c>
       <c r="CB37" t="s">
-        <v>1371</v>
+        <v>1347</v>
       </c>
       <c r="CC37" t="s">
-        <v>1370</v>
+        <v>1346</v>
       </c>
       <c r="CD37" t="s">
-        <v>1372</v>
-      </c>
-    </row>
-    <row r="38" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+        <v>1348</v>
+      </c>
+    </row>
+    <row r="38" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>1373</v>
+        <v>1349</v>
       </c>
       <c r="B38" t="s">
         <v>1270</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>1342</v>
+        <v>1318</v>
       </c>
       <c r="D38" t="s">
         <v>181</v>
@@ -19083,85 +19191,85 @@
         <v>182</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>1374</v>
+        <v>1350</v>
       </c>
       <c r="G38" t="s">
         <v>126</v>
       </c>
       <c r="H38" t="s">
-        <v>1373</v>
+        <v>1349</v>
       </c>
       <c r="I38" t="s">
-        <v>1373</v>
+        <v>1349</v>
       </c>
       <c r="J38" t="s">
-        <v>1373</v>
+        <v>1349</v>
       </c>
       <c r="K38" t="s">
-        <v>1373</v>
+        <v>1349</v>
       </c>
       <c r="L38" t="s">
-        <v>1291</v>
+        <v>1285</v>
       </c>
       <c r="M38" t="s">
-        <v>1345</v>
+        <v>1321</v>
       </c>
       <c r="N38" s="14" t="s">
-        <v>1346</v>
+        <v>1322</v>
       </c>
       <c r="O38" t="s">
         <v>1276</v>
       </c>
       <c r="P38" t="s">
-        <v>1292</v>
+        <v>1286</v>
       </c>
       <c r="Q38" t="s">
-        <v>1347</v>
+        <v>1323</v>
       </c>
       <c r="R38" s="14" t="s">
-        <v>1348</v>
+        <v>1324</v>
       </c>
       <c r="T38" t="s">
-        <v>1293</v>
+        <v>1287</v>
       </c>
       <c r="U38" t="s">
-        <v>1349</v>
+        <v>1325</v>
       </c>
       <c r="V38" s="14" t="s">
-        <v>1350</v>
+        <v>1326</v>
       </c>
       <c r="X38" t="s">
-        <v>1294</v>
+        <v>1288</v>
       </c>
       <c r="Y38" t="s">
-        <v>1351</v>
+        <v>1327</v>
       </c>
       <c r="Z38" s="14" t="s">
-        <v>1352</v>
+        <v>1328</v>
       </c>
       <c r="AB38" t="s">
-        <v>1334</v>
+        <v>1310</v>
       </c>
       <c r="AC38" t="s">
-        <v>1353</v>
+        <v>1329</v>
       </c>
       <c r="AD38" s="14" t="s">
-        <v>1354</v>
+        <v>1330</v>
       </c>
       <c r="AE38" t="s">
-        <v>1329</v>
+        <v>1305</v>
       </c>
       <c r="AF38" t="s">
-        <v>1335</v>
+        <v>1311</v>
       </c>
       <c r="AG38" t="s">
+        <v>1307</v>
+      </c>
+      <c r="AH38" s="14" t="s">
         <v>1331</v>
       </c>
-      <c r="AH38" s="14" t="s">
-        <v>1355</v>
-      </c>
       <c r="AI38" t="s">
-        <v>1333</v>
+        <v>1309</v>
       </c>
       <c r="AJ38">
         <v>45</v>
@@ -19188,93 +19296,93 @@
         <v>146</v>
       </c>
       <c r="AU38" t="s">
+        <v>1332</v>
+      </c>
+      <c r="BB38" t="s">
+        <v>1351</v>
+      </c>
+      <c r="BC38" t="s">
+        <v>1408</v>
+      </c>
+      <c r="BD38" t="s">
+        <v>1353</v>
+      </c>
+      <c r="BE38" t="s">
+        <v>1352</v>
+      </c>
+      <c r="BF38" t="s">
+        <v>1354</v>
+      </c>
+      <c r="BH38" t="s">
+        <v>1355</v>
+      </c>
+      <c r="BI38" t="s">
+        <v>1409</v>
+      </c>
+      <c r="BJ38" t="s">
+        <v>1357</v>
+      </c>
+      <c r="BK38" t="s">
         <v>1356</v>
       </c>
-      <c r="BB38" t="s">
-        <v>1375</v>
-      </c>
-      <c r="BC38" t="s">
-        <v>1432</v>
-      </c>
-      <c r="BD38" t="s">
-        <v>1377</v>
-      </c>
-      <c r="BE38" t="s">
-        <v>1376</v>
-      </c>
-      <c r="BF38" t="s">
-        <v>1378</v>
-      </c>
-      <c r="BH38" t="s">
-        <v>1379</v>
-      </c>
-      <c r="BI38" t="s">
-        <v>1433</v>
-      </c>
-      <c r="BJ38" t="s">
-        <v>1381</v>
-      </c>
-      <c r="BK38" t="s">
-        <v>1380</v>
-      </c>
       <c r="BL38" t="s">
-        <v>1382</v>
+        <v>1358</v>
       </c>
       <c r="BN38" t="s">
-        <v>1383</v>
+        <v>1359</v>
       </c>
       <c r="BO38" t="s">
-        <v>1434</v>
+        <v>1410</v>
       </c>
       <c r="BP38" t="s">
-        <v>1385</v>
+        <v>1361</v>
       </c>
       <c r="BQ38" t="s">
-        <v>1384</v>
+        <v>1360</v>
       </c>
       <c r="BR38" t="s">
-        <v>1386</v>
+        <v>1362</v>
       </c>
       <c r="BT38" t="s">
-        <v>1387</v>
+        <v>1363</v>
       </c>
       <c r="BU38" t="s">
-        <v>1435</v>
+        <v>1411</v>
       </c>
       <c r="BV38" t="s">
-        <v>1389</v>
+        <v>1365</v>
       </c>
       <c r="BW38" t="s">
-        <v>1388</v>
+        <v>1364</v>
       </c>
       <c r="BX38" t="s">
-        <v>1390</v>
+        <v>1366</v>
       </c>
       <c r="BZ38" t="s">
-        <v>1387</v>
+        <v>1363</v>
       </c>
       <c r="CA38" t="s">
-        <v>1435</v>
+        <v>1411</v>
       </c>
       <c r="CB38" t="s">
-        <v>1389</v>
+        <v>1365</v>
       </c>
       <c r="CC38" t="s">
-        <v>1388</v>
+        <v>1364</v>
       </c>
       <c r="CD38" t="s">
-        <v>1390</v>
-      </c>
-    </row>
-    <row r="39" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+        <v>1366</v>
+      </c>
+    </row>
+    <row r="39" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>1391</v>
+        <v>1367</v>
       </c>
       <c r="B39" t="s">
         <v>1270</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>1342</v>
+        <v>1318</v>
       </c>
       <c r="D39" t="s">
         <v>220</v>
@@ -19283,85 +19391,85 @@
         <v>221</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>1392</v>
+        <v>1368</v>
       </c>
       <c r="G39" t="s">
         <v>126</v>
       </c>
       <c r="H39" t="s">
-        <v>1391</v>
+        <v>1367</v>
       </c>
       <c r="I39" t="s">
-        <v>1391</v>
+        <v>1367</v>
       </c>
       <c r="J39" t="s">
-        <v>1391</v>
+        <v>1367</v>
       </c>
       <c r="K39" t="s">
-        <v>1391</v>
+        <v>1367</v>
       </c>
       <c r="L39" t="s">
-        <v>1303</v>
+        <v>1291</v>
       </c>
       <c r="M39" t="s">
-        <v>1345</v>
+        <v>1321</v>
       </c>
       <c r="N39" s="14" t="s">
-        <v>1346</v>
+        <v>1322</v>
       </c>
       <c r="O39" t="s">
         <v>1276</v>
       </c>
       <c r="P39" t="s">
-        <v>1304</v>
+        <v>1292</v>
       </c>
       <c r="Q39" t="s">
-        <v>1347</v>
+        <v>1323</v>
       </c>
       <c r="R39" s="14" t="s">
-        <v>1348</v>
+        <v>1324</v>
       </c>
       <c r="T39" t="s">
+        <v>1293</v>
+      </c>
+      <c r="U39" t="s">
+        <v>1325</v>
+      </c>
+      <c r="V39" s="14" t="s">
+        <v>1326</v>
+      </c>
+      <c r="X39" t="s">
+        <v>1294</v>
+      </c>
+      <c r="Y39" t="s">
+        <v>1327</v>
+      </c>
+      <c r="Z39" s="14" t="s">
+        <v>1328</v>
+      </c>
+      <c r="AB39" t="s">
+        <v>1312</v>
+      </c>
+      <c r="AC39" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AD39" s="14" t="s">
+        <v>1330</v>
+      </c>
+      <c r="AE39" t="s">
         <v>1305</v>
       </c>
-      <c r="U39" t="s">
-        <v>1349</v>
-      </c>
-      <c r="V39" s="14" t="s">
-        <v>1350</v>
-      </c>
-      <c r="X39" t="s">
-        <v>1306</v>
-      </c>
-      <c r="Y39" t="s">
-        <v>1351</v>
-      </c>
-      <c r="Z39" s="14" t="s">
-        <v>1352</v>
-      </c>
-      <c r="AB39" t="s">
-        <v>1336</v>
-      </c>
-      <c r="AC39" t="s">
-        <v>1353</v>
-      </c>
-      <c r="AD39" s="14" t="s">
-        <v>1354</v>
-      </c>
-      <c r="AE39" t="s">
-        <v>1329</v>
-      </c>
       <c r="AF39" t="s">
-        <v>1337</v>
+        <v>1313</v>
       </c>
       <c r="AG39" t="s">
+        <v>1307</v>
+      </c>
+      <c r="AH39" s="14" t="s">
         <v>1331</v>
       </c>
-      <c r="AH39" s="14" t="s">
-        <v>1355</v>
-      </c>
       <c r="AI39" t="s">
-        <v>1333</v>
+        <v>1309</v>
       </c>
       <c r="AJ39">
         <v>45</v>
@@ -19388,93 +19496,93 @@
         <v>146</v>
       </c>
       <c r="AU39" t="s">
-        <v>1356</v>
+        <v>1332</v>
       </c>
       <c r="BB39" t="s">
-        <v>1393</v>
+        <v>1369</v>
       </c>
       <c r="BC39" t="s">
-        <v>1436</v>
+        <v>1412</v>
       </c>
       <c r="BD39" t="s">
-        <v>1395</v>
+        <v>1371</v>
       </c>
       <c r="BE39" t="s">
-        <v>1394</v>
+        <v>1370</v>
       </c>
       <c r="BF39" t="s">
-        <v>1396</v>
+        <v>1372</v>
       </c>
       <c r="BH39" t="s">
-        <v>1397</v>
+        <v>1373</v>
       </c>
       <c r="BI39" t="s">
-        <v>1437</v>
+        <v>1413</v>
       </c>
       <c r="BJ39" t="s">
-        <v>1399</v>
+        <v>1375</v>
       </c>
       <c r="BK39" t="s">
-        <v>1398</v>
+        <v>1374</v>
       </c>
       <c r="BL39" t="s">
-        <v>1400</v>
+        <v>1376</v>
       </c>
       <c r="BN39" t="s">
-        <v>1401</v>
+        <v>1377</v>
       </c>
       <c r="BO39" t="s">
-        <v>1438</v>
+        <v>1414</v>
       </c>
       <c r="BP39" t="s">
-        <v>1403</v>
+        <v>1379</v>
       </c>
       <c r="BQ39" t="s">
-        <v>1402</v>
+        <v>1378</v>
       </c>
       <c r="BR39" t="s">
-        <v>1404</v>
+        <v>1380</v>
       </c>
       <c r="BT39" t="s">
-        <v>1405</v>
+        <v>1381</v>
       </c>
       <c r="BU39" t="s">
-        <v>1439</v>
+        <v>1415</v>
       </c>
       <c r="BV39" t="s">
-        <v>1407</v>
+        <v>1383</v>
       </c>
       <c r="BW39" t="s">
-        <v>1406</v>
+        <v>1382</v>
       </c>
       <c r="BX39" t="s">
-        <v>1408</v>
+        <v>1384</v>
       </c>
       <c r="BZ39" t="s">
-        <v>1405</v>
+        <v>1381</v>
       </c>
       <c r="CA39" t="s">
-        <v>1439</v>
+        <v>1415</v>
       </c>
       <c r="CB39" t="s">
-        <v>1407</v>
+        <v>1383</v>
       </c>
       <c r="CC39" t="s">
-        <v>1406</v>
+        <v>1382</v>
       </c>
       <c r="CD39" t="s">
-        <v>1408</v>
-      </c>
-    </row>
-    <row r="40" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+        <v>1384</v>
+      </c>
+    </row>
+    <row r="40" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>1409</v>
+        <v>1385</v>
       </c>
       <c r="B40" t="s">
         <v>1270</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>1342</v>
+        <v>1318</v>
       </c>
       <c r="D40" t="s">
         <v>258</v>
@@ -19483,85 +19591,85 @@
         <v>259</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>1410</v>
+        <v>1386</v>
       </c>
       <c r="G40" t="s">
         <v>126</v>
       </c>
       <c r="H40" t="s">
-        <v>1411</v>
+        <v>1387</v>
       </c>
       <c r="I40" t="s">
-        <v>1411</v>
+        <v>1387</v>
       </c>
       <c r="J40" t="s">
-        <v>1411</v>
+        <v>1387</v>
       </c>
       <c r="K40" t="s">
-        <v>1411</v>
+        <v>1387</v>
       </c>
       <c r="L40" t="s">
-        <v>1316</v>
+        <v>1298</v>
       </c>
       <c r="M40" t="s">
-        <v>1345</v>
+        <v>1321</v>
       </c>
       <c r="N40" s="14" t="s">
-        <v>1346</v>
+        <v>1322</v>
       </c>
       <c r="O40" t="s">
         <v>1276</v>
       </c>
       <c r="P40" t="s">
-        <v>1317</v>
+        <v>1299</v>
       </c>
       <c r="Q40" t="s">
-        <v>1347</v>
+        <v>1323</v>
       </c>
       <c r="R40" s="14" t="s">
-        <v>1348</v>
+        <v>1324</v>
       </c>
       <c r="T40" t="s">
-        <v>1318</v>
+        <v>1300</v>
       </c>
       <c r="U40" t="s">
-        <v>1349</v>
+        <v>1325</v>
       </c>
       <c r="V40" s="14" t="s">
-        <v>1350</v>
+        <v>1326</v>
       </c>
       <c r="X40" t="s">
-        <v>1319</v>
+        <v>1301</v>
       </c>
       <c r="Y40" t="s">
-        <v>1351</v>
+        <v>1327</v>
       </c>
       <c r="Z40" s="14" t="s">
-        <v>1352</v>
+        <v>1328</v>
       </c>
       <c r="AB40" t="s">
-        <v>1338</v>
+        <v>1314</v>
       </c>
       <c r="AC40" t="s">
-        <v>1353</v>
+        <v>1329</v>
       </c>
       <c r="AD40" s="14" t="s">
-        <v>1354</v>
+        <v>1330</v>
       </c>
       <c r="AE40" t="s">
-        <v>1329</v>
+        <v>1305</v>
       </c>
       <c r="AF40" t="s">
-        <v>1339</v>
+        <v>1315</v>
       </c>
       <c r="AG40" t="s">
+        <v>1307</v>
+      </c>
+      <c r="AH40" s="14" t="s">
         <v>1331</v>
       </c>
-      <c r="AH40" s="14" t="s">
-        <v>1355</v>
-      </c>
       <c r="AI40" t="s">
-        <v>1333</v>
+        <v>1309</v>
       </c>
       <c r="AJ40">
         <v>45</v>
@@ -19588,82 +19696,82 @@
         <v>146</v>
       </c>
       <c r="AU40" t="s">
-        <v>1356</v>
+        <v>1332</v>
       </c>
       <c r="BB40" t="s">
-        <v>1412</v>
+        <v>1388</v>
       </c>
       <c r="BC40" t="s">
-        <v>1440</v>
+        <v>1416</v>
       </c>
       <c r="BD40" t="s">
-        <v>1414</v>
+        <v>1390</v>
       </c>
       <c r="BE40" t="s">
-        <v>1413</v>
+        <v>1389</v>
       </c>
       <c r="BF40" t="s">
-        <v>1415</v>
+        <v>1391</v>
       </c>
       <c r="BH40" t="s">
-        <v>1416</v>
+        <v>1392</v>
       </c>
       <c r="BI40" t="s">
-        <v>1441</v>
+        <v>1417</v>
       </c>
       <c r="BJ40" t="s">
+        <v>1394</v>
+      </c>
+      <c r="BK40" t="s">
+        <v>1393</v>
+      </c>
+      <c r="BL40" t="s">
+        <v>1395</v>
+      </c>
+      <c r="BN40" t="s">
+        <v>1396</v>
+      </c>
+      <c r="BO40" t="s">
         <v>1418</v>
       </c>
-      <c r="BK40" t="s">
-        <v>1417</v>
-      </c>
-      <c r="BL40" t="s">
+      <c r="BP40" t="s">
+        <v>1398</v>
+      </c>
+      <c r="BQ40" t="s">
+        <v>1397</v>
+      </c>
+      <c r="BR40" t="s">
+        <v>1399</v>
+      </c>
+      <c r="BT40" t="s">
+        <v>1400</v>
+      </c>
+      <c r="BU40" t="s">
         <v>1419</v>
       </c>
-      <c r="BN40" t="s">
-        <v>1420</v>
-      </c>
-      <c r="BO40" t="s">
-        <v>1442</v>
-      </c>
-      <c r="BP40" t="s">
-        <v>1422</v>
-      </c>
-      <c r="BQ40" t="s">
-        <v>1421</v>
-      </c>
-      <c r="BR40" t="s">
-        <v>1423</v>
-      </c>
-      <c r="BT40" t="s">
-        <v>1424</v>
-      </c>
-      <c r="BU40" t="s">
-        <v>1443</v>
-      </c>
       <c r="BV40" t="s">
-        <v>1426</v>
+        <v>1402</v>
       </c>
       <c r="BW40" t="s">
-        <v>1425</v>
+        <v>1401</v>
       </c>
       <c r="BX40" t="s">
-        <v>1427</v>
+        <v>1403</v>
       </c>
       <c r="BZ40" t="s">
-        <v>1424</v>
+        <v>1400</v>
       </c>
       <c r="CA40" t="s">
-        <v>1443</v>
+        <v>1419</v>
       </c>
       <c r="CB40" t="s">
-        <v>1426</v>
+        <v>1402</v>
       </c>
       <c r="CC40" t="s">
-        <v>1425</v>
+        <v>1401</v>
       </c>
       <c r="CD40" t="s">
-        <v>1427</v>
+        <v>1403</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Amazon ES: SKU y ASIN de los 38 productos en el maestro
- Maestro: columnas amazon_sku_es / amazon_asin_es (96-97) desde el listado de
  Seller Central (activos y agotados). Varios SKU por ASIN: se usa el _FBM, o el
  que no es _FBA. Ganchos, 006/022 y combos fuera (no estan en el maestro).
- ListingLoader ES: el precio sale de la fila de Espana de Leroy (la tienen los
  38 productos y la actualiza el CSV) antes que de otros portales; Makro excluido.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/datos/FICHERO_MAESTRO2.xlsx
+++ b/public/datos/FICHERO_MAESTRO2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Helian\Desktop\Fichero Maestro\Sistema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A1C7CFF-FE87-40E6-A87F-9F04B82B8B7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F7DAEC0-C0D9-4236-B962-D9FF537BB6AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="591" xr2:uid="{90124268-D67C-4387-8829-7E3B806257E6}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3657" uniqueCount="1500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3735" uniqueCount="1543">
   <si>
     <t>Marketplace</t>
   </si>
@@ -4650,6 +4650,135 @@
   </si>
   <si>
     <t>https://res.cloudinary.com/dzvf24bae/image/upload/v1790694932/bancos/B.MET.090/byn/en/pt05.jpg</t>
+  </si>
+  <si>
+    <t>amazon_sku_es</t>
+  </si>
+  <si>
+    <t>amazon_asin_es</t>
+  </si>
+  <si>
+    <t>R.EMD.001_NE_FBM</t>
+  </si>
+  <si>
+    <t>B0CZJ9B1FT</t>
+  </si>
+  <si>
+    <t>R.EMD.001_BL_FBM</t>
+  </si>
+  <si>
+    <t>B0CZJ9M432</t>
+  </si>
+  <si>
+    <t>R.EMD.001_B&amp;N_FBM</t>
+  </si>
+  <si>
+    <t>B0CZJC16XV</t>
+  </si>
+  <si>
+    <t>R.SYN.003_GR_FBM</t>
+  </si>
+  <si>
+    <t>B0GYBNKGY8</t>
+  </si>
+  <si>
+    <t>R.SYN.007_FBM</t>
+  </si>
+  <si>
+    <t>R.SYN.007_N_FBM</t>
+  </si>
+  <si>
+    <t>R.SYN.007_B_FBM</t>
+  </si>
+  <si>
+    <t>R.SYN.010_N_FBM</t>
+  </si>
+  <si>
+    <t>R.SYN.010_B_FBM</t>
+  </si>
+  <si>
+    <t>R.SYN.011_FBM</t>
+  </si>
+  <si>
+    <t>R.SYN.011_BL_FBM</t>
+  </si>
+  <si>
+    <t>B0GJNPFNR6</t>
+  </si>
+  <si>
+    <t>B0HJD89CVS</t>
+  </si>
+  <si>
+    <t>B0GJNJ1PPS</t>
+  </si>
+  <si>
+    <t>B0HJD6BRRF</t>
+  </si>
+  <si>
+    <t>B0GJNX5GMM</t>
+  </si>
+  <si>
+    <t>B0HJD84TMG</t>
+  </si>
+  <si>
+    <t>B0GJNMZ58T</t>
+  </si>
+  <si>
+    <t>B0HJDGPVDS</t>
+  </si>
+  <si>
+    <t>B0GJNC7GQB</t>
+  </si>
+  <si>
+    <t>B0HJDGSJZN</t>
+  </si>
+  <si>
+    <t>B.MET.090_FBM</t>
+  </si>
+  <si>
+    <t>B0H87XLN16</t>
+  </si>
+  <si>
+    <t>B.MET.090_N_FBM</t>
+  </si>
+  <si>
+    <t>B0H87ZKHNP</t>
+  </si>
+  <si>
+    <t>B.MET.090_B_FBM</t>
+  </si>
+  <si>
+    <t>B0H87ZT4NP</t>
+  </si>
+  <si>
+    <t>B.MET.090_B&amp;N_FBM</t>
+  </si>
+  <si>
+    <t>B0H87WB6LJ</t>
+  </si>
+  <si>
+    <t>B.MET.150_G_FBM</t>
+  </si>
+  <si>
+    <t>B0HJFDYFTW</t>
+  </si>
+  <si>
+    <t>B.MET.150_N_FBM</t>
+  </si>
+  <si>
+    <t>B0HJF5VVM3</t>
+  </si>
+  <si>
+    <t>B.MET.150_B_FBM</t>
+  </si>
+  <si>
+    <t>B0HJFJLPW3</t>
+  </si>
+  <si>
+    <t>B.MET.150_B&amp;N_FBM</t>
+  </si>
+  <si>
+    <t>B0HJF33CFQ</t>
   </si>
 </sst>
 </file>
@@ -11573,7 +11702,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C52A7A11-77C7-4197-B539-DBD653EC8E79}">
-  <dimension ref="A1:CQ40"/>
+  <dimension ref="A1:CS40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -11592,7 +11721,7 @@
     <col min="53" max="53" width="15.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:95" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:97" x14ac:dyDescent="0.35">
       <c r="BB1" s="17" t="s">
         <v>55</v>
       </c>
@@ -11650,7 +11779,7 @@
       <c r="CP1" s="16"/>
       <c r="CQ1" s="16"/>
     </row>
-    <row r="2" spans="1:95" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>62</v>
       </c>
@@ -11936,8 +12065,14 @@
       <c r="CQ2" s="13" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="3" spans="1:95" x14ac:dyDescent="0.35">
+      <c r="CR2" s="6" t="s">
+        <v>1500</v>
+      </c>
+      <c r="CS2" s="6" t="s">
+        <v>1501</v>
+      </c>
+    </row>
+    <row r="3" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
@@ -12145,8 +12280,14 @@
       <c r="CD3" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="4" spans="1:95" x14ac:dyDescent="0.35">
+      <c r="CR3" t="s">
+        <v>152</v>
+      </c>
+      <c r="CS3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="4" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>15</v>
       </c>
@@ -12354,8 +12495,14 @@
       <c r="CD4" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="5" spans="1:95" x14ac:dyDescent="0.35">
+      <c r="CR4" t="s">
+        <v>1502</v>
+      </c>
+      <c r="CS4" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="5" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
         <v>16</v>
       </c>
@@ -12563,8 +12710,14 @@
       <c r="CD5" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="6" spans="1:95" x14ac:dyDescent="0.35">
+      <c r="CR5" t="s">
+        <v>1504</v>
+      </c>
+      <c r="CS5" t="s">
+        <v>1505</v>
+      </c>
+    </row>
+    <row r="6" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
         <v>18</v>
       </c>
@@ -12772,8 +12925,14 @@
       <c r="CD6" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="7" spans="1:95" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR6" t="s">
+        <v>1506</v>
+      </c>
+      <c r="CS6" t="s">
+        <v>1507</v>
+      </c>
+    </row>
+    <row r="7" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
@@ -12981,8 +13140,14 @@
       <c r="CD7" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="8" spans="1:95" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR7" t="s">
+        <v>1508</v>
+      </c>
+      <c r="CS7" t="s">
+        <v>1509</v>
+      </c>
+    </row>
+    <row r="8" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
@@ -13190,8 +13355,14 @@
       <c r="CD8" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="9" spans="1:95" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR8" t="s">
+        <v>350</v>
+      </c>
+      <c r="CS8" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="9" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
         <v>21</v>
       </c>
@@ -13399,8 +13570,14 @@
       <c r="CD9" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="10" spans="1:95" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR9" t="s">
+        <v>385</v>
+      </c>
+      <c r="CS9" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="10" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
         <v>22</v>
       </c>
@@ -13608,8 +13785,14 @@
       <c r="CD10" t="s">
         <v>451</v>
       </c>
-    </row>
-    <row r="11" spans="1:95" x14ac:dyDescent="0.35">
+      <c r="CR10" t="s">
+        <v>423</v>
+      </c>
+      <c r="CS10" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="11" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
         <v>23</v>
       </c>
@@ -13832,8 +14015,14 @@
       <c r="CE11" t="s">
         <v>498</v>
       </c>
-    </row>
-    <row r="12" spans="1:95" x14ac:dyDescent="0.35">
+      <c r="CR11" t="s">
+        <v>1510</v>
+      </c>
+      <c r="CS11" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="12" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
         <v>25</v>
       </c>
@@ -14056,8 +14245,14 @@
       <c r="CE12" t="s">
         <v>539</v>
       </c>
-    </row>
-    <row r="13" spans="1:95" x14ac:dyDescent="0.35">
+      <c r="CR12" t="s">
+        <v>1511</v>
+      </c>
+      <c r="CS12" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="13" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
         <v>26</v>
       </c>
@@ -14280,8 +14475,14 @@
       <c r="CE13" t="s">
         <v>579</v>
       </c>
-    </row>
-    <row r="14" spans="1:95" x14ac:dyDescent="0.35">
+      <c r="CR13" t="s">
+        <v>1512</v>
+      </c>
+      <c r="CS13" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="14" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
         <v>28</v>
       </c>
@@ -14504,8 +14705,14 @@
       <c r="CE14" t="s">
         <v>620</v>
       </c>
-    </row>
-    <row r="15" spans="1:95" x14ac:dyDescent="0.35">
+      <c r="CR14" t="s">
+        <v>587</v>
+      </c>
+      <c r="CS14" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="15" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
         <v>29</v>
       </c>
@@ -14728,8 +14935,14 @@
       <c r="CE15" t="s">
         <v>667</v>
       </c>
-    </row>
-    <row r="16" spans="1:95" x14ac:dyDescent="0.35">
+      <c r="CR15" t="s">
+        <v>633</v>
+      </c>
+      <c r="CS15" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="16" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
         <v>30</v>
       </c>
@@ -14952,8 +15165,14 @@
       <c r="CE16" t="s">
         <v>708</v>
       </c>
-    </row>
-    <row r="17" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR16" t="s">
+        <v>1513</v>
+      </c>
+      <c r="CS16" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="17" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
         <v>31</v>
       </c>
@@ -15176,8 +15395,14 @@
       <c r="CE17" t="s">
         <v>749</v>
       </c>
-    </row>
-    <row r="18" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR17" t="s">
+        <v>1514</v>
+      </c>
+      <c r="CS17" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="18" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
         <v>32</v>
       </c>
@@ -15400,8 +15625,14 @@
       <c r="CE18" t="s">
         <v>790</v>
       </c>
-    </row>
-    <row r="19" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR18" t="s">
+        <v>756</v>
+      </c>
+      <c r="CS18" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="19" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
         <v>33</v>
       </c>
@@ -15624,8 +15855,14 @@
       <c r="CE19" t="s">
         <v>836</v>
       </c>
-    </row>
-    <row r="20" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR19" t="s">
+        <v>1515</v>
+      </c>
+      <c r="CS19" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="20" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
         <v>35</v>
       </c>
@@ -15848,8 +16085,14 @@
       <c r="CE20" t="s">
         <v>877</v>
       </c>
-    </row>
-    <row r="21" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR20" t="s">
+        <v>844</v>
+      </c>
+      <c r="CS20" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="21" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
         <v>36</v>
       </c>
@@ -16072,8 +16315,14 @@
       <c r="CE21" t="s">
         <v>916</v>
       </c>
-    </row>
-    <row r="22" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR21" t="s">
+        <v>1516</v>
+      </c>
+      <c r="CS21" t="s">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="22" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
         <v>38</v>
       </c>
@@ -16296,8 +16545,14 @@
       <c r="CE22" t="s">
         <v>955</v>
       </c>
-    </row>
-    <row r="23" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR22" t="s">
+        <v>922</v>
+      </c>
+      <c r="CS22" t="s">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="23" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
         <v>956</v>
       </c>
@@ -16487,8 +16742,14 @@
       <c r="CD23" t="s">
         <v>988</v>
       </c>
-    </row>
-    <row r="24" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR23" t="s">
+        <v>956</v>
+      </c>
+      <c r="CS23" t="s">
+        <v>1517</v>
+      </c>
+    </row>
+    <row r="24" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
         <v>989</v>
       </c>
@@ -16678,8 +16939,14 @@
       <c r="CD24" t="s">
         <v>1021</v>
       </c>
-    </row>
-    <row r="25" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR24" t="s">
+        <v>989</v>
+      </c>
+      <c r="CS24" t="s">
+        <v>1518</v>
+      </c>
+    </row>
+    <row r="25" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
         <v>1022</v>
       </c>
@@ -16869,8 +17136,14 @@
       <c r="CD25" t="s">
         <v>1052</v>
       </c>
-    </row>
-    <row r="26" spans="1:83" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR25" t="s">
+        <v>1022</v>
+      </c>
+      <c r="CS25" t="s">
+        <v>1519</v>
+      </c>
+    </row>
+    <row r="26" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
         <v>1053</v>
       </c>
@@ -17060,8 +17333,14 @@
       <c r="CD26" t="s">
         <v>1083</v>
       </c>
-    </row>
-    <row r="27" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR26" t="s">
+        <v>1053</v>
+      </c>
+      <c r="CS26" t="s">
+        <v>1520</v>
+      </c>
+    </row>
+    <row r="27" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A27" s="7" t="s">
         <v>1084</v>
       </c>
@@ -17251,8 +17530,14 @@
       <c r="CD27" t="s">
         <v>1114</v>
       </c>
-    </row>
-    <row r="28" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR27" t="s">
+        <v>1084</v>
+      </c>
+      <c r="CS27" t="s">
+        <v>1521</v>
+      </c>
+    </row>
+    <row r="28" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A28" s="7" t="s">
         <v>1115</v>
       </c>
@@ -17442,8 +17727,14 @@
       <c r="CD28" t="s">
         <v>1145</v>
       </c>
-    </row>
-    <row r="29" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR28" t="s">
+        <v>1115</v>
+      </c>
+      <c r="CS28" t="s">
+        <v>1522</v>
+      </c>
+    </row>
+    <row r="29" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A29" s="7" t="s">
         <v>1146</v>
       </c>
@@ -17633,8 +17924,14 @@
       <c r="CD29" t="s">
         <v>1176</v>
       </c>
-    </row>
-    <row r="30" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR29" t="s">
+        <v>1146</v>
+      </c>
+      <c r="CS29" t="s">
+        <v>1523</v>
+      </c>
+    </row>
+    <row r="30" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A30" s="7" t="s">
         <v>1177</v>
       </c>
@@ -17824,8 +18121,14 @@
       <c r="CD30" t="s">
         <v>1207</v>
       </c>
-    </row>
-    <row r="31" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR30" t="s">
+        <v>1177</v>
+      </c>
+      <c r="CS30" t="s">
+        <v>1524</v>
+      </c>
+    </row>
+    <row r="31" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A31" s="7" t="s">
         <v>1208</v>
       </c>
@@ -18018,8 +18321,14 @@
       <c r="CD31" t="s">
         <v>1238</v>
       </c>
-    </row>
-    <row r="32" spans="1:83" x14ac:dyDescent="0.35">
+      <c r="CR31" t="s">
+        <v>1208</v>
+      </c>
+      <c r="CS31" t="s">
+        <v>1525</v>
+      </c>
+    </row>
+    <row r="32" spans="1:97" x14ac:dyDescent="0.35">
       <c r="A32" s="7" t="s">
         <v>1239</v>
       </c>
@@ -18209,8 +18518,14 @@
       <c r="CD32" t="s">
         <v>1268</v>
       </c>
-    </row>
-    <row r="33" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR32" t="s">
+        <v>1239</v>
+      </c>
+      <c r="CS32" t="s">
+        <v>1526</v>
+      </c>
+    </row>
+    <row r="33" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>1269</v>
       </c>
@@ -18400,8 +18715,14 @@
       <c r="CD33" t="s">
         <v>1439</v>
       </c>
-    </row>
-    <row r="34" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR33" t="s">
+        <v>1527</v>
+      </c>
+      <c r="CS33" t="s">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="34" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>1283</v>
       </c>
@@ -18591,8 +18912,14 @@
       <c r="CD34" t="s">
         <v>1459</v>
       </c>
-    </row>
-    <row r="35" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR34" t="s">
+        <v>1529</v>
+      </c>
+      <c r="CS34" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="35" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>1289</v>
       </c>
@@ -18782,8 +19109,14 @@
       <c r="CD35" t="s">
         <v>1479</v>
       </c>
-    </row>
-    <row r="36" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR35" t="s">
+        <v>1531</v>
+      </c>
+      <c r="CS35" t="s">
+        <v>1532</v>
+      </c>
+    </row>
+    <row r="36" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>1295</v>
       </c>
@@ -18973,8 +19306,14 @@
       <c r="CD36" t="s">
         <v>1499</v>
       </c>
-    </row>
-    <row r="37" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR36" t="s">
+        <v>1533</v>
+      </c>
+      <c r="CS36" t="s">
+        <v>1534</v>
+      </c>
+    </row>
+    <row r="37" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>1317</v>
       </c>
@@ -19173,8 +19512,14 @@
       <c r="CD37" t="s">
         <v>1348</v>
       </c>
-    </row>
-    <row r="38" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR37" t="s">
+        <v>1535</v>
+      </c>
+      <c r="CS37" t="s">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="38" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>1349</v>
       </c>
@@ -19373,8 +19718,14 @@
       <c r="CD38" t="s">
         <v>1366</v>
       </c>
-    </row>
-    <row r="39" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR38" t="s">
+        <v>1537</v>
+      </c>
+      <c r="CS38" t="s">
+        <v>1538</v>
+      </c>
+    </row>
+    <row r="39" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>1367</v>
       </c>
@@ -19573,8 +19924,14 @@
       <c r="CD39" t="s">
         <v>1384</v>
       </c>
-    </row>
-    <row r="40" spans="1:82" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="CR39" t="s">
+        <v>1539</v>
+      </c>
+      <c r="CS39" t="s">
+        <v>1540</v>
+      </c>
+    </row>
+    <row r="40" spans="1:97" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>1385</v>
       </c>
@@ -19772,6 +20129,12 @@
       </c>
       <c r="CD40" t="s">
         <v>1403</v>
+      </c>
+      <c r="CR40" t="s">
+        <v>1541</v>
+      </c>
+      <c r="CS40" t="s">
+        <v>1542</v>
       </c>
     </row>
   </sheetData>

</xml_diff>